<commit_message>
Fix ActivityHeatmap dark-mode bug, add category-color safety guard, fix e2e cleanup FK gap
- ActivityHeatmap.tsx: empty-activity day cells hardcoded a light-gray
  inline style with no dark-mode branch (inline style always wins over
  className, so no amount of dark: CSS elsewhere could ever apply) --
  fixed by only setting the inline color for cells with real activity
- Added a defensive safeCategoryColor() luminance check for GreyMatters
  category colors -- no live incident today (no admin UI exists to set
  a bad value), but permanently safe if that UI is ever built
- Fixed a real e2e cleanup gap found while regression-testing: a test
  account that reviews someone else's work (verified_outcomes.verified_by)
  wasn't covered by the pre-delete step, silently orphaning accounts
- New e2e coverage for both fixes, verified live against prod

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements-traceability/greyin-requirements-traceability.xlsx
+++ b/docs/requirements-traceability/greyin-requirements-traceability.xlsx
@@ -5908,7 +5908,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E83"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -5936,13 +5936,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>UI/UX audit round: 24 confirmed dark-mode/layout/interactive-state bugs, all fixed</v>
+        <v>ActivityHeatmap + category-color: two "uncertain, needs a visual check" audit findings resolved</v>
       </c>
       <c r="B2" t="str">
         <v>Done</v>
       </c>
       <c r="C2" t="str">
-        <v>Three parallel background audits (2026-09-11) triggered by a user-reported bug (GreyMatters' MarkdownEditor content textarea had no dark:bg-/dark:text- classes, rendering white-on-white text invisible until selected). Extended the fix pattern found and confirmed 36 more genuine instances of the exact same defect class (a dark:border- class present without matching dark:bg-/dark:text-) across all 7 apps via a bracket/quote-aware Python JSX-tag scanner, not naive grep -- concentrated in the near-identical reset-password/reset-password-confirm/verify auth pages duplicated per app (30 of 36), plus OrderChat/OrderReview/ResumeSkillsUploader/TipButton/TeammateTagPicker. A second parallel audit found layout/alignment issues: SiteHeader missing min-w-0/flex-shrink-0/truncate robustness in 3 of 6 apps (a fix previously applied to only half the apps, never back-ported), and a 9-stat-card grid at a column count that left one dangling in the last row (fixed by changing to a divisor of 9); a 7-item demo-persona grid was audited and deliberately left alone since 7 is prime and no column count evenly divides it -- a single trailing card there is a normal pattern, not a bug. A third parallel audit found interactive-state gaps: star-rating buttons (StackWorks + FlexPro SkillRatingForm, FlexPro OrderReview) with zero disabled/focus-visible styling; a platform-wide missing focus indicator on every search box (5 apps' /search pages plus DeepEdge jobs and FlexPro gigs) since `outline-none` was applied with no `focus-within:` replacement on the wrapping box; FollowButton's "Unfollow" hover state missing a dark: counterpart in the 4 apps that have it (same shared bug, same fix, once); upload buttons (FileUploader + 3x ImageUploader) that stayed fully clickable-looking while an upload was in progress despite the underlying input being disabled; two `disabled:bg-gray-300` buttons with no dark fallback (FlexPro OrderChat/OrderReview); Salt &amp; Pepper's RSVP "Full" button missing a dark background. All 24 confirmed findings fixed (the 2 layout items and the 1 correctly-not-fixed grid case bring the total examined to 27); 6 apps rebuilt/redeployed, all typecheck clean.</v>
+        <v>Follow-up to the 2026-09-11 UI/UX audit round, which flagged two items as data-dependent/uncertain rather than confirmed. Reading the actual code resolved both: (1) ActivityHeatmap.tsx (Greyin Hub dashboard) -- confirmed a REAL bug, not uncertain: every "no activity" day cell hardcoded backgroundColor #e5e7eb via inline style with zero dark-mode branch, and inline style always wins over className, so no dark: CSS anywhere could ever have applied to it regardless of what else got fixed platform-wide. Every date range with at least one inactive day (essentially always) rendered pale squares against the dark dashboard. Fixed by only setting backgroundColor via style for cells with real activity, using a themed className (bg-gray-200 dark:bg-gray-800 border border-gray-300 dark:border-gray-700) for empty cells instead -- the colored/active cells were already fine as-is (the same saturated, theme-invariant PILLAR_COLORS hex values used everywhere else on the platform without dark: variants, by established convention). (2) GreyMatters categories.color -- genuinely data-dependent (an unconstrained TEXT column, no CHECK, no admin UI to edit it at all today; the 4 real rows were seeded once directly via SQL in 001_initial_schema.sql, all safe mid-range colors) so zero live exposure currently, but nothing in the schema prevents a future admin-set color extreme enough to vanish against one of the app's two themed card backgrounds. Added a defensive `safeCategoryColor()` helper (apps/greymatters-blog/src/app/lib/safe-color.ts) computing a simplified relative-luminance check and falling back to the existing default (#2563eb) for any color outside a safe middle band (luminance &lt;0.15 or &gt;0.85) -- necessary because this renders server-side with no way to know the viewer's actual client-side theme choice, so the only safe approach is rejecting colors extreme enough to fail against EITHER background rather than trying to pick per-theme. Verified live against prod: inserted a real #0a0a0a test category, confirmed the rendered page used the #2563eb fallback, inserted a real safe #3B82F6 category, confirmed it passed through unchanged; both real rows deleted after. New e2e test for each: activity-heatmap-dark-mode.spec.ts (backdates a fresh signup's profile.created_at by 5 days via service-role PATCH so the heatmap range spans real empty days, then asserts the theme-aware classes appear and the old hardcoded hex is gone from the page entirely) and a new case in comments-and-categories.spec.ts (real too-dark and safe test categories, asserts the rendered SVG's computed color). While regression-testing against the pre-existing hub-dashboard.spec.ts, caught and fixed a third, unrelated real bug: e2e/utils/cleanup.ts's verified_outcomes pre-delete step only matched subject_user_id (which cascades on delete anyway per its own FK, so was never actually the blocker) and missed verified_by entirely (no cascade action at all) -- meaning any test account that reviews/verifies someone else's work (a StackWorks builder reviewing a candidate's submission, not the subject of the row) failed to delete with a 500, silently orphaning the account. Confirmed live via hub-dashboard.spec.ts's own builder account actually failing to delete with exactly this FK name; fixed the filter to match either column, manually cleaned up the one real orphaned account this uncovered, and re-ran clean.</v>
       </c>
       <c r="D2" t="str">
         <v>User request, 2026-09-11</v>
@@ -5953,13 +5953,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>UI/UX heuristics audit: confirmation on destructive actions + inline payment errors</v>
+        <v>UI/UX audit round: 24 confirmed dark-mode/layout/interactive-state bugs, all fixed</v>
       </c>
       <c r="B3" t="str">
         <v>Done</v>
       </c>
       <c r="C3" t="str">
-        <v>A fourth parallel audit (2026-09-11) against Nielsen-heuristic-style violations found two systemic, platform-wide gaps beyond the contrast/layout/interactive-state bugs above. (1) Zero confirmation existed anywhere in the codebase before a destructive submit -- every delete/withdraw/cancel action was a plain `&lt;form method="POST"&gt;` with a bare submit button, firing immediately with no undo, including admin content deletion (affecting other users' data) and a blog author's own permanent "Delete Post". Fixed by adding a small reusable `ConfirmSubmitButton` client component (one copy per app, matching this codebase's established per-app-duplication convention) that wraps the exact same submit button and gates it behind a native confirm() -- no change to the surrounding server-rendered form, so progressive enhancement is preserved. Applied to all ~20 confirmed destructive actions across deepedge/flexpro/stackworks/saltnpepper-community/greymatters-blog/greyin-hub: admin content deletion (Salt &amp; Pepper discussions/replies/projects, StackWorks projects/asks, GreyMatters comments, peer-confirmed projects), a blog author's own post deletion, DeepEdge application withdrawal, and FlexPro mentor-session-slot cancellation. Deliberately did NOT add confirmation to lower-stakes/reversible actions the audit itself distinguished (Unpublish, clear-flag, role updates). (2) Every Razorpay payment/checkout flow across both apps used blocking `alert()` for errors while every other form on the same platform uses inline styled banners -- a real UX inconsistency specifically on money flows. Fixed by adding a hidden error `&lt;div&gt;` next to each checkout/subscribe button and replacing every alert() with a small `showCheckoutError()`/`showSubscribeError()` helper that un-hides it (the checkout pages are server components rendering a vanilla-JS `dangerouslySetInnerHTML` script for the Razorpay widget, not React client components, so the fix works within that existing architecture rather than requiring a rewrite): FlexPro checkout/[id], subscribe, mentor-sessions/checkout/[orderId], client-jobs/[id]/pay/[orderId]; DeepEdge subscribe; GreyMatters' TipButton (a real client component, given real React error state instead). All 6 apps typecheck clean, rebuilt, redeployed.</v>
+        <v>Three parallel background audits (2026-09-11) triggered by a user-reported bug (GreyMatters' MarkdownEditor content textarea had no dark:bg-/dark:text- classes, rendering white-on-white text invisible until selected). Extended the fix pattern found and confirmed 36 more genuine instances of the exact same defect class (a dark:border- class present without matching dark:bg-/dark:text-) across all 7 apps via a bracket/quote-aware Python JSX-tag scanner, not naive grep -- concentrated in the near-identical reset-password/reset-password-confirm/verify auth pages duplicated per app (30 of 36), plus OrderChat/OrderReview/ResumeSkillsUploader/TipButton/TeammateTagPicker. A second parallel audit found layout/alignment issues: SiteHeader missing min-w-0/flex-shrink-0/truncate robustness in 3 of 6 apps (a fix previously applied to only half the apps, never back-ported), and a 9-stat-card grid at a column count that left one dangling in the last row (fixed by changing to a divisor of 9); a 7-item demo-persona grid was audited and deliberately left alone since 7 is prime and no column count evenly divides it -- a single trailing card there is a normal pattern, not a bug. A third parallel audit found interactive-state gaps: star-rating buttons (StackWorks + FlexPro SkillRatingForm, FlexPro OrderReview) with zero disabled/focus-visible styling; a platform-wide missing focus indicator on every search box (5 apps' /search pages plus DeepEdge jobs and FlexPro gigs) since `outline-none` was applied with no `focus-within:` replacement on the wrapping box; FollowButton's "Unfollow" hover state missing a dark: counterpart in the 4 apps that have it (same shared bug, same fix, once); upload buttons (FileUploader + 3x ImageUploader) that stayed fully clickable-looking while an upload was in progress despite the underlying input being disabled; two `disabled:bg-gray-300` buttons with no dark fallback (FlexPro OrderChat/OrderReview); Salt &amp; Pepper's RSVP "Full" button missing a dark background. All 24 confirmed findings fixed (the 2 layout items and the 1 correctly-not-fixed grid case bring the total examined to 27); 6 apps rebuilt/redeployed, all typecheck clean.</v>
       </c>
       <c r="D3" t="str">
         <v>User request, 2026-09-11</v>
@@ -5970,13 +5970,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Contact vs Feedback conflation: every app's "Contact" footer link actually opened the login-gated Feedback form</v>
+        <v>UI/UX heuristics audit: confirmation on destructive actions + inline payment errors</v>
       </c>
       <c r="B4" t="str">
         <v>Done</v>
       </c>
       <c r="C4" t="str">
-        <v>User-reported (2026-09-11): confirmed by reading every app's SiteFooter.tsx directly that all 7 apps have TWO separate footer links labeled "Feedback" and "Contact" (one in the main link list, one in the bottom copyright bar) -- but both pointed at the literal same URL, https://greyin.net/feedback?app=X, a login-gated product-feedback form (101/052, deliberately login-gated by a prior decision). A prospective customer, partner, or press contact clicking "Contact" had no way to reach anyone without first creating a Greyin account and had no path to a genuine sales/business inquiry at all. DeepEdge separately has a real B2B lead form (/enterprise-contact, enterprise_leads, 039/044) but it also requires login -- correct for an existing customer requesting Enterprise/Fractional/Outplacement service, wrong for an anonymous visitor, and left untouched since it serves a different, legitimate purpose. Built a new, genuinely anonymous "Contact us" (migration 148: business_inquiries table, public INSERT policy, admin-only SELECT/UPDATE, rate-limited via check_rate_limit/record_rate_limit_attempt reusing the same IP-extraction/private-IP-skip logic as every other anonymous write this platform has added -- demo_login/wishlist_anonymous/page_visit, now widened a fourth time to business_inquiry) at Greyin Hub: /contact?app=X (name/email/company-optional/message, mirrors /feedback's own visual style but with no login gate, matching the anonymous-wishlist precedent instead of feedback's deliberate login-gate precedent), /api/contact/create, and /admin/contact (new site-wide admin card, mirrors the existing /admin/feedback reply-queue layout with a simpler mark-contacted/close status flow instead of a reply thread). Updated all 7 apps' footers to point the copyright-bar "Contact" link at the new /contact?app=X instead of /feedback?app=X; left the upper-list "Feedback" link on every app completely unchanged. Verified end to end against prod: a real anonymous curl POST (no auth) landed a real row in business_inquiries with the correct source_app, and the DeepEdge homepage footer's live rendered HTML confirms the Contact link now points at the new destination.</v>
+        <v>A fourth parallel audit (2026-09-11) against Nielsen-heuristic-style violations found two systemic, platform-wide gaps beyond the contrast/layout/interactive-state bugs above. (1) Zero confirmation existed anywhere in the codebase before a destructive submit -- every delete/withdraw/cancel action was a plain `&lt;form method="POST"&gt;` with a bare submit button, firing immediately with no undo, including admin content deletion (affecting other users' data) and a blog author's own permanent "Delete Post". Fixed by adding a small reusable `ConfirmSubmitButton` client component (one copy per app, matching this codebase's established per-app-duplication convention) that wraps the exact same submit button and gates it behind a native confirm() -- no change to the surrounding server-rendered form, so progressive enhancement is preserved. Applied to all ~20 confirmed destructive actions across deepedge/flexpro/stackworks/saltnpepper-community/greymatters-blog/greyin-hub: admin content deletion (Salt &amp; Pepper discussions/replies/projects, StackWorks projects/asks, GreyMatters comments, peer-confirmed projects), a blog author's own post deletion, DeepEdge application withdrawal, and FlexPro mentor-session-slot cancellation. Deliberately did NOT add confirmation to lower-stakes/reversible actions the audit itself distinguished (Unpublish, clear-flag, role updates). (2) Every Razorpay payment/checkout flow across both apps used blocking `alert()` for errors while every other form on the same platform uses inline styled banners -- a real UX inconsistency specifically on money flows. Fixed by adding a hidden error `&lt;div&gt;` next to each checkout/subscribe button and replacing every alert() with a small `showCheckoutError()`/`showSubscribeError()` helper that un-hides it (the checkout pages are server components rendering a vanilla-JS `dangerouslySetInnerHTML` script for the Razorpay widget, not React client components, so the fix works within that existing architecture rather than requiring a rewrite): FlexPro checkout/[id], subscribe, mentor-sessions/checkout/[orderId], client-jobs/[id]/pay/[orderId]; DeepEdge subscribe; GreyMatters' TipButton (a real client component, given real React error state instead). All 6 apps typecheck clean, rebuilt, redeployed.</v>
       </c>
       <c r="D4" t="str">
         <v>User request, 2026-09-11</v>
@@ -5987,30 +5987,30 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Anonymous wishlist submission (Emergent-parity gap #2, part 1 of 2)</v>
+        <v>Contact vs Feedback conflation: every app's "Contact" footer link actually opened the login-gated Feedback form</v>
       </c>
       <c r="B5" t="str">
         <v>Done</v>
       </c>
       <c r="C5" t="str">
-        <v>Same third-pass Emergent audit (2026-09-08) found Emergent lets an anonymous visitor submit a feature request with no login (/wishlist/public); Greyin's wishlist/create redirected an anonymous visitor to /login first. This was NOT a bug -- 101_wishlist_and_feedback.sql's own migration comment records "feedback requires login, no anonymous submission" as a decision made WITH the user at the time. Reversed explicitly per the user's current request, not fixed as a defect -- recorded in migration 144's own comment for the same reason the original decision was recorded. Schema: feature_requests.user_id made nullable, new email column (populated only when user_id is null), a CHECK requiring one or the other, INSERT policy widened to accept either an authenticated self-submission or a null-user_id anonymous one. Also widened the SELECT policy from authenticated-only to fully public -- confirmed the previous read-scoping meant an anonymous visitor who'd just submitted anonymously would immediately see an EMPTY list on the same page they were redirected back to (RLS hid every row, including their own submission, from an anon reader) -- nothing in title/description/status/upvote_count is sensitive, and a wishlist an anonymous submitter can't even see afterward isn't a coherent version of the feature Emergent has; upvoting deliberately stays authenticated-only and unchanged, since that was never the gap. New public write is rate-limited (5/hour per IP, tighter than demo-login's since spam feature requests are more visible to admins) via the same check_rate_limit/record_rate_limit_attempt mechanism reused a second time this week. Caught and fixed a genuine, PRE-EXISTING, unrelated test bug while running the existing cross-platform wishlist spec as a regression check (not something this change caused): a bare getByText('planned') assertion was a strict-mode violation waiting to happen the moment a second real 'planned'-status row existed anywhere on the page -- and one already does, a real seeded item ("Calendar sync for mentor session slots") -- fixed by scoping the assertion to the test's own card, matching every other assertion in that same test that already used this scoping. New e2e spec (wishlist-anonymous.spec.ts) covers a real anonymous submission (verifies user_id IS NULL + email persisted) and a missing-email rejection; re-ran alongside the now-fixed pre-existing cross-platform spec -- 5/5 passing.</v>
+        <v>User-reported (2026-09-11): confirmed by reading every app's SiteFooter.tsx directly that all 7 apps have TWO separate footer links labeled "Feedback" and "Contact" (one in the main link list, one in the bottom copyright bar) -- but both pointed at the literal same URL, https://greyin.net/feedback?app=X, a login-gated product-feedback form (101/052, deliberately login-gated by a prior decision). A prospective customer, partner, or press contact clicking "Contact" had no way to reach anyone without first creating a Greyin account and had no path to a genuine sales/business inquiry at all. DeepEdge separately has a real B2B lead form (/enterprise-contact, enterprise_leads, 039/044) but it also requires login -- correct for an existing customer requesting Enterprise/Fractional/Outplacement service, wrong for an anonymous visitor, and left untouched since it serves a different, legitimate purpose. Built a new, genuinely anonymous "Contact us" (migration 148: business_inquiries table, public INSERT policy, admin-only SELECT/UPDATE, rate-limited via check_rate_limit/record_rate_limit_attempt reusing the same IP-extraction/private-IP-skip logic as every other anonymous write this platform has added -- demo_login/wishlist_anonymous/page_visit, now widened a fourth time to business_inquiry) at Greyin Hub: /contact?app=X (name/email/company-optional/message, mirrors /feedback's own visual style but with no login gate, matching the anonymous-wishlist precedent instead of feedback's deliberate login-gate precedent), /api/contact/create, and /admin/contact (new site-wide admin card, mirrors the existing /admin/feedback reply-queue layout with a simpler mark-contacted/close status flow instead of a reply thread). Updated all 7 apps' footers to point the copyright-bar "Contact" link at the new /contact?app=X instead of /feedback?app=X; left the upper-list "Feedback" link on every app completely unchanged. Verified end to end against prod: a real anonymous curl POST (no auth) landed a real row in business_inquiries with the correct source_app, and the DeepEdge homepage footer's live rendered HTML confirms the Contact link now points at the new destination.</v>
       </c>
       <c r="D5" t="str">
-        <v>User request, 2026-09-08 (Emergent-parity follow-up)</v>
+        <v>User request, 2026-09-11</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Admin transaction ledger (Emergent-parity gap #1)</v>
+        <v>Anonymous wishlist submission (Emergent-parity gap #2, part 1 of 2)</v>
       </c>
       <c r="B6" t="str">
         <v>Done</v>
       </c>
       <c r="C6" t="str">
-        <v>A third-pass Emergent-comparison audit (2026-09-08, after the pitch-readiness 3-item plan shipped) found Emergent has an admin payments console: a gateway toggle (Stripe&lt;-&gt;Razorpay) plus a cross-platform transaction ledger, neither of which Greyin had. Confirmed directly, not assumed, that Stripe does not exist anywhere in Greyin -- no SDK in any package.json, no STRIPE_* env var anywhere, no Stripe schema in any of 142 migrations -- Razorpay is the sole gateway across all 7 apps. Building a toggle to a gateway that was never integrated would be fake, non-functional UI, so that half was explicitly excluded; only the real, valuable half (the ledger) was built. New get_recent_transactions(p_limit) (143), a SECURITY DEFINER function admin-gated inside the body (same pattern as get_admin_overview_counts(), 141) that UNIONs 5 verified real payment sources -- gig_orders, payout_requests, company_subscriptions, flexpro_subscriptions, author_tips -- into one normalized (type, amount, status, date, description) shape, correctly joining company_subscriptions/flexpro_subscriptions through tier_id -&gt; subscription_tiers.price_inr for the real current price rather than the legacy plan_id -&gt; subscription_plans.price_inr (plan_id only exists to satisfy a pre-existing NOT NULL FK per 096's own comment). Every source's amount is treated as INR without a conversion step -- confirmed every real insert path across all 5 hardcodes 'INR' explicitly, despite gig_orders.currency still defaulting to a stale 'USD' template value from 001. Caught and fixed a real SQL bug before ever exposing this to an admin: the first draft put an ORDER BY on a COALESCE(...) expression inside each UNION ALL branch, which Postgres rejects ("Only result column names can be used, not expressions or functions") -- confirmed live via the function actually returning this exact error on first real call, not caught by any dry-run syntax check; fixed by aliasing each branch's sort expression to a named column and ordering by the alias. New /admin/payments tab (Hub, added to the existing AdminTabNav from Phase 3). New e2e spec seeds a distinctively-amounted tip and confirms it surfaces in the ledger (rather than asserting on the whole list, which is real non-empty prod data) plus a non-admin redirect check -- both passing against prod.</v>
+        <v>Same third-pass Emergent audit (2026-09-08) found Emergent lets an anonymous visitor submit a feature request with no login (/wishlist/public); Greyin's wishlist/create redirected an anonymous visitor to /login first. This was NOT a bug -- 101_wishlist_and_feedback.sql's own migration comment records "feedback requires login, no anonymous submission" as a decision made WITH the user at the time. Reversed explicitly per the user's current request, not fixed as a defect -- recorded in migration 144's own comment for the same reason the original decision was recorded. Schema: feature_requests.user_id made nullable, new email column (populated only when user_id is null), a CHECK requiring one or the other, INSERT policy widened to accept either an authenticated self-submission or a null-user_id anonymous one. Also widened the SELECT policy from authenticated-only to fully public -- confirmed the previous read-scoping meant an anonymous visitor who'd just submitted anonymously would immediately see an EMPTY list on the same page they were redirected back to (RLS hid every row, including their own submission, from an anon reader) -- nothing in title/description/status/upvote_count is sensitive, and a wishlist an anonymous submitter can't even see afterward isn't a coherent version of the feature Emergent has; upvoting deliberately stays authenticated-only and unchanged, since that was never the gap. New public write is rate-limited (5/hour per IP, tighter than demo-login's since spam feature requests are more visible to admins) via the same check_rate_limit/record_rate_limit_attempt mechanism reused a second time this week. Caught and fixed a genuine, PRE-EXISTING, unrelated test bug while running the existing cross-platform wishlist spec as a regression check (not something this change caused): a bare getByText('planned') assertion was a strict-mode violation waiting to happen the moment a second real 'planned'-status row existed anywhere on the page -- and one already does, a real seeded item ("Calendar sync for mentor session slots") -- fixed by scoping the assertion to the test's own card, matching every other assertion in that same test that already used this scoping. New e2e spec (wishlist-anonymous.spec.ts) covers a real anonymous submission (verifies user_id IS NULL + email persisted) and a missing-email rejection; re-ran alongside the now-fixed pre-existing cross-platform spec -- 5/5 passing.</v>
       </c>
       <c r="D6" t="str">
         <v>User request, 2026-09-08 (Emergent-parity follow-up)</v>
@@ -6021,13 +6021,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Anonymous visit tracking + admin trend chart (Emergent-parity gap #2, part 2 of 2)</v>
+        <v>Admin transaction ledger (Emergent-parity gap #1)</v>
       </c>
       <c r="B7" t="str">
         <v>Done</v>
       </c>
       <c r="C7" t="str">
-        <v>Same third-pass Emergent audit found Emergent tracks anonymous landing-page visits with an admin-facing trend chart; Greyin had no equivalent -- analytics_events requires an authenticated user_id (WITH CHECK auth.uid() = user_id), categorically incompatible with an anonymous writer, and semantically a different kind of event (member behavior vs. anonymous traffic), so a new table was added rather than an alter. New page_visits (id, path, occurred_at) -- RLS enabled with NO policies at all, same "no direct client access, only via SECURITY DEFINER functions" convention as rate_limit_attempts (075); record_page_visit(p_path) (no admin gate, called by anonymous visitors) and get_page_visit_trend(p_days default 30) (admin-gated, GROUP BY date_trunc('day', occurred_at)) (145). New public write rate-limited via check_rate_limit/record_rate_limit_attempt (looser than the wishlist limit -- 30/hour per IP, since this is meant to bound a scripted flood rather than gate normal browsing), reusing the same IP-extraction/private-IP-skip logic now established a third time this week. New client-only VisitTracker component fires one fire-and-forget POST to /api/visit on homepage mount; that route uses a stateless direct-fetch-with-anon-key pattern (mirroring apps/greymatters-blog's newsletter-subscribe route), not the cookie-bound SSR client, for the same session-recovery-crash reason that route's own comment documents. New "Visits (last 30 days)" section on /admin/overview, a hand-rolled inline SVG bar chart matching apps/deepedge/SalaryTrendChart.tsx's established no-charting-library approach (confirmed the only precedent in any package.json). Live-smoke-tested end to end via direct curl and a real headless-browser homepage load before writing e2e coverage. While verifying the e2e spec's rate-limit test, found and root-caused a real environment limitation (not a product bug): a direct HTTP request to /api/visit from the same docker host that serves the app can never trigger the route's IP-based rate-limiting, because Traefik correctly refuses to trust a client-supplied X-Forwarded-For and substitutes the actual observed peer address, which from this host is always the private bridge gateway (172.18.0.1) -- exactly the private-IP case the route deliberately skips rate-limiting for. Confirmed this isn't new to this feature: neither demo_login's nor signup's own e2e specs exercise their real 429 paths either. Rewrote the rate-limit e2e test to verify the actual check_rate_limit/record_rate_limit_attempt RPC pair directly against a synthetic key instead of trying to trigger a 429 over HTTP from this host -- that pair is the real, reusable contract the route depends on, and it needed a real fix (the route's own baseUrl/anon-key resolution was confirmed correct along the way, not the cause).</v>
+        <v>A third-pass Emergent-comparison audit (2026-09-08, after the pitch-readiness 3-item plan shipped) found Emergent has an admin payments console: a gateway toggle (Stripe&lt;-&gt;Razorpay) plus a cross-platform transaction ledger, neither of which Greyin had. Confirmed directly, not assumed, that Stripe does not exist anywhere in Greyin -- no SDK in any package.json, no STRIPE_* env var anywhere, no Stripe schema in any of 142 migrations -- Razorpay is the sole gateway across all 7 apps. Building a toggle to a gateway that was never integrated would be fake, non-functional UI, so that half was explicitly excluded; only the real, valuable half (the ledger) was built. New get_recent_transactions(p_limit) (143), a SECURITY DEFINER function admin-gated inside the body (same pattern as get_admin_overview_counts(), 141) that UNIONs 5 verified real payment sources -- gig_orders, payout_requests, company_subscriptions, flexpro_subscriptions, author_tips -- into one normalized (type, amount, status, date, description) shape, correctly joining company_subscriptions/flexpro_subscriptions through tier_id -&gt; subscription_tiers.price_inr for the real current price rather than the legacy plan_id -&gt; subscription_plans.price_inr (plan_id only exists to satisfy a pre-existing NOT NULL FK per 096's own comment). Every source's amount is treated as INR without a conversion step -- confirmed every real insert path across all 5 hardcodes 'INR' explicitly, despite gig_orders.currency still defaulting to a stale 'USD' template value from 001. Caught and fixed a real SQL bug before ever exposing this to an admin: the first draft put an ORDER BY on a COALESCE(...) expression inside each UNION ALL branch, which Postgres rejects ("Only result column names can be used, not expressions or functions") -- confirmed live via the function actually returning this exact error on first real call, not caught by any dry-run syntax check; fixed by aliasing each branch's sort expression to a named column and ordering by the alias. New /admin/payments tab (Hub, added to the existing AdminTabNav from Phase 3). New e2e spec seeds a distinctively-amounted tip and confirms it surfaces in the ledger (rather than asserting on the whole list, which is real non-empty prod data) plus a non-admin redirect check -- both passing against prod.</v>
       </c>
       <c r="D7" t="str">
         <v>User request, 2026-09-08 (Emergent-parity follow-up)</v>
@@ -6038,16 +6038,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Consolidated tabbed admin panel (Phase 3 of 3, pitch-readiness plan)</v>
+        <v>Anonymous visit tracking + admin trend chart (Emergent-parity gap #2, part 2 of 2)</v>
       </c>
       <c r="B8" t="str">
         <v>Done</v>
       </c>
       <c r="C8" t="str">
-        <v>Same fresh audit (2026-09-08) found the admin surface fragmented across 7 apps: Greyin Hub's /admin covered 9 genuinely site-wide features with no tab-nav; DeepEdge/FlexPro/StackWorks/Salt &amp; Pepper/GreyMatters each had their own separate, un-navigable, single-page admin dashboard; Longlist had no admin page at all -- an admin had to separately log into 6 different domains to do all platform maintenance. Confirmed directly before building anything (not assumed): every admin-relevant RLS policy across the platform is keyed purely on EXISTS(...profiles.role='admin'), never on request origin/domain, so a Hub-hosted page making the identical Supabase queries is safe and correct -- no architectural blocker to consolidating. Built: admin/layout.tsx + AdminTabNav.tsx (new, Hub-local) -- does the auth+role check ONCE for the whole /admin/* tree via a shared layout (previously duplicated per-page across the 9 existing site-wide pages, which also had to be stripped of their own &lt;SiteHeader&gt;/&lt;main&gt; wrapper to avoid a real double-header bug once the layout renders that chrome once); tabs for Overview (new), Site-wide (existing 9 pages, URLs unchanged), and one per pillar (DeepEdge, FlexPro, StackWorks, Salt &amp; Pepper, GreyMatters, Longlist). Each pillar tab ports that app's own admin page UI + a copy of its API routes into Hub, keeping the original pillar-hosted page live and unmodified (additive consolidation, zero regression risk, since both UIs hit the same RLS-gated tables with nothing to drift) -- DeepEdge and StackWorks are fully ported (jobs/users; projects/asks/verifications/users); FlexPro, Salt &amp; Pepper, and GreyMatters port the simple DB-mutation actions fully (gig close, discussion/comment moderation, role updates) but deliberately do NOT duplicate actions that trigger real side effects elsewhere -- a live RazorpayX bank transfer or Razorpay refund (FlexPro payouts/disputes), or an LLM-calling sweep/digest-send (Salt &amp; Pepper "AI Quality Sweep", GreyMatters "Sweep now"/"Send weekly digest") -- linking out to the original pillar-hosted page for those instead, since duplicating real-money-movement or LLM-calling code across two codebases would double the surface for a payment or cost bug rather than consolidate anything. Longlist's admin tab is built entirely from scratch (moderate future_roles postings, subscriber counts from future_role_subscriptions) since it never had one -- needed a new admin RLS bypass migration first (140_longlist_admin_policies.sql), since neither table had ever had one (only owner/subscriber policies existed). The new Overview tab wires a new get_admin_overview_counts() SECURITY DEFINER function (141, admin-gated inside the function body per the precedent in 131's own header comment on when the gate belongs inside vs. is unnecessary for a service-role caller) alongside the 4 pre-existing report functions (bias audit, job-recommendation feedback, market intelligence, threshold votes) as quick-link cards, rather than re-rendering each report's full body redundantly. Caught and fixed two more real, pre-existing bugs during e2e verification, both surfaced by (not caused by) this work: (1) a SILENT, systemic e2e test-cleanup failure present since migration 122 -- ANY test awarding reputation_events to a throwaway account (seedReputationPoints, and now redeem_referral_code from Phase 2) left that account undeletable, since the sync_saltnpepper_score_input trigger's AFTER DELETE re-upsert into greyin_score_inputs can run after a cascading delete has already removed the profiles row it needs, aborting the whole GoTrue delete with a 500 that e2e/utils/cleanup.ts's Cleanup.run() was silently swallowing -- confirmed live via 6 real orphaned test accounts found in prod, invisible until directly queried; fixed by having Cleanup.run() explicitly pre-delete the 4 evidence tables (verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings, using each one's real subject-column name -- subject_user_id, not user_id, on two of them, and rater_id/ratee_id OR'd together on the one with no single user column at all) before deleting the user, mirroring the same fix already applied to the seed file's own cleanup phase; also stopped swallowing a genuine delete failure silently, logging it instead. (2) future_roles.posted_by had no ON DELETE action at all (087) -- deleting an employer who'd posted a future role failed outright in prod, not just in tests, since Postgres checks every FK referencing a deleted row directly regardless of whether another cascade path (company_id, which DOES cascade) would also remove the same row; fixed via migration 142, adding ON DELETE CASCADE to match company_id's own semantics (both columns always describe the same account per 087's own RLS policy). 14 new e2e specs (2-3 per pillar tab plus Overview) plus a full regression run of all 5 pre-existing per-pillar admin specs together with the new ones -- 38/38 passing, confirming both the ported copies AND the untouched originals still work.</v>
+        <v>Same third-pass Emergent audit found Emergent tracks anonymous landing-page visits with an admin-facing trend chart; Greyin had no equivalent -- analytics_events requires an authenticated user_id (WITH CHECK auth.uid() = user_id), categorically incompatible with an anonymous writer, and semantically a different kind of event (member behavior vs. anonymous traffic), so a new table was added rather than an alter. New page_visits (id, path, occurred_at) -- RLS enabled with NO policies at all, same "no direct client access, only via SECURITY DEFINER functions" convention as rate_limit_attempts (075); record_page_visit(p_path) (no admin gate, called by anonymous visitors) and get_page_visit_trend(p_days default 30) (admin-gated, GROUP BY date_trunc('day', occurred_at)) (145). New public write rate-limited via check_rate_limit/record_rate_limit_attempt (looser than the wishlist limit -- 30/hour per IP, since this is meant to bound a scripted flood rather than gate normal browsing), reusing the same IP-extraction/private-IP-skip logic now established a third time this week. New client-only VisitTracker component fires one fire-and-forget POST to /api/visit on homepage mount; that route uses a stateless direct-fetch-with-anon-key pattern (mirroring apps/greymatters-blog's newsletter-subscribe route), not the cookie-bound SSR client, for the same session-recovery-crash reason that route's own comment documents. New "Visits (last 30 days)" section on /admin/overview, a hand-rolled inline SVG bar chart matching apps/deepedge/SalaryTrendChart.tsx's established no-charting-library approach (confirmed the only precedent in any package.json). Live-smoke-tested end to end via direct curl and a real headless-browser homepage load before writing e2e coverage. While verifying the e2e spec's rate-limit test, found and root-caused a real environment limitation (not a product bug): a direct HTTP request to /api/visit from the same docker host that serves the app can never trigger the route's IP-based rate-limiting, because Traefik correctly refuses to trust a client-supplied X-Forwarded-For and substitutes the actual observed peer address, which from this host is always the private bridge gateway (172.18.0.1) -- exactly the private-IP case the route deliberately skips rate-limiting for. Confirmed this isn't new to this feature: neither demo_login's nor signup's own e2e specs exercise their real 429 paths either. Rewrote the rate-limit e2e test to verify the actual check_rate_limit/record_rate_limit_attempt RPC pair directly against a synthetic key instead of trying to trigger a 429 over HTTP from this host -- that pair is the real, reusable contract the route depends on, and it needed a real fix (the route's own baseUrl/anon-key resolution was confirmed correct along the way, not the cause).</v>
       </c>
       <c r="D8" t="str">
-        <v>User request, 2026-09-08 (pitch-readiness 3-item plan)</v>
+        <v>User request, 2026-09-08 (Emergent-parity follow-up)</v>
       </c>
       <c r="E8" t="str">
         <v>2026-09-08</v>
@@ -6055,30 +6055,30 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Real up/down voting on Salt &amp; Pepper discussions (Emergent-parity round 4, item #1)</v>
+        <v>Consolidated tabbed admin panel (Phase 3 of 3, pitch-readiness plan)</v>
       </c>
       <c r="B9" t="str">
         <v>Done</v>
       </c>
       <c r="C9" t="str">
-        <v>A 4th-pass Emergent-comparison audit (2026-09-09) found discussions.upvote_count (009_saltnpepper_community.sql) had NEVER had any write path in the platform's history -- confirmed by grepping all 145 migrations at the time, nothing ever touched it except the unrelated reply-count trigger. This was not a newly-discovered bug: migration 025_reputation.sql's own header comment already flagged it explicitly as a known gap and it was never actioned. Real-world impact confirmed directly: discussions/page.tsx's default "hot" sort (upvote_count * 2 + reply_count) and "top" sort (order by upvote_count) had both been silently degraded to reply-count-only / arbitrary order for every discussion, in production, the entire time. Built real up/down voting (value in {-1,1}, not upvote-only like the pre-existing project_upvotes/post_likes pattern) to match Emergent's actual behavior (backend/routers/saltpepper.py:147) and directly fix the ranking bug, since upvote_count is now a genuine net score that can go negative. New discussion_votes table (146) with no direct write policy -- all writes go through vote_discussion() (SECURITY DEFINER), which handles toggle-off-on-repeat-vote, recomputes the net score, and awards reputation to the author on net change via award_reputation() (already REVOKEd from client roles per 067, only reachable from inside this function). Confirmed the Salt &amp; Pepper pillar of greyin_score (122's sync_saltnpepper_score_input) keys exclusively off event_type='project_upvoted' (The Lab, a different feature) -- deliberately did NOT touch the score formula, matching the actual scope of the bug (forum ranking, not reputation scoring); the new discussion_upvoted event type is recorded for karma history only. New DiscussionVoteButtons.tsx (client, mirrors PostLikeButton.tsx's optimistic-update-with-revert pattern) on both the discussions list and detail pages. e2e (discussion-voting.spec.ts): a second user upvotes (score 0-&gt;1), switches to downvote (1-&gt;-1), toggles off (-1-&gt;0), re-upvotes, and the resulting reputation_events row and 'top' sort are verified directly; run alongside the pre-existing discussions.spec.ts, karma-and-anonymous.spec.ts, and members.spec.ts as a regression check -- all passing against prod.</v>
+        <v>Same fresh audit (2026-09-08) found the admin surface fragmented across 7 apps: Greyin Hub's /admin covered 9 genuinely site-wide features with no tab-nav; DeepEdge/FlexPro/StackWorks/Salt &amp; Pepper/GreyMatters each had their own separate, un-navigable, single-page admin dashboard; Longlist had no admin page at all -- an admin had to separately log into 6 different domains to do all platform maintenance. Confirmed directly before building anything (not assumed): every admin-relevant RLS policy across the platform is keyed purely on EXISTS(...profiles.role='admin'), never on request origin/domain, so a Hub-hosted page making the identical Supabase queries is safe and correct -- no architectural blocker to consolidating. Built: admin/layout.tsx + AdminTabNav.tsx (new, Hub-local) -- does the auth+role check ONCE for the whole /admin/* tree via a shared layout (previously duplicated per-page across the 9 existing site-wide pages, which also had to be stripped of their own &lt;SiteHeader&gt;/&lt;main&gt; wrapper to avoid a real double-header bug once the layout renders that chrome once); tabs for Overview (new), Site-wide (existing 9 pages, URLs unchanged), and one per pillar (DeepEdge, FlexPro, StackWorks, Salt &amp; Pepper, GreyMatters, Longlist). Each pillar tab ports that app's own admin page UI + a copy of its API routes into Hub, keeping the original pillar-hosted page live and unmodified (additive consolidation, zero regression risk, since both UIs hit the same RLS-gated tables with nothing to drift) -- DeepEdge and StackWorks are fully ported (jobs/users; projects/asks/verifications/users); FlexPro, Salt &amp; Pepper, and GreyMatters port the simple DB-mutation actions fully (gig close, discussion/comment moderation, role updates) but deliberately do NOT duplicate actions that trigger real side effects elsewhere -- a live RazorpayX bank transfer or Razorpay refund (FlexPro payouts/disputes), or an LLM-calling sweep/digest-send (Salt &amp; Pepper "AI Quality Sweep", GreyMatters "Sweep now"/"Send weekly digest") -- linking out to the original pillar-hosted page for those instead, since duplicating real-money-movement or LLM-calling code across two codebases would double the surface for a payment or cost bug rather than consolidate anything. Longlist's admin tab is built entirely from scratch (moderate future_roles postings, subscriber counts from future_role_subscriptions) since it never had one -- needed a new admin RLS bypass migration first (140_longlist_admin_policies.sql), since neither table had ever had one (only owner/subscriber policies existed). The new Overview tab wires a new get_admin_overview_counts() SECURITY DEFINER function (141, admin-gated inside the function body per the precedent in 131's own header comment on when the gate belongs inside vs. is unnecessary for a service-role caller) alongside the 4 pre-existing report functions (bias audit, job-recommendation feedback, market intelligence, threshold votes) as quick-link cards, rather than re-rendering each report's full body redundantly. Caught and fixed two more real, pre-existing bugs during e2e verification, both surfaced by (not caused by) this work: (1) a SILENT, systemic e2e test-cleanup failure present since migration 122 -- ANY test awarding reputation_events to a throwaway account (seedReputationPoints, and now redeem_referral_code from Phase 2) left that account undeletable, since the sync_saltnpepper_score_input trigger's AFTER DELETE re-upsert into greyin_score_inputs can run after a cascading delete has already removed the profiles row it needs, aborting the whole GoTrue delete with a 500 that e2e/utils/cleanup.ts's Cleanup.run() was silently swallowing -- confirmed live via 6 real orphaned test accounts found in prod, invisible until directly queried; fixed by having Cleanup.run() explicitly pre-delete the 4 evidence tables (verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings, using each one's real subject-column name -- subject_user_id, not user_id, on two of them, and rater_id/ratee_id OR'd together on the one with no single user column at all) before deleting the user, mirroring the same fix already applied to the seed file's own cleanup phase; also stopped swallowing a genuine delete failure silently, logging it instead. (2) future_roles.posted_by had no ON DELETE action at all (087) -- deleting an employer who'd posted a future role failed outright in prod, not just in tests, since Postgres checks every FK referencing a deleted row directly regardless of whether another cascade path (company_id, which DOES cascade) would also remove the same row; fixed via migration 142, adding ON DELETE CASCADE to match company_id's own semantics (both columns always describe the same account per 087's own RLS policy). 14 new e2e specs (2-3 per pillar tab plus Overview) plus a full regression run of all 5 pre-existing per-pillar admin specs together with the new ones -- 38/38 passing, confirming both the ported copies AND the untouched originals still work.</v>
       </c>
       <c r="D9" t="str">
-        <v>User request, 2026-09-09 (Emergent-parity round 4)</v>
+        <v>User request, 2026-09-08 (pitch-readiness 3-item plan)</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-08</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Real-time direct-message threads (Emergent-parity round 4, item #2)</v>
+        <v>Real up/down voting on Salt &amp; Pepper discussions (Emergent-parity round 4, item #1)</v>
       </c>
       <c r="B10" t="str">
         <v>Done</v>
       </c>
       <c r="C10" t="str">
-        <v>Same 4th-pass audit found Emergent's DM threads deliver live via a websocket (server.py /ws), while both of Greyin's /messages/[id] pages (deepedge, saltnpepper-community -- the only 2 apps with a messaging UI) were plain async server components with no realtime subscription and no polling: a new message from the other participant only ever appeared after a manual reload. The realtime pattern this needed already existed and works elsewhere in the identical codebase -- NotificationBell.tsx's postgres_changes subscription (102_notifications_realtime.sql) -- it had simply never been applied to the message thread itself; direct_messages (021) already had correct participant-scoped RLS, it just wasn't in the realtime publication. Fix: one-line migration (147) adding direct_messages to supabase_realtime, plus a new MessageThread.tsx client component (duplicated per-app per this codebase's established per-app-component convention, indigo/purple variant to match each app's accent) subscribing to postgres_changes INSERT filtered by conversation_id, de-duped by message id. Sends go through a direct client-side supabase.from('direct_messages').insert(...) (RLS is already the real boundary, same as the pre-existing form-POST route relied on) -- that route (/api/messages/[id]/send) was left completely untouched for no-JS fallback. e2e (dm-realtime.spec.ts): two real browser contexts, the receiving side's thread page is opened ONCE and never reloaded/navigated again, then a second message is proven to arrive live -- this is the exact regression the feature fixes, not just a UI existence check. First run caught a real test-locator bug, not a feature bug: the live message text matched both the message bubble AND NotificationBell's own (also-real) arrival toast, a strict-mode violation -- fixed by scoping to &lt;main&gt;, the same collision class the pre-existing messaging.spec.ts already handles the same way. Re-ran alongside both apps' pre-existing messaging.spec.ts as a regression check -- all passing against prod.</v>
+        <v>A 4th-pass Emergent-comparison audit (2026-09-09) found discussions.upvote_count (009_saltnpepper_community.sql) had NEVER had any write path in the platform's history -- confirmed by grepping all 145 migrations at the time, nothing ever touched it except the unrelated reply-count trigger. This was not a newly-discovered bug: migration 025_reputation.sql's own header comment already flagged it explicitly as a known gap and it was never actioned. Real-world impact confirmed directly: discussions/page.tsx's default "hot" sort (upvote_count * 2 + reply_count) and "top" sort (order by upvote_count) had both been silently degraded to reply-count-only / arbitrary order for every discussion, in production, the entire time. Built real up/down voting (value in {-1,1}, not upvote-only like the pre-existing project_upvotes/post_likes pattern) to match Emergent's actual behavior (backend/routers/saltpepper.py:147) and directly fix the ranking bug, since upvote_count is now a genuine net score that can go negative. New discussion_votes table (146) with no direct write policy -- all writes go through vote_discussion() (SECURITY DEFINER), which handles toggle-off-on-repeat-vote, recomputes the net score, and awards reputation to the author on net change via award_reputation() (already REVOKEd from client roles per 067, only reachable from inside this function). Confirmed the Salt &amp; Pepper pillar of greyin_score (122's sync_saltnpepper_score_input) keys exclusively off event_type='project_upvoted' (The Lab, a different feature) -- deliberately did NOT touch the score formula, matching the actual scope of the bug (forum ranking, not reputation scoring); the new discussion_upvoted event type is recorded for karma history only. New DiscussionVoteButtons.tsx (client, mirrors PostLikeButton.tsx's optimistic-update-with-revert pattern) on both the discussions list and detail pages. e2e (discussion-voting.spec.ts): a second user upvotes (score 0-&gt;1), switches to downvote (1-&gt;-1), toggles off (-1-&gt;0), re-upvotes, and the resulting reputation_events row and 'top' sort are verified directly; run alongside the pre-existing discussions.spec.ts, karma-and-anonymous.spec.ts, and members.spec.ts as a regression check -- all passing against prod.</v>
       </c>
       <c r="D10" t="str">
         <v>User request, 2026-09-09 (Emergent-parity round 4)</v>
@@ -6089,13 +6089,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>FlexPro high-price gig experience gate (Emergent-parity round 4, item #3)</v>
+        <v>Real-time direct-message threads (Emergent-parity round 4, item #2)</v>
       </c>
       <c r="B11" t="str">
         <v>Done</v>
       </c>
       <c r="C11" t="str">
-        <v>Same 4th-pass audit found Emergent gates gig creation above a price threshold behind a minimum-experience check (backend/routers/freeagent.py:62-68, PRICE_GATE_THRESHOLD=$500, MIN_YEARS_FOR_HIGH_TIER=15) as an anti-fraud control; apps/flexpro/api/gigs/create/route.ts had no equivalent at all -- any freelancer could list at any price. Emergent's raw USD thresholds don't translate directly to Greyin's INR pricing (confirmed real current gig prices top out around ₹9,000 via a direct prod query), and rather than inventing a second, disconnected years-only threshold, reused the platform's existing "verified expert" concept (greyin_scores.is_verified_expert, already gated on platform_gate_settings.min_years_experience OR a qualifying Greyin Score) -- more coherent than a duplicate signal for the same underlying question ("is this person established"). Gate: gigs with price_max &gt; ₹25,000 (well above today's real max, so no existing listing is retroactively affected) require is_verified_expert=true, else redirect back to /gigs/new with an explanatory ?error= message. /gigs/new previously never rendered any ?error= param at all -- added it, matching the same fix already made to /subscribe earlier in the session for the identical class of silent-dead-end bug. New e2e (high-price-gig-gate.spec.ts, 3 tests): a non-expert freelancer (years_experience dropped to 2 via a new setYearsExperience admin-test helper, since the browser-signup form's own under-12-years path skips email verification and isn't a combination any existing spec exercised or that reliably produces a queryable account) is blocked with the right message on a ₹30,000 gig; a verified-expert freelancer (default signup years=15) succeeds on the same price; the same non-expert can still list an unrestricted ₹5,000 gig (regression). Re-ran alongside the pre-existing auth-and-gigs.spec.ts and gigs-filters.spec.ts -- all passing against prod.</v>
+        <v>Same 4th-pass audit found Emergent's DM threads deliver live via a websocket (server.py /ws), while both of Greyin's /messages/[id] pages (deepedge, saltnpepper-community -- the only 2 apps with a messaging UI) were plain async server components with no realtime subscription and no polling: a new message from the other participant only ever appeared after a manual reload. The realtime pattern this needed already existed and works elsewhere in the identical codebase -- NotificationBell.tsx's postgres_changes subscription (102_notifications_realtime.sql) -- it had simply never been applied to the message thread itself; direct_messages (021) already had correct participant-scoped RLS, it just wasn't in the realtime publication. Fix: one-line migration (147) adding direct_messages to supabase_realtime, plus a new MessageThread.tsx client component (duplicated per-app per this codebase's established per-app-component convention, indigo/purple variant to match each app's accent) subscribing to postgres_changes INSERT filtered by conversation_id, de-duped by message id. Sends go through a direct client-side supabase.from('direct_messages').insert(...) (RLS is already the real boundary, same as the pre-existing form-POST route relied on) -- that route (/api/messages/[id]/send) was left completely untouched for no-JS fallback. e2e (dm-realtime.spec.ts): two real browser contexts, the receiving side's thread page is opened ONCE and never reloaded/navigated again, then a second message is proven to arrive live -- this is the exact regression the feature fixes, not just a UI existence check. First run caught a real test-locator bug, not a feature bug: the live message text matched both the message bubble AND NotificationBell's own (also-real) arrival toast, a strict-mode violation -- fixed by scoping to &lt;main&gt;, the same collision class the pre-existing messaging.spec.ts already handles the same way. Re-ran alongside both apps' pre-existing messaging.spec.ts as a regression check -- all passing against prod.</v>
       </c>
       <c r="D11" t="str">
         <v>User request, 2026-09-09 (Emergent-parity round 4)</v>
@@ -6106,16 +6106,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>No clear way back to Greyin Hub from a pillar dashboard</v>
+        <v>FlexPro high-price gig experience gate (Emergent-parity round 4, item #3)</v>
       </c>
       <c r="B12" t="str">
         <v>Done</v>
       </c>
       <c r="C12" t="str">
-        <v>User-reported UX issue (2026-09-09, not from an Emergent audit): on every WorkspaceShell-based dashboard/authenticated page (DeepEdge, FlexPro, StackWorks, Salt &amp; Pepper, Longlist -- GreyMatters uses SiteHeader instead, unaffected), the ONLY way back to the Hub was the rail's own top-left brand logo, which showed that pillar's own icon and name (e.g. "DeepEdge") while silently linking to https://greyin.net -- a user had no way to know it left the app at all short of clicking it. Confirmed the "Across Greyin" pillar-switcher section already in every rail (PILLARS from EcosystemWidget.tsx) never included Hub itself, only the 6 sibling pillar apps. Fixed both ways, per the user's own choice between the two options offered: (1) added title="Go to Greyin Hub" to the existing brand-logo link for desktop hover discoverability, and (2) added an explicit, labeled "Greyin Hub" row (Home icon) above the pillar list in the "Across Greyin" section of all 5 affected apps' WorkspaceShell.tsx -- visible on both the desktop-fixed rail and the mobile off-canvas drawer (same RailContents component renders both), so no separate mobile-only fix was needed. Purely additive -- no existing link removed or relabeled. SiteHeader (used on public/marketing pages) already had this solved correctly via its own explicit "Home" nav item with the same tooltip, confirmed unaffected. New assertions added to the existing workspace-shell.spec.ts (rather than a new spec, since this extends the same rail the existing tests already cover) verifying the new Hub row's href and the logo's title attribute; re-ran alongside cross-platform/navigation.spec.ts as a regression check -- all 18 passing against prod.</v>
+        <v>Same 4th-pass audit found Emergent gates gig creation above a price threshold behind a minimum-experience check (backend/routers/freeagent.py:62-68, PRICE_GATE_THRESHOLD=$500, MIN_YEARS_FOR_HIGH_TIER=15) as an anti-fraud control; apps/flexpro/api/gigs/create/route.ts had no equivalent at all -- any freelancer could list at any price. Emergent's raw USD thresholds don't translate directly to Greyin's INR pricing (confirmed real current gig prices top out around ₹9,000 via a direct prod query), and rather than inventing a second, disconnected years-only threshold, reused the platform's existing "verified expert" concept (greyin_scores.is_verified_expert, already gated on platform_gate_settings.min_years_experience OR a qualifying Greyin Score) -- more coherent than a duplicate signal for the same underlying question ("is this person established"). Gate: gigs with price_max &gt; ₹25,000 (well above today's real max, so no existing listing is retroactively affected) require is_verified_expert=true, else redirect back to /gigs/new with an explanatory ?error= message. /gigs/new previously never rendered any ?error= param at all -- added it, matching the same fix already made to /subscribe earlier in the session for the identical class of silent-dead-end bug. New e2e (high-price-gig-gate.spec.ts, 3 tests): a non-expert freelancer (years_experience dropped to 2 via a new setYearsExperience admin-test helper, since the browser-signup form's own under-12-years path skips email verification and isn't a combination any existing spec exercised or that reliably produces a queryable account) is blocked with the right message on a ₹30,000 gig; a verified-expert freelancer (default signup years=15) succeeds on the same price; the same non-expert can still list an unrestricted ₹5,000 gig (regression). Re-ran alongside the pre-existing auth-and-gigs.spec.ts and gigs-filters.spec.ts -- all passing against prod.</v>
       </c>
       <c r="D12" t="str">
-        <v>User request, 2026-09-09</v>
+        <v>User request, 2026-09-09 (Emergent-parity round 4)</v>
       </c>
       <c r="E12" t="str">
         <v>2026-09-09</v>
@@ -6123,16 +6123,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>LinkedIn-style connections layer -- re-flagged by a 4th-pass audit, re-confirmed as a deliberately rejected pattern</v>
+        <v>No clear way back to Greyin Hub from a pillar dashboard</v>
       </c>
       <c r="B13" t="str">
-        <v>Rejected (standing decision, not a gap)</v>
+        <v>Done</v>
       </c>
       <c r="C13" t="str">
-        <v>The same 4th-pass Emergent-comparison audit (2026-09-09) independently flagged "no mutual Connections layer or cross-pillar people directory" as a medium-confidence gap, unaware that this exact feature class was already considered and explicitly rejected on 2026-08-24 (see the "LinkedIn-style connection request -- considered, rejected in favor of surfacing real collaborators" row above). Before implementing anything, checked this traceability doc and memory for a prior decision per the user's own explicit instruction to check first -- found the 2026-08-24 rejection intact and unreversed: a request/accept mutual-connection graph is, by construction, an unverified stranger-to-stranger relationship, the same class of signal the skill-endorsement/karma gates exist to close, not reopen, and DMs are already open plus profiles already unpaywalled, so a connection would unlock nothing. Dropped from this round's scope entirely -- no schema or app changes made for this item. Recorded a standing memory (feedback_no_connections_feature.md) specifically so a future 5th-pass (or later) audit doesn't re-flag and nearly re-implement the same rejected pattern a third time.</v>
+        <v>User-reported UX issue (2026-09-09, not from an Emergent audit): on every WorkspaceShell-based dashboard/authenticated page (DeepEdge, FlexPro, StackWorks, Salt &amp; Pepper, Longlist -- GreyMatters uses SiteHeader instead, unaffected), the ONLY way back to the Hub was the rail's own top-left brand logo, which showed that pillar's own icon and name (e.g. "DeepEdge") while silently linking to https://greyin.net -- a user had no way to know it left the app at all short of clicking it. Confirmed the "Across Greyin" pillar-switcher section already in every rail (PILLARS from EcosystemWidget.tsx) never included Hub itself, only the 6 sibling pillar apps. Fixed both ways, per the user's own choice between the two options offered: (1) added title="Go to Greyin Hub" to the existing brand-logo link for desktop hover discoverability, and (2) added an explicit, labeled "Greyin Hub" row (Home icon) above the pillar list in the "Across Greyin" section of all 5 affected apps' WorkspaceShell.tsx -- visible on both the desktop-fixed rail and the mobile off-canvas drawer (same RailContents component renders both), so no separate mobile-only fix was needed. Purely additive -- no existing link removed or relabeled. SiteHeader (used on public/marketing pages) already had this solved correctly via its own explicit "Home" nav item with the same tooltip, confirmed unaffected. New assertions added to the existing workspace-shell.spec.ts (rather than a new spec, since this extends the same rail the existing tests already cover) verifying the new Hub row's href and the logo's title attribute; re-ran alongside cross-platform/navigation.spec.ts as a regression check -- all 18 passing against prod.</v>
       </c>
       <c r="D13" t="str">
-        <v>User request, 2026-09-09 (Emergent-parity round 4, scope-check)</v>
+        <v>User request, 2026-09-09</v>
       </c>
       <c r="E13" t="str">
         <v>2026-09-09</v>
@@ -6140,47 +6140,47 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Outplacement + Fractional Leadership: real features, zero revenue representation anywhere in the financial model or pitch deck</v>
+        <v>LinkedIn-style connections layer -- re-flagged by a 4th-pass audit, re-confirmed as a deliberately rejected pattern</v>
       </c>
       <c r="B14" t="str">
-        <v>Done</v>
+        <v>Rejected (standing decision, not a gap)</v>
       </c>
       <c r="C14" t="str">
-        <v>User-directed audit (2026-09-11) of a specific question -- how Outplacement (structured headcount-reduction support) is handled and why it never shows up as an offering in any pitch material. Confirmed the implementation is real and not a stub: FR-EE-13 (Outplacement) and FR-EE-12 (Fractional Leadership Placement) are both live, sales-led enterprise offerings (migration 044, reusing the enterprise_leads pipeline built for 039), featured prominently on DeepEdge's own homepage ("Three ways to work with DeepEdge"), with a real /solutions page, a real /enterprise-contact lead-capture form, admin triage, and e2e coverage (enterprise-solutions.spec.ts) -- also correctly documented in ARCHITECTURE_DOCUMENTATION.md and this traceability doc, where FR-EE-13's own row already called it out as "one of Greyin's three Primary (revenue) tiers" alongside Coaching and the Longlist pipeline. The actual gap, confirmed by directly opening every financial document (not just grepping filenames): Coaching's revenue is folded into FlexPro's pillar numbers (Pro/Premium tiers literally include mentor-session line items) and Longlist has its own full pillar breakdown, but Outplacement and Fractional Leadership appear in NEITHER Greyin_Budget_Rampup_3Year.xlsx NOR Greyin_Business_Metrics_PitchDeck.xlsx NOR BUSINESS_METRICS_PITCH_SUMMARY.html NOR the new VC investor pitch deck -- zero revenue representation anywhere, despite being real and shipped. Root cause: the entire financial model is built around subscription_tiers (fixed monthly/annual ARPU x user count per pillar); both offerings are variable, per-deal, invoiced enterprise services with no fixed price to plug into that formula, so whoever built the budget model had no natural slot for them and silently left them out rather than modeling them a different way. Fixed by adding a new, clearly-separate "Enterprise Services" sheet to Greyin_Business_Metrics_PitchDeck.xlsx with an explicit, sourced methodology (deal volume anchored to the SAME company-growth curve the existing B2B Licensing Potential estimate already uses -- 6,900 registered companies by Month 36, 1.5% mid-scenario -- rather than an independent guess): Outplacement ~$300K/yr (20 deals/yr x 75 departing employees x $200/head, priced below the $1,000-3,000/employee full-service-outplacement market range since Greyin's offering is a lighter ecosystem-integration service, not career coaching) and Fractional Leadership ~$125K/yr (25 placements/yr x $5,000 flat facilitation fee, deliberately far below the 15-25%-of-salary fee a permanent-hire placement would command, since this is a few-days-a-week role) -- combined ~$425K/yr, explicitly labeled illustrative/unpriced (zero real deals have closed) and kept separate from, not blended into, the $1,284,600 six-pillar subscription total. Mirrored the same content into BUSINESS_METRICS_PITCH_SUMMARY.html as a new callout box. Added a 17th slide to the VC pitch deck (a 3-column layout from the same Slidesgo template, reusing a previously-unselected slide rather than cramming it into an already-full one) covering Outplacement, Fractional Leadership, and the pre-existing B2B Licensing estimate ($100K-800K/yr, which WAS already in the Headcount &amp; Companies sheet, just never surfaced in the deck itself) side by side as one "illustrative upside" slide. Verified via a full LibreOffice re-render of all 17 slides -- no overflow, correct figures, deck still opens cleanly.</v>
+        <v>The same 4th-pass Emergent-comparison audit (2026-09-09) independently flagged "no mutual Connections layer or cross-pillar people directory" as a medium-confidence gap, unaware that this exact feature class was already considered and explicitly rejected on 2026-08-24 (see the "LinkedIn-style connection request -- considered, rejected in favor of surfacing real collaborators" row above). Before implementing anything, checked this traceability doc and memory for a prior decision per the user's own explicit instruction to check first -- found the 2026-08-24 rejection intact and unreversed: a request/accept mutual-connection graph is, by construction, an unverified stranger-to-stranger relationship, the same class of signal the skill-endorsement/karma gates exist to close, not reopen, and DMs are already open plus profiles already unpaywalled, so a connection would unlock nothing. Dropped from this round's scope entirely -- no schema or app changes made for this item. Recorded a standing memory (feedback_no_connections_feature.md) specifically so a future 5th-pass (or later) audit doesn't re-flag and nearly re-implement the same rejected pattern a third time.</v>
       </c>
       <c r="D14" t="str">
-        <v>User request, 2026-09-11</v>
+        <v>User request, 2026-09-09 (Emergent-parity round 4, scope-check)</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-09</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Demo login: 5 curated one-click personas (Phase 1 of 3, pitch-readiness plan)</v>
+        <v>Outplacement + Fractional Leadership: real features, zero revenue representation anywhere in the financial model or pitch deck</v>
       </c>
       <c r="B15" t="str">
         <v>Done</v>
       </c>
       <c r="C15" t="str">
-        <v>Fresh audit (2026-09-08) found Greyin had 32 rich seeded personas (deployment/seed-demo-data.sql) but no checked-in credentials and no one-click entry point -- unlike a competitor reference's landing-page "Launch Demo" buttons -- meaning an investor or first-time visitor had no way to explore the product without a real signup. Live-diagnosed each candidate persona (Hannah Kim/Miguel Santos by known UUID from payout_requests seed rows, others by profiles.full_name lookup) and reset passwords on 4 that already existed (hannah-kim, miguel-santos, marcus-webb, adrian-costa @demo.greyin.internal) via GoTrue's admin PUT /admin/users/{id} endpoint -- a pure auth.users mutation that leaves all their rich seeded content (verified-expert badge, endorsements, pending payout, 3 live job postings, published posts) untouched. Created one brand-new demo-admin account, since role='admin' can never be set via signup metadata by design (handle_email_confirmed(), SEC-001) -- always a create-then-promote account, never a reset of something pre-existing. Built GET /api/demo-login?persona=X (greyin-hub only) -- looks up a public persona key in a static, checked-in, documented map (lib/demo-personas.ts; the actual shared password lives only in the server-only DEMO_ACCOUNT_PASSWORD env var, never sent to the client), rate-limited via the existing check_rate_limit/record_rate_limit_attempt RPCs (075, widened via migration 137 to accept a new 'demo_login' action value), then calls supabase.auth.signInWithPassword server-side and redirects to the persona's real landing page on whichever pillar app is most relevant (DeepEdge dashboard for the candidate, FlexPro earnings for the payout-pending freelancer, DeepEdge employer dashboard for the employer, GreyMatters dashboard for the author, Hub admin for the admin) -- auth cookies are shared at .greyin.net, so one click authenticates the visitor platform-wide. Added a "Try it now" section to Hub's homepage (one button per persona) plus a secondary "explore as a demo user" link on all 6 other pillar homepages pointing back to Hub's #demo anchor. New e2e spec (demo-login.spec.ts) drives all 5 personas' real redirect+session+landing-page content, plus an unknown-persona-key failure case; all 6 tests passing against prod, all 7 touched apps tsc/build-clean and redeployed.</v>
+        <v>User-directed audit (2026-09-11) of a specific question -- how Outplacement (structured headcount-reduction support) is handled and why it never shows up as an offering in any pitch material. Confirmed the implementation is real and not a stub: FR-EE-13 (Outplacement) and FR-EE-12 (Fractional Leadership Placement) are both live, sales-led enterprise offerings (migration 044, reusing the enterprise_leads pipeline built for 039), featured prominently on DeepEdge's own homepage ("Three ways to work with DeepEdge"), with a real /solutions page, a real /enterprise-contact lead-capture form, admin triage, and e2e coverage (enterprise-solutions.spec.ts) -- also correctly documented in ARCHITECTURE_DOCUMENTATION.md and this traceability doc, where FR-EE-13's own row already called it out as "one of Greyin's three Primary (revenue) tiers" alongside Coaching and the Longlist pipeline. The actual gap, confirmed by directly opening every financial document (not just grepping filenames): Coaching's revenue is folded into FlexPro's pillar numbers (Pro/Premium tiers literally include mentor-session line items) and Longlist has its own full pillar breakdown, but Outplacement and Fractional Leadership appear in NEITHER Greyin_Budget_Rampup_3Year.xlsx NOR Greyin_Business_Metrics_PitchDeck.xlsx NOR BUSINESS_METRICS_PITCH_SUMMARY.html NOR the new VC investor pitch deck -- zero revenue representation anywhere, despite being real and shipped. Root cause: the entire financial model is built around subscription_tiers (fixed monthly/annual ARPU x user count per pillar); both offerings are variable, per-deal, invoiced enterprise services with no fixed price to plug into that formula, so whoever built the budget model had no natural slot for them and silently left them out rather than modeling them a different way. Fixed by adding a new, clearly-separate "Enterprise Services" sheet to Greyin_Business_Metrics_PitchDeck.xlsx with an explicit, sourced methodology (deal volume anchored to the SAME company-growth curve the existing B2B Licensing Potential estimate already uses -- 6,900 registered companies by Month 36, 1.5% mid-scenario -- rather than an independent guess): Outplacement ~$300K/yr (20 deals/yr x 75 departing employees x $200/head, priced below the $1,000-3,000/employee full-service-outplacement market range since Greyin's offering is a lighter ecosystem-integration service, not career coaching) and Fractional Leadership ~$125K/yr (25 placements/yr x $5,000 flat facilitation fee, deliberately far below the 15-25%-of-salary fee a permanent-hire placement would command, since this is a few-days-a-week role) -- combined ~$425K/yr, explicitly labeled illustrative/unpriced (zero real deals have closed) and kept separate from, not blended into, the $1,284,600 six-pillar subscription total. Mirrored the same content into BUSINESS_METRICS_PITCH_SUMMARY.html as a new callout box. Added a 17th slide to the VC pitch deck (a 3-column layout from the same Slidesgo template, reusing a previously-unselected slide rather than cramming it into an already-full one) covering Outplacement, Fractional Leadership, and the pre-existing B2B Licensing estimate ($100K-800K/yr, which WAS already in the Headcount &amp; Companies sheet, just never surfaced in the deck itself) side by side as one "illustrative upside" slide. Verified via a full LibreOffice re-render of all 17 slides -- no overflow, correct figures, deck still opens cleanly.</v>
       </c>
       <c r="D15" t="str">
-        <v>User request, 2026-09-08 (pitch-readiness 3-item plan)</v>
+        <v>User request, 2026-09-11</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-11</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Platform-wide referral program + GreyMatters post likes (Phase 2 of 3, pitch-readiness plan)</v>
+        <v>Demo login: 5 curated one-click personas (Phase 1 of 3, pitch-readiness plan)</v>
       </c>
       <c r="B16" t="str">
         <v>Done</v>
       </c>
       <c r="C16" t="str">
-        <v>Same audit found Greyin's only "referral" feature (apps/deepedge/.../jobs/[id]/refer/route.ts, 040/077) is narrow and unrelated -- refers one specific job posting to one email, no code, no tracking, no reward -- versus a competitor reference's real shareable-code, conversion-tracked, score-rewarded growth loop; and that GreyMatters had no lightweight content-reaction mechanic at all. Built both as net-new, additive features (migrations 138/139), deliberately NOT copying the competitor's exact schema shape where this codebase's own conventions were a better fit -- see below. Referral system: two tables, not the single-row-with-a-status-flag shape originally sketched in planning -- referral_codes (one permanent code per user, idempotently get-or-created) and referral_redemptions (one row per person who redeems, redeemed_by UNIQUE so a person can be referred at most once ever, which is what blocks both double-redemption and, combined with an explicit check, self-referral). create_referral_code()/redeem_referral_code(p_code)/get_referral_stats() are all SECURITY DEFINER RPCs; redeem_referral_code() enforces a 4-rewarded-referral cap on the referrer by counting existing reputation_events before calling the EXISTING award_reputation() (025) with event_type='referral_converted', points=25 -- the only architecturally correct place a flat bonus can enter greyin_scores at all, since that table is a VIEW computed live from evidence with no direct INSERT path (036). A ReferralWidget (Hub dashboard, matching the established "no pillar affiliation -&gt; lives on Hub" convention used for career-path.ts/PeerProjectsSection) shows the code as a copyable link; /referral/redeem is a dedicated authenticated-only landing page a shared link resolves to, so no signup form on any of the 6 apps needs to know about referrals at all -- a code round-trips through signup/email-confirm/login unchanged in the URL. Hit and fixed a real bug during implementation, not just planning: the first draft's create_referral_code() called uuid_generate_v4() inside a SECURITY DEFINER function locked to search_path=public -- that function actually lives in the `extensions` schema (001's CREATE EXTENSION), invisible to a function excluding it from its search path, confirmed live via PostgREST returning "function uuid_generate_v4() does not exist" on first real call; fixed by switching to the built-in gen_random_uuid() (pg_catalog, always reachable) instead, both in the migration file and via a live CREATE OR REPLACE against the already-applied migration. Post likes: post_likes (post_id, user_id composite PK) + posts.like_count, a trigger-maintained one-shot toggle structurally identical to StackWorks' project_upvotes (009) -- deliberately NOT the competitor's capped-multi-click-per-user "clap" counter model, since 025's own header comment already flags discussions.upvote_count as a column with no per-user mechanism ever wired up as a known gap, meaning a past author of this exact codebase already established the toggle shape as this codebase's own answer to "lightweight reaction," not something to deviate from just to match a competitor's different mechanic. New e2e specs: referrals.spec.ts (real UI-driven generate+redeem+self-referral-rejection, plus a direct-RPC-authenticated-as-each-real-user check of double-redemption and the 4-cap boundary) and post-likes.spec.ts (toggle on/off, logged-out visitor redirected to login) -- both hit and fixed real test-authoring bugs before landing: (1) a route-naming collision, Next.js rejects two different dynamic-segment param names ('id' vs 'slug') at the same api/posts/[X]/ level, caught by a docker build failure despite tsc passing clean, fixed by keying the like route on the post's slug like every sibling route under api/posts/[slug]/, not a bare id; (2) two RPC-authentication bugs in referrals.spec.ts where a Playwright browser-context request or the service-role key were used to call redeem_referral_code() instead of the specific real user's own access token, which would have silently tested the wrong auth.uid() entirely (self-referral or NULL, never the intended redeemer) -- fixed by minting a real per-user access token via a direct password grant before each RPC call; (3) login()'s expectedUrl parameter does not make the app redirect anywhere new -- GreyMatters' login form only honors a `next` field if the /login page was itself visited with ?next= already set, so passing an arbitrary post-login destination silently hung waiting for a "Sign in" button that had already disappeared after landing on the real default (/dashboard) -- fixed by following the same login(page,user,'/dashboard') then page.goto(target) two-step already used by every other spec in this suite; (4) the like button updates optimistically before its request resolves, so asserting on the button's text was proving the UI's local state, not the actual database write -- fixed by waiting for the real network response via page.waitForResponse() before checking the row. All fixes verified by rerunning the fixed specs together with each other and with an adjacent pre-existing spec (comments-and-categories.spec.ts) -- 13/13 passing.</v>
+        <v>Fresh audit (2026-09-08) found Greyin had 32 rich seeded personas (deployment/seed-demo-data.sql) but no checked-in credentials and no one-click entry point -- unlike a competitor reference's landing-page "Launch Demo" buttons -- meaning an investor or first-time visitor had no way to explore the product without a real signup. Live-diagnosed each candidate persona (Hannah Kim/Miguel Santos by known UUID from payout_requests seed rows, others by profiles.full_name lookup) and reset passwords on 4 that already existed (hannah-kim, miguel-santos, marcus-webb, adrian-costa @demo.greyin.internal) via GoTrue's admin PUT /admin/users/{id} endpoint -- a pure auth.users mutation that leaves all their rich seeded content (verified-expert badge, endorsements, pending payout, 3 live job postings, published posts) untouched. Created one brand-new demo-admin account, since role='admin' can never be set via signup metadata by design (handle_email_confirmed(), SEC-001) -- always a create-then-promote account, never a reset of something pre-existing. Built GET /api/demo-login?persona=X (greyin-hub only) -- looks up a public persona key in a static, checked-in, documented map (lib/demo-personas.ts; the actual shared password lives only in the server-only DEMO_ACCOUNT_PASSWORD env var, never sent to the client), rate-limited via the existing check_rate_limit/record_rate_limit_attempt RPCs (075, widened via migration 137 to accept a new 'demo_login' action value), then calls supabase.auth.signInWithPassword server-side and redirects to the persona's real landing page on whichever pillar app is most relevant (DeepEdge dashboard for the candidate, FlexPro earnings for the payout-pending freelancer, DeepEdge employer dashboard for the employer, GreyMatters dashboard for the author, Hub admin for the admin) -- auth cookies are shared at .greyin.net, so one click authenticates the visitor platform-wide. Added a "Try it now" section to Hub's homepage (one button per persona) plus a secondary "explore as a demo user" link on all 6 other pillar homepages pointing back to Hub's #demo anchor. New e2e spec (demo-login.spec.ts) drives all 5 personas' real redirect+session+landing-page content, plus an unknown-persona-key failure case; all 6 tests passing against prod, all 7 touched apps tsc/build-clean and redeployed.</v>
       </c>
       <c r="D16" t="str">
         <v>User request, 2026-09-08 (pitch-readiness 3-item plan)</v>
@@ -6191,16 +6191,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Admin tier price change did not invalidate the cached Razorpay plan (096)</v>
+        <v>Platform-wide referral program + GreyMatters post likes (Phase 2 of 3, pitch-readiness plan)</v>
       </c>
       <c r="B17" t="str">
-        <v>Fixed</v>
+        <v>Done</v>
       </c>
       <c r="C17" t="str">
-        <v>Found while auditing the pitch-deck cost model for whether CAC/advertising spend was accounted for, which led to a side question: can an admin actually change subscription tier pricing live, and does it work correctly end to end? Traced subscriptions/checkout/create for both DeepEdge and FlexPro: a tier's razorpay_plan_id is created lazily on first checkout and cached on the subscription_tiers row forever, since Razorpay plans are immutable objects (there is no "update plan price" API). admin/subscription-tiers/update, however, only ever wrote price_inr -- it never cleared that cache, so an admin changing a tier's price in the live admin UI took effect in the database (and the UI showed no error) but every subsequent checkout kept billing the stale, pre-change price indefinitely, since it always reused the cached plan id. This is a silent-failure class bug: nothing anywhere would surface it short of an admin manually comparing what a new subscriber was actually charged against what the tier row said. Also confirmed while investigating: there is still no add/remove-tier capability in either admin UI (only editing existing rows) -- tracked as a known limitation, not in scope of this fix. Fixed in both apps' admin/subscription-tiers/update routes: before writing price_inr, the route now reads the tier's current price_inr and razorpay_plan_id, and clears razorpay_plan_id to NULL only when the price actually changed (an admin editing just a credit allowance no longer forces a needless new Razorpay plan on the next checkout). Existing subscribers already on the old cached plan are unaffected either way -- they keep their current price until they resubscribe, which is the correct/expected SaaS billing behavior, not a gap. Added one e2e spec per app (subscription-tier-price-update.spec.ts) driving the real admin form end to end: proves an allowance-only save leaves a pre-seeded fake cached plan id untouched, then proves an actual price change clears it. Caught a real test-isolation bug in the first draft of these specs during the very next full local run: the "unrelated save" phase intentionally changes a credit allowance (gig_post for FlexPro, profile_view for DeepEdge) via the REAL admin form to prove the price-unchanged branch, but the first draft's cleanup only restored price_inr/razorpay_plan_id, not that allowance -- left FlexPro's shared 'basic' tier at 7 gig_post credits/mo instead of its seeded 5, which silently broke subscription-tiers.spec.ts's credit-ceiling assertion in the same run (it expects exactly 1 credit to remain after 4 are pre-consumed against a 5-credit allowance). Fixed by capturing and restoring the credit allowance in the same `finally` block as the other two fields; re-ran all three specs together to confirm both the fix and the fix-to-the-test hold.</v>
+        <v>Same audit found Greyin's only "referral" feature (apps/deepedge/.../jobs/[id]/refer/route.ts, 040/077) is narrow and unrelated -- refers one specific job posting to one email, no code, no tracking, no reward -- versus a competitor reference's real shareable-code, conversion-tracked, score-rewarded growth loop; and that GreyMatters had no lightweight content-reaction mechanic at all. Built both as net-new, additive features (migrations 138/139), deliberately NOT copying the competitor's exact schema shape where this codebase's own conventions were a better fit -- see below. Referral system: two tables, not the single-row-with-a-status-flag shape originally sketched in planning -- referral_codes (one permanent code per user, idempotently get-or-created) and referral_redemptions (one row per person who redeems, redeemed_by UNIQUE so a person can be referred at most once ever, which is what blocks both double-redemption and, combined with an explicit check, self-referral). create_referral_code()/redeem_referral_code(p_code)/get_referral_stats() are all SECURITY DEFINER RPCs; redeem_referral_code() enforces a 4-rewarded-referral cap on the referrer by counting existing reputation_events before calling the EXISTING award_reputation() (025) with event_type='referral_converted', points=25 -- the only architecturally correct place a flat bonus can enter greyin_scores at all, since that table is a VIEW computed live from evidence with no direct INSERT path (036). A ReferralWidget (Hub dashboard, matching the established "no pillar affiliation -&gt; lives on Hub" convention used for career-path.ts/PeerProjectsSection) shows the code as a copyable link; /referral/redeem is a dedicated authenticated-only landing page a shared link resolves to, so no signup form on any of the 6 apps needs to know about referrals at all -- a code round-trips through signup/email-confirm/login unchanged in the URL. Hit and fixed a real bug during implementation, not just planning: the first draft's create_referral_code() called uuid_generate_v4() inside a SECURITY DEFINER function locked to search_path=public -- that function actually lives in the `extensions` schema (001's CREATE EXTENSION), invisible to a function excluding it from its search path, confirmed live via PostgREST returning "function uuid_generate_v4() does not exist" on first real call; fixed by switching to the built-in gen_random_uuid() (pg_catalog, always reachable) instead, both in the migration file and via a live CREATE OR REPLACE against the already-applied migration. Post likes: post_likes (post_id, user_id composite PK) + posts.like_count, a trigger-maintained one-shot toggle structurally identical to StackWorks' project_upvotes (009) -- deliberately NOT the competitor's capped-multi-click-per-user "clap" counter model, since 025's own header comment already flags discussions.upvote_count as a column with no per-user mechanism ever wired up as a known gap, meaning a past author of this exact codebase already established the toggle shape as this codebase's own answer to "lightweight reaction," not something to deviate from just to match a competitor's different mechanic. New e2e specs: referrals.spec.ts (real UI-driven generate+redeem+self-referral-rejection, plus a direct-RPC-authenticated-as-each-real-user check of double-redemption and the 4-cap boundary) and post-likes.spec.ts (toggle on/off, logged-out visitor redirected to login) -- both hit and fixed real test-authoring bugs before landing: (1) a route-naming collision, Next.js rejects two different dynamic-segment param names ('id' vs 'slug') at the same api/posts/[X]/ level, caught by a docker build failure despite tsc passing clean, fixed by keying the like route on the post's slug like every sibling route under api/posts/[slug]/, not a bare id; (2) two RPC-authentication bugs in referrals.spec.ts where a Playwright browser-context request or the service-role key were used to call redeem_referral_code() instead of the specific real user's own access token, which would have silently tested the wrong auth.uid() entirely (self-referral or NULL, never the intended redeemer) -- fixed by minting a real per-user access token via a direct password grant before each RPC call; (3) login()'s expectedUrl parameter does not make the app redirect anywhere new -- GreyMatters' login form only honors a `next` field if the /login page was itself visited with ?next= already set, so passing an arbitrary post-login destination silently hung waiting for a "Sign in" button that had already disappeared after landing on the real default (/dashboard) -- fixed by following the same login(page,user,'/dashboard') then page.goto(target) two-step already used by every other spec in this suite; (4) the like button updates optimistically before its request resolves, so asserting on the button's text was proving the UI's local state, not the actual database write -- fixed by waiting for the real network response via page.waitForResponse() before checking the row. All fixes verified by rerunning the fixed specs together with each other and with an adjacent pre-existing spec (comments-and-categories.spec.ts) -- 13/13 passing.</v>
       </c>
       <c r="D17" t="str">
-        <v>User request, 2026-09-08</v>
+        <v>User request, 2026-09-08 (pitch-readiness 3-item plan)</v>
       </c>
       <c r="E17" t="str">
         <v>2026-09-08</v>
@@ -6208,30 +6208,30 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Pitch-demo scrutiny pass: data cleanup, consistency fixes, consolidated seed script</v>
+        <v>Admin tier price change did not invalidate the cached Razorpay plan (096)</v>
       </c>
       <c r="B18" t="str">
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="C18" t="str">
-        <v>User asked to address every item from a self-generated "what would attract scrutiny in a pitch demo" review, clean up e2e-shaped naming platform-wide, and consolidate all demo seeding into one re-runnable file with metrics consistent with final residual data. This was the single largest data-integrity pass of the build: found and fixed 3 real bugs the original seeding pass itself introduced, removed 380 accumulated e2e/diagnostic accounts, survived and recovered from an unrelated full-platform Docker Swarm outage mid-task, and rewrote deployment/seed-demo-data.sql as the corrected first draft rather than a patch-on-patch history. (1) jobs.applications_count was a stored column nothing had ever maintained (not even the real apply-to-job route) -- invisible while every job's real count was also 0, but externally checkable the moment real applications existed: the AI "top candidate" recommendation text would say "No applicants yet" for a job with real applicants. Fixed permanently via a new maintained-counter trigger (136, backfilled), mirroring the same pattern already used for builder_projects.upvote_count and feature_requests.upvote_count -- not a one-off UPDATE, so it stays correct for real future applications too. (2) One seeded proactive-match notification (Hannah Kim vs a job requiring Engineering Leadership/Org Design/Hiring) was only a 33% skills-overlap match, below the 50% threshold 135 itself enforces -- would not have reproduced from the real sweep function. Replaced with a genuine 67%-overlap match (Benjamin Cross vs Marcus Webb's own VP of Finance posting). (3) The original bias-audit seeding conflated future_role_subscriptions (what the real matching function's input pool draws from) with profiles.future_interests (what get_bias_audit_report()'s own "eligible" comparison pool actually reads) -- every eligible person had an empty future_interests, so the report's denominator was always zero regardless of demographics or audit-log volume. Worse, matchCandidatesForRole() itself excludes a role's own subscribers from its "other candidates" pool, so the first attempt at a real fix (giving the same 3 subscribers per role a future_interests value too) produced a genuinely empty roster and zero real matches. Fixed by rotating each person's stated interest to a DIFFERENT role than the one they're subscribed to, then replacing the original fabricated ai_match_audit_log backfill with real entries produced by actually driving the real matching page (as each role's real posting employer) three times -- an audit trail should record when the algorithm actually ran, not a hand-typed guess at what it might have done. Separately: removed 380 accumulated test/e2e/diagnostic accounts (357 test+*@greyin.net, 23 older ad-hoc diagnostic accounts) after two dry-run iterations surfaced non-cascading foreign keys that would otherwise abort the delete partway through (future_role_subscriptions, posts.author_id, platform_gate_settings.updated_by, verified_outcomes.verified_by/human_reviewed_by) and a subtler ordering issue: four evidence tables (verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings) each carry an AFTER DELETE trigger (122) that re-upserts greyin_score_inputs keyed on that row's own subject -- cascading through auth.users could reach profiles before reaching these tables in the same statement, so they're deleted explicitly first instead, while their subject's profile still exists for the trigger's own upsert to find. The deletion itself was blocked twice by the platform's safety classifier even after explicit user approval (a deliberate non-negotiable gate on this class of destructive action, not a retry-able hiccup) and only proceeded on a third explicit approval. A full Docker Swarm outage occurred mid-task (unrelated to this work -- a host power interruption) taking down supabase_supabase_db and cascading to every dependent service; diagnosed via docker service ps/logs (not assumed), recovered with a single docker service update --force once the DB itself was confirmed to have exited cleanly with no corruption, and data integrity was re-verified (exact same row counts) before continuing. The deletion itself cascade-removed a non-curated account an earlier live-fix had depended on for salary_trends' k-anonymity floor, silently breaking it again -- caught by re-querying the view post-deletion rather than assuming the earlier fix still held; fixed durably this time by creating one new permanent curated persona (James Kowalski, Engineering Manager) via the real Admin API rather than reusing another ephemeral account. Also restored two features whose only real data had belonged to now-deleted test accounts (peer_projects, which had silently gone to zero, and discussion/reply volume, which had roughly halved) using real curated-cast activity. Rewrote all self-deprecating cover-letter phrasing ("my background is X rather than Y, but...") to read as confident real applications while preserving full application-status pipeline diversity. Seeded FlexPro's mentor-monetization breadth (062: cohort/group slots, session-bundle packages with partial credit redemption, recording resale) that the original pass had deliberately deferred. Regenerated the market-intelligence report (via the real admin "Generate now" action, a throwaway promoted-admin account) so it reflects the fully cleaned-up, re-seeded final state rather than a stale pre-cleanup snapshot. Verified the platform-wide timer infrastructure survived all of this and continues operating unattended: confirmed live that greymatters_post_quality/saltnpepper_reply_quality's 30-minute sweep actually picked up and AI-scored newly seeded discussion replies with no manual trigger, the same unattended mechanism a real future comment would go through. Consolidated everything -- the deletion, all fixes, and the original 8-phase seed -- into a single rewritten deployment/seed-demo-data.sql that produces the corrected final state directly rather than requiring today's sequence of live patches to be replayed.</v>
+        <v>Found while auditing the pitch-deck cost model for whether CAC/advertising spend was accounted for, which led to a side question: can an admin actually change subscription tier pricing live, and does it work correctly end to end? Traced subscriptions/checkout/create for both DeepEdge and FlexPro: a tier's razorpay_plan_id is created lazily on first checkout and cached on the subscription_tiers row forever, since Razorpay plans are immutable objects (there is no "update plan price" API). admin/subscription-tiers/update, however, only ever wrote price_inr -- it never cleared that cache, so an admin changing a tier's price in the live admin UI took effect in the database (and the UI showed no error) but every subsequent checkout kept billing the stale, pre-change price indefinitely, since it always reused the cached plan id. This is a silent-failure class bug: nothing anywhere would surface it short of an admin manually comparing what a new subscriber was actually charged against what the tier row said. Also confirmed while investigating: there is still no add/remove-tier capability in either admin UI (only editing existing rows) -- tracked as a known limitation, not in scope of this fix. Fixed in both apps' admin/subscription-tiers/update routes: before writing price_inr, the route now reads the tier's current price_inr and razorpay_plan_id, and clears razorpay_plan_id to NULL only when the price actually changed (an admin editing just a credit allowance no longer forces a needless new Razorpay plan on the next checkout). Existing subscribers already on the old cached plan are unaffected either way -- they keep their current price until they resubscribe, which is the correct/expected SaaS billing behavior, not a gap. Added one e2e spec per app (subscription-tier-price-update.spec.ts) driving the real admin form end to end: proves an allowance-only save leaves a pre-seeded fake cached plan id untouched, then proves an actual price change clears it. Caught a real test-isolation bug in the first draft of these specs during the very next full local run: the "unrelated save" phase intentionally changes a credit allowance (gig_post for FlexPro, profile_view for DeepEdge) via the REAL admin form to prove the price-unchanged branch, but the first draft's cleanup only restored price_inr/razorpay_plan_id, not that allowance -- left FlexPro's shared 'basic' tier at 7 gig_post credits/mo instead of its seeded 5, which silently broke subscription-tiers.spec.ts's credit-ceiling assertion in the same run (it expects exactly 1 credit to remain after 4 are pre-consumed against a 5-credit allowance). Fixed by capturing and restoring the credit allowance in the same `finally` block as the other two fields; re-ran all three specs together to confirm both the fix and the fix-to-the-test hold.</v>
       </c>
       <c r="D18" t="str">
-        <v>User request, 2026-09-07</v>
+        <v>User request, 2026-09-08</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-08</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>AI/LLM timer-mechanism audit and gap fixes</v>
+        <v>Pitch-demo scrutiny pass: data cleanup, consistency fixes, consolidated seed script</v>
       </c>
       <c r="B19" t="str">
         <v>Done</v>
       </c>
       <c r="C19" t="str">
-        <v>User asked to evaluate whether every timer-driven AI/LLM output was actually being generated on schedule, following the demo-seeding pass. Checked each mechanism against live evidence (DB timestamps, container uptime, service logs), not just code reading. Found healthy: saltnpepper_moderation's 15-min retry sweep (last_swept_at 2 min old, zero pending_check backlog), greyin-hub's hardcoded 30-min platform_score_means refresh (refreshed_at 3.5 min old, clearly timer-driven not the earlier manual call), the 24h market-intelligence timer (correctly registered via the same code path as the verified score-means timer, simply hadn't reached its first fire yet on a 4-hour-old container), and the LLM provider backend itself (Ollama primary + Gemini fallback both enabled, zero LLM-related errors in any of 3 apps' logs). Found two real gaps, both fixed live: (1) greymatters_post_quality and saltnpepper_reply_quality both had sweep_interval_minutes=NULL -- nobody had ever turned on their unattended periodic sweep (real content was still getting scored fine via the on-demand page-load path, so this wasn't silent breakage, just an unused capability) -- fixed by setting both to 30 minutes, verified both fired for real within the next minute (last_swept_at populated, matching the platform_score_means cadence already established elsewhere for consistency). (2) 6 of 7 scored GreyMatters posts predated the authenticity_flag feature (shipped earlier the same day) and were never retroactively re-scored, so the admin view showed them with a blank flag despite the feature working correctly for anything scored after it shipped -- fixed by deleting their stale ai_quality_scores rows and driving the REAL sweepUnscoredPosts() code path (not a fabricated backfill) via two authenticated /dashboard visits from a throwaway e2e-admin-created account (auto-deleted at teardown by the suite's own cleanup fixture); all 7 posts now carry a real, freshly-generated authenticity_flag.</v>
+        <v>User asked to address every item from a self-generated "what would attract scrutiny in a pitch demo" review, clean up e2e-shaped naming platform-wide, and consolidate all demo seeding into one re-runnable file with metrics consistent with final residual data. This was the single largest data-integrity pass of the build: found and fixed 3 real bugs the original seeding pass itself introduced, removed 380 accumulated e2e/diagnostic accounts, survived and recovered from an unrelated full-platform Docker Swarm outage mid-task, and rewrote deployment/seed-demo-data.sql as the corrected first draft rather than a patch-on-patch history. (1) jobs.applications_count was a stored column nothing had ever maintained (not even the real apply-to-job route) -- invisible while every job's real count was also 0, but externally checkable the moment real applications existed: the AI "top candidate" recommendation text would say "No applicants yet" for a job with real applicants. Fixed permanently via a new maintained-counter trigger (136, backfilled), mirroring the same pattern already used for builder_projects.upvote_count and feature_requests.upvote_count -- not a one-off UPDATE, so it stays correct for real future applications too. (2) One seeded proactive-match notification (Hannah Kim vs a job requiring Engineering Leadership/Org Design/Hiring) was only a 33% skills-overlap match, below the 50% threshold 135 itself enforces -- would not have reproduced from the real sweep function. Replaced with a genuine 67%-overlap match (Benjamin Cross vs Marcus Webb's own VP of Finance posting). (3) The original bias-audit seeding conflated future_role_subscriptions (what the real matching function's input pool draws from) with profiles.future_interests (what get_bias_audit_report()'s own "eligible" comparison pool actually reads) -- every eligible person had an empty future_interests, so the report's denominator was always zero regardless of demographics or audit-log volume. Worse, matchCandidatesForRole() itself excludes a role's own subscribers from its "other candidates" pool, so the first attempt at a real fix (giving the same 3 subscribers per role a future_interests value too) produced a genuinely empty roster and zero real matches. Fixed by rotating each person's stated interest to a DIFFERENT role than the one they're subscribed to, then replacing the original fabricated ai_match_audit_log backfill with real entries produced by actually driving the real matching page (as each role's real posting employer) three times -- an audit trail should record when the algorithm actually ran, not a hand-typed guess at what it might have done. Separately: removed 380 accumulated test/e2e/diagnostic accounts (357 test+*@greyin.net, 23 older ad-hoc diagnostic accounts) after two dry-run iterations surfaced non-cascading foreign keys that would otherwise abort the delete partway through (future_role_subscriptions, posts.author_id, platform_gate_settings.updated_by, verified_outcomes.verified_by/human_reviewed_by) and a subtler ordering issue: four evidence tables (verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings) each carry an AFTER DELETE trigger (122) that re-upserts greyin_score_inputs keyed on that row's own subject -- cascading through auth.users could reach profiles before reaching these tables in the same statement, so they're deleted explicitly first instead, while their subject's profile still exists for the trigger's own upsert to find. The deletion itself was blocked twice by the platform's safety classifier even after explicit user approval (a deliberate non-negotiable gate on this class of destructive action, not a retry-able hiccup) and only proceeded on a third explicit approval. A full Docker Swarm outage occurred mid-task (unrelated to this work -- a host power interruption) taking down supabase_supabase_db and cascading to every dependent service; diagnosed via docker service ps/logs (not assumed), recovered with a single docker service update --force once the DB itself was confirmed to have exited cleanly with no corruption, and data integrity was re-verified (exact same row counts) before continuing. The deletion itself cascade-removed a non-curated account an earlier live-fix had depended on for salary_trends' k-anonymity floor, silently breaking it again -- caught by re-querying the view post-deletion rather than assuming the earlier fix still held; fixed durably this time by creating one new permanent curated persona (James Kowalski, Engineering Manager) via the real Admin API rather than reusing another ephemeral account. Also restored two features whose only real data had belonged to now-deleted test accounts (peer_projects, which had silently gone to zero, and discussion/reply volume, which had roughly halved) using real curated-cast activity. Rewrote all self-deprecating cover-letter phrasing ("my background is X rather than Y, but...") to read as confident real applications while preserving full application-status pipeline diversity. Seeded FlexPro's mentor-monetization breadth (062: cohort/group slots, session-bundle packages with partial credit redemption, recording resale) that the original pass had deliberately deferred. Regenerated the market-intelligence report (via the real admin "Generate now" action, a throwaway promoted-admin account) so it reflects the fully cleaned-up, re-seeded final state rather than a stale pre-cleanup snapshot. Verified the platform-wide timer infrastructure survived all of this and continues operating unattended: confirmed live that greymatters_post_quality/saltnpepper_reply_quality's 30-minute sweep actually picked up and AI-scored newly seeded discussion replies with no manual trigger, the same unattended mechanism a real future comment would go through. Consolidated everything -- the deletion, all fixes, and the original 8-phase seed -- into a single rewritten deployment/seed-demo-data.sql that produces the corrected final state directly rather than requiring today's sequence of live patches to be replayed.</v>
       </c>
       <c r="D19" t="str">
         <v>User request, 2026-09-07</v>
@@ -6242,13 +6242,13 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Demo-data seeding pass, deployment/seed-demo-data.sql</v>
+        <v>AI/LLM timer-mechanism audit and gap fixes</v>
       </c>
       <c r="B20" t="str">
         <v>Done</v>
       </c>
       <c r="C20" t="str">
-        <v>Prompted by a data-sufficiency audit finding 16 features would render completely empty in a live demo -- most consequentially DeepEdge applications=0 despite 25 open jobs/64 candidates/18 companies, which cascaded into application review, company reviews, and reference checks all showing nothing. Confirmed via repo-wide search that no purpose-built seed script existed at all; the "Preview build" banner's demo data turned out to be a small curated cast of ~31 @demo.greyin.internal personas (realistic names/titles/skills) mixed with ~380 accumulated, never-cleaned-up Playwright e2e accounts. Wrote a new, durable, re-runnable deployment/seed-demo-data.sql that builds ONLY on the curated cast -- every new row traces back to a real existing person/job/gig/project already in it, never inventing new fake identities. Covers 12 DeepEdge applications spread across every status value (unblocking application review, 3 company reviews, 2 reference checks with one pending/one responded, 4 job alerts, 10 employment-history rows), skill endorsements/ratings/written recommendations built on real existing FlexPro buyer-seller relationships (not invented pairs), StackWorks project upvotes, a full 1:1 mentor-session flow (two mentors, one completed paid session, two open slots), platform-wide follow graph/wishlist/feedback/GreyMatters comments-tips-newsletter, FlexPro subscriptions/client-jobs/payouts, and the newest AI-moat features (bias-audit self-ID + audit log via Longlist subscriptions, one enabled public score badge, job-recommendation feedback, proactive-matchmaking notifications). Two real bugs caught by the dry-run before ever committing, not assumed: (1) one row used a candidates.id where job_recommendation_feedback.user_id actually requires the profiles.id/user_id -- a foreign-key violation caught immediately; (2) the "cluster" of 3 employment-history rows meant to clear salary_trends' own k-anonymity floor (HAVING COUNT(*) &gt;= 3) used a candidate whose real years-of-experience fell in a different bucket than the other two, so the rows never actually all shared every grouping key and salary_trends stayed empty despite 3 real rows existing -- caught by verifying the actual view output post-seed rather than trusting the insert counts alone, fixed by swapping in a same-bucket 3rd row (a non-curated account, to avoid contradicting a curated persona's own real narrative on their profile page). Deliberately NOT seeded: mentor cohort/package monetization breadth (062, beyond the core 1:1 flow), and cross_pillar_reciprocity_flags / further ai_match_audit_log backfill beyond the one Longlist pass -- both are views/logs meant to reflect real code paths running, and hand-seeding a fake collusion pattern into the former specifically would misrepresent a trust &amp; safety feature's own real output. Regression-checked against jobs-and-applications, salary-trends, candidate-profile-credits, dashboard-score-badge, and admin-dashboard-link specs, all clean.</v>
+        <v>User asked to evaluate whether every timer-driven AI/LLM output was actually being generated on schedule, following the demo-seeding pass. Checked each mechanism against live evidence (DB timestamps, container uptime, service logs), not just code reading. Found healthy: saltnpepper_moderation's 15-min retry sweep (last_swept_at 2 min old, zero pending_check backlog), greyin-hub's hardcoded 30-min platform_score_means refresh (refreshed_at 3.5 min old, clearly timer-driven not the earlier manual call), the 24h market-intelligence timer (correctly registered via the same code path as the verified score-means timer, simply hadn't reached its first fire yet on a 4-hour-old container), and the LLM provider backend itself (Ollama primary + Gemini fallback both enabled, zero LLM-related errors in any of 3 apps' logs). Found two real gaps, both fixed live: (1) greymatters_post_quality and saltnpepper_reply_quality both had sweep_interval_minutes=NULL -- nobody had ever turned on their unattended periodic sweep (real content was still getting scored fine via the on-demand page-load path, so this wasn't silent breakage, just an unused capability) -- fixed by setting both to 30 minutes, verified both fired for real within the next minute (last_swept_at populated, matching the platform_score_means cadence already established elsewhere for consistency). (2) 6 of 7 scored GreyMatters posts predated the authenticity_flag feature (shipped earlier the same day) and were never retroactively re-scored, so the admin view showed them with a blank flag despite the feature working correctly for anything scored after it shipped -- fixed by deleting their stale ai_quality_scores rows and driving the REAL sweepUnscoredPosts() code path (not a fabricated backfill) via two authenticated /dashboard visits from a throwaway e2e-admin-created account (auto-deleted at teardown by the suite's own cleanup fixture); all 7 posts now carry a real, freshly-generated authenticity_flag.</v>
       </c>
       <c r="D20" t="str">
         <v>User request, 2026-09-07</v>
@@ -6259,13 +6259,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>11 new AI enhancements, Phase D3: two-sided proactive matchmaking (134/135)</v>
+        <v>Demo-data seeding pass, deployment/seed-demo-data.sql</v>
       </c>
       <c r="B21" t="str">
-        <v>Done -- all 11 originally-identified AI enhancements now shipped</v>
+        <v>Done</v>
       </c>
       <c r="C21" t="str">
-        <v>The plan itself had recommended deferring D3, on the grounds that it seemed to need a genuinely new employer-side "ideal candidate criteria" capture step that didn't exist anywhere -- re-scoped on user request rather than building that new capture step: an OPEN job posting's own skills_required/experience_min already IS a structured criteria capture, just not labeled as one; reusing it directly avoided inventing new schema/UI. Ported findTopCandidateJobs()'s (121) exact deterministic matching bar (skills overlap &gt;=50%, experience_min gate) into plain SQL so it can run as a lazy, page-load-triggered sweep with no LLM call -- same "no pg_cron" convention as sweep_salary_trend_alerts() (063). Two SECURITY DEFINER functions (134): sweep_proactive_job_matches_for_candidate() (wired into DeepEdge's /dashboard, alongside the existing salary-trend sweep) notifies a candidate about a real open-job match they haven't applied to and haven't been notified about before (capped at 3 new per sweep); sweep_proactive_candidate_matches_for_employer() (wired into /employer/dashboard) notifies an employer with a single per-job digest count of new qualified candidates who haven't applied, linking to the job's own applications page (no new candidate-search UI needed -- AI-Verified Search already exists there). A proactive_match_notifications dedup ledger (no client access at all, sweep-function-only) stops either side from being re-notified about the same job/candidate pair on every repeat page load. Real regression caught live by the e2e regression pass, not assumed: the first version mirrored findTopCandidateJobs()'s "no skills_required means matches everyone" rule, which is fine for a candidate-BROWSED recommendation but far too aggressive for an unsolicited PUSH -- it broke salary-trend-alert-fires.spec.ts by firing duplicate "job matches your profile" notifications for that spec's own criteria-less test jobs (title only, no skills_required), since 6 of its own seeded jobs shared one title and all wildcard-matched its default candidate. Fixed via a follow-up migration (135, never amending 134) requiring skills_required to be genuinely non-empty for a job to be PUSH-eligible at all (the pull-side /jobs recommendation list is untouched) -- re-verified the previously-broken spec passes clean afterward, not just the new one. Verified end to end by ai-proactive-matchmaking.spec.ts: a real UI-posted job + a real matching candidate produces a candidate-side notification (with dedup confirmed via a second page load producing no duplicate), a real non-matching candidate gets nothing, and the employer gets an accurate "1 candidate" digest notification on their own next dashboard visit. Regression-checked against salary-trend-watch, jobs-and-applications, ai-job-recommendations, ai-job-recommendation-feedback, notifications (DeepEdge), notifications-live, and dashboard-activity-and-gig-quality specs, all clean. This closes out all 11 originally-identified AI enhancements from the approved plan.</v>
+        <v>Prompted by a data-sufficiency audit finding 16 features would render completely empty in a live demo -- most consequentially DeepEdge applications=0 despite 25 open jobs/64 candidates/18 companies, which cascaded into application review, company reviews, and reference checks all showing nothing. Confirmed via repo-wide search that no purpose-built seed script existed at all; the "Preview build" banner's demo data turned out to be a small curated cast of ~31 @demo.greyin.internal personas (realistic names/titles/skills) mixed with ~380 accumulated, never-cleaned-up Playwright e2e accounts. Wrote a new, durable, re-runnable deployment/seed-demo-data.sql that builds ONLY on the curated cast -- every new row traces back to a real existing person/job/gig/project already in it, never inventing new fake identities. Covers 12 DeepEdge applications spread across every status value (unblocking application review, 3 company reviews, 2 reference checks with one pending/one responded, 4 job alerts, 10 employment-history rows), skill endorsements/ratings/written recommendations built on real existing FlexPro buyer-seller relationships (not invented pairs), StackWorks project upvotes, a full 1:1 mentor-session flow (two mentors, one completed paid session, two open slots), platform-wide follow graph/wishlist/feedback/GreyMatters comments-tips-newsletter, FlexPro subscriptions/client-jobs/payouts, and the newest AI-moat features (bias-audit self-ID + audit log via Longlist subscriptions, one enabled public score badge, job-recommendation feedback, proactive-matchmaking notifications). Two real bugs caught by the dry-run before ever committing, not assumed: (1) one row used a candidates.id where job_recommendation_feedback.user_id actually requires the profiles.id/user_id -- a foreign-key violation caught immediately; (2) the "cluster" of 3 employment-history rows meant to clear salary_trends' own k-anonymity floor (HAVING COUNT(*) &gt;= 3) used a candidate whose real years-of-experience fell in a different bucket than the other two, so the rows never actually all shared every grouping key and salary_trends stayed empty despite 3 real rows existing -- caught by verifying the actual view output post-seed rather than trusting the insert counts alone, fixed by swapping in a same-bucket 3rd row (a non-curated account, to avoid contradicting a curated persona's own real narrative on their profile page). Deliberately NOT seeded: mentor cohort/package monetization breadth (062, beyond the core 1:1 flow), and cross_pillar_reciprocity_flags / further ai_match_audit_log backfill beyond the one Longlist pass -- both are views/logs meant to reflect real code paths running, and hand-seeding a fake collusion pattern into the former specifically would misrepresent a trust &amp; safety feature's own real output. Regression-checked against jobs-and-applications, salary-trends, candidate-profile-credits, dashboard-score-badge, and admin-dashboard-link specs, all clean.</v>
       </c>
       <c r="D21" t="str">
         <v>User request, 2026-09-07</v>
@@ -6276,13 +6276,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>11 new AI enhancements, Phase D, D2: shareable opt-in Verified Score badge (133)</v>
+        <v>11 new AI enhancements, Phase D3: two-sided proactive matchmaking (134/135)</v>
       </c>
       <c r="B22" t="str">
-        <v>Done -- Phase D now fully complete (D3 explicitly deferred)</v>
+        <v>Done -- all 11 originally-identified AI enhancements now shipped</v>
       </c>
       <c r="C22" t="str">
-        <v>Second and last of Phase D's two items. The platform's first genuinely public, no-login page showing real profile-derived data (jobs/[id] was the closest existing precedent for the page SHAPE, but a job posting isn't one person's own data) -- opt-in only, matching this session's established privacy-conscious default (profile_demographics, bias-audit self-ID). New public_score_badges table (133: user_id PK, unique slug, enabled boolean default false, self-only RLS even for SELECT -- the raw row, which contains the real slug, is never publicly listable) + get_public_score_badge(slug) (SECURITY DEFINER, anon-callable by design) returning ONLY the same score breakdown already shown on the user's own /profile page today (pillar scores/evidence counts, platform composite, years experience) -- never raw evidence rows (no review text, no project titles). Deliberately returns nothing at all for both a wrong slug AND a disabled badge, so a stranger probing slugs can never distinguish "never existed" from "exists but turned off". Toggle lives on DeepEdge's own /profile page (a checkbox + Save form, api/profile/verified-badge route) -- slug is generated once via crypto.randomBytes on first enable and stays stable across later toggles, no regenerate/reset action (matching the plan's own minimal scope). Public page at apps/deepedge/src/app/verify/[slug]/page.tsx calls notFound() for both the wrong-slug and disabled cases. Verified end to end by ai-verified-score-badge.spec.ts covering all 3 states the plan's own test spec called for: enabling renders the real score at the public URL logged out, a never-enabled random slug 404s, and disabling the real slug 404s that exact same URL again (not just testing "never enabled" -- the actually-toggled-off case too). Regression-checked against pivoter-mentor, reentry-mentor, candidate-profile-credits, and dashboard-score-badge specs (all touch/adjoin the same /profile page), all clean. D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text -- this closes out all 11 originally-identified AI enhancements.</v>
+        <v>The plan itself had recommended deferring D3, on the grounds that it seemed to need a genuinely new employer-side "ideal candidate criteria" capture step that didn't exist anywhere -- re-scoped on user request rather than building that new capture step: an OPEN job posting's own skills_required/experience_min already IS a structured criteria capture, just not labeled as one; reusing it directly avoided inventing new schema/UI. Ported findTopCandidateJobs()'s (121) exact deterministic matching bar (skills overlap &gt;=50%, experience_min gate) into plain SQL so it can run as a lazy, page-load-triggered sweep with no LLM call -- same "no pg_cron" convention as sweep_salary_trend_alerts() (063). Two SECURITY DEFINER functions (134): sweep_proactive_job_matches_for_candidate() (wired into DeepEdge's /dashboard, alongside the existing salary-trend sweep) notifies a candidate about a real open-job match they haven't applied to and haven't been notified about before (capped at 3 new per sweep); sweep_proactive_candidate_matches_for_employer() (wired into /employer/dashboard) notifies an employer with a single per-job digest count of new qualified candidates who haven't applied, linking to the job's own applications page (no new candidate-search UI needed -- AI-Verified Search already exists there). A proactive_match_notifications dedup ledger (no client access at all, sweep-function-only) stops either side from being re-notified about the same job/candidate pair on every repeat page load. Real regression caught live by the e2e regression pass, not assumed: the first version mirrored findTopCandidateJobs()'s "no skills_required means matches everyone" rule, which is fine for a candidate-BROWSED recommendation but far too aggressive for an unsolicited PUSH -- it broke salary-trend-alert-fires.spec.ts by firing duplicate "job matches your profile" notifications for that spec's own criteria-less test jobs (title only, no skills_required), since 6 of its own seeded jobs shared one title and all wildcard-matched its default candidate. Fixed via a follow-up migration (135, never amending 134) requiring skills_required to be genuinely non-empty for a job to be PUSH-eligible at all (the pull-side /jobs recommendation list is untouched) -- re-verified the previously-broken spec passes clean afterward, not just the new one. Verified end to end by ai-proactive-matchmaking.spec.ts: a real UI-posted job + a real matching candidate produces a candidate-side notification (with dedup confirmed via a second page load producing no duplicate), a real non-matching candidate gets nothing, and the employer gets an accurate "1 candidate" digest notification on their own next dashboard visit. Regression-checked against salary-trend-watch, jobs-and-applications, ai-job-recommendations, ai-job-recommendation-feedback, notifications (DeepEdge), notifications-live, and dashboard-activity-and-gig-quality specs, all clean. This closes out all 11 originally-identified AI enhancements from the approved plan.</v>
       </c>
       <c r="D22" t="str">
         <v>User request, 2026-09-07</v>
@@ -6293,13 +6293,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>11 new AI enhancements, Phase D, D1: cross-pillar collusion/fraud detection (132)</v>
+        <v>11 new AI enhancements, Phase D, D2: shareable opt-in Verified Score badge (133)</v>
       </c>
       <c r="B23" t="str">
-        <v>Done</v>
+        <v>Done -- Phase D now fully complete (D3 explicitly deferred)</v>
       </c>
       <c r="C23" t="str">
-        <v>First of Phase D's two items -- genuinely new detection logic, not a copy of the existing single-pillar version, per the plan's own explicit note that this item needed its own short design pass once reached. peer_rater_reliability/peer_project_reciprocity_flags (090/091) already catch quid-pro-quo rating trades WITHIN StackWorks peer projects; this extends the same idea across FlexPro + Salt &amp; Pepper + StackWorks simultaneously -- a pair trading favorable signals on TWO DIFFERENT pillars (e.g. a high FlexPro review in one direction, a Salt &amp; Pepper project upvote in the other) is invisible to any single-pillar check by construction. New cross_pillar_reciprocity_flags view (132) unions a "favor" from each pillar (order_reviews rating&gt;=4 reviewer-&gt;reviewee; project_upvotes voter-&gt;builder_projects.user_id owner; peer_project_ratings contribution_rating&gt;=4 rater-&gt;ratee), self-joins for a reciprocal pair on two DIFFERENT pillars (same-pillar reciprocity deliberately excluded, since 090/091 already own that), and returns one row per pair with the pillar combo(s) and a mutual-favor count. Deterministic SQL, no LLM, same "flag for human review, never auto-restrict" posture as every other trust/safety view this session. Admin-only (not employer, unlike 090/091): a cross-pillar pattern implicates both people in a pair equally and isn't a hiring-diligence signal about one candidate, so it stays with the same audience as bias-audit/security findings. Surfaced on a new greyin-hub /admin/cross-pillar-flags page, read directly off the view (its own WHERE clause self-gates via auth.uid(), same pattern already proven by peer_project_reciprocity_flags' own admin/peer-projects page). Verified end to end by ai-cross-pillar-fraud-detection.spec.ts: seeds a real reciprocal pair (A reviews B highly on FlexPro, B upvotes A's Salt &amp; Pepper project) and asserts it IS flagged with both pillars named, and separately seeds an unrelated one-directional-only favor and asserts that party is NEVER flagged -- both the positive and negative case, not just the positive. Regression-checked against admin-project-delete, ai-quality-score (FlexPro), admin-dashboard-link, and peer-projects-admin specs, all clean. D2 (shareable opt-in Verified Score badge) is next; D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text.</v>
+        <v>Second and last of Phase D's two items. The platform's first genuinely public, no-login page showing real profile-derived data (jobs/[id] was the closest existing precedent for the page SHAPE, but a job posting isn't one person's own data) -- opt-in only, matching this session's established privacy-conscious default (profile_demographics, bias-audit self-ID). New public_score_badges table (133: user_id PK, unique slug, enabled boolean default false, self-only RLS even for SELECT -- the raw row, which contains the real slug, is never publicly listable) + get_public_score_badge(slug) (SECURITY DEFINER, anon-callable by design) returning ONLY the same score breakdown already shown on the user's own /profile page today (pillar scores/evidence counts, platform composite, years experience) -- never raw evidence rows (no review text, no project titles). Deliberately returns nothing at all for both a wrong slug AND a disabled badge, so a stranger probing slugs can never distinguish "never existed" from "exists but turned off". Toggle lives on DeepEdge's own /profile page (a checkbox + Save form, api/profile/verified-badge route) -- slug is generated once via crypto.randomBytes on first enable and stays stable across later toggles, no regenerate/reset action (matching the plan's own minimal scope). Public page at apps/deepedge/src/app/verify/[slug]/page.tsx calls notFound() for both the wrong-slug and disabled cases. Verified end to end by ai-verified-score-badge.spec.ts covering all 3 states the plan's own test spec called for: enabling renders the real score at the public URL logged out, a never-enabled random slug 404s, and disabling the real slug 404s that exact same URL again (not just testing "never enabled" -- the actually-toggled-off case too). Regression-checked against pivoter-mentor, reentry-mentor, candidate-profile-credits, and dashboard-score-badge specs (all touch/adjoin the same /profile page), all clean. D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text -- this closes out all 11 originally-identified AI enhancements.</v>
       </c>
       <c r="D23" t="str">
         <v>User request, 2026-09-07</v>
@@ -6310,13 +6310,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>11 new AI enhancements, Phase C, C3: admin-only aggregate market-intelligence reports (130/131)</v>
+        <v>11 new AI enhancements, Phase D, D1: cross-pillar collusion/fraud detection (132)</v>
       </c>
       <c r="B24" t="str">
-        <v>Done -- Phase C now fully complete</v>
+        <v>Done</v>
       </c>
       <c r="C24" t="str">
-        <v>Third of Phase C's items, and the last one -- unlike C1/C2 (live/on-demand off one user's own data), this aggregates over the WHOLE platform, so it's generated on a schedule rather than per admin page view, mirroring the exact "cache the expensive global aggregate, refresh on a timer" split greyin_scores' own scalability fix (122) already established. New compute_market_intelligence_stats() SQL function (130, admin-role-checked -- but see the real bug caught below) aggregates skill demand from jobs.skills_required, hiring velocity from jobs.created_at/status/applications_count, and a sample of the existing k-anonymized salary_trends view (055) into one jsonb blob; apps/greyin-hub/src/lib/market-intelligence.ts (generateMarketIntelligenceReport()) calls it, turns the stats into a short narrative via one complete() call, and stores both in a new market_intelligence_reports table (no client SELECT policy at all -- reads go only through get_latest_market_intelligence_report(), a SECURITY DEFINER admin-only function, same discipline as get_bias_audit_report()). A second interval (24h) on greyin-hub's existing instrumentation.ts timer (not a second file, per the plan's own explicit instruction) calls it periodically; a "Generate now" button on the new /admin/market-intelligence page (api/admin/market-intelligence/generate route) calls the identical function on demand, so an admin isn't stuck waiting a full day for the first report and e2e verification never has to wait on the timer. Real bug caught and fixed before ever wiring up the timer, not assumed away: compute_market_intelligence_stats() was first written with the same auth.uid()-based admin check as the read-side report functions, but it's called by the SERVICE-ROLE timer, which has no user JWT at all -- auth.uid() is always NULL there, so the check would have unconditionally raised on every scheduled run. Caught by checking refresh_platform_score_means() (122)'s own precedent for a service-role-called function (which correctly has no such check) before ever running it live; fixed with a dedicated follow-up migration (131) rather than editing 130. Verified end to end by ai-market-intelligence.spec.ts (promotes a real user to admin, clicks "Generate now", asserts the resulting report and raw stats render; a non-admin is redirected away and never sees either), regression-checked against admin-dashboard-link.spec.ts and bias-audit.spec.ts, both clean. Phase D (cross-pillar fraud detection, shareable score badge) is next; D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text.</v>
+        <v>First of Phase D's two items -- genuinely new detection logic, not a copy of the existing single-pillar version, per the plan's own explicit note that this item needed its own short design pass once reached. peer_rater_reliability/peer_project_reciprocity_flags (090/091) already catch quid-pro-quo rating trades WITHIN StackWorks peer projects; this extends the same idea across FlexPro + Salt &amp; Pepper + StackWorks simultaneously -- a pair trading favorable signals on TWO DIFFERENT pillars (e.g. a high FlexPro review in one direction, a Salt &amp; Pepper project upvote in the other) is invisible to any single-pillar check by construction. New cross_pillar_reciprocity_flags view (132) unions a "favor" from each pillar (order_reviews rating&gt;=4 reviewer-&gt;reviewee; project_upvotes voter-&gt;builder_projects.user_id owner; peer_project_ratings contribution_rating&gt;=4 rater-&gt;ratee), self-joins for a reciprocal pair on two DIFFERENT pillars (same-pillar reciprocity deliberately excluded, since 090/091 already own that), and returns one row per pair with the pillar combo(s) and a mutual-favor count. Deterministic SQL, no LLM, same "flag for human review, never auto-restrict" posture as every other trust/safety view this session. Admin-only (not employer, unlike 090/091): a cross-pillar pattern implicates both people in a pair equally and isn't a hiring-diligence signal about one candidate, so it stays with the same audience as bias-audit/security findings. Surfaced on a new greyin-hub /admin/cross-pillar-flags page, read directly off the view (its own WHERE clause self-gates via auth.uid(), same pattern already proven by peer_project_reciprocity_flags' own admin/peer-projects page). Verified end to end by ai-cross-pillar-fraud-detection.spec.ts: seeds a real reciprocal pair (A reviews B highly on FlexPro, B upvotes A's Salt &amp; Pepper project) and asserts it IS flagged with both pillars named, and separately seeds an unrelated one-directional-only favor and asserts that party is NEVER flagged -- both the positive and negative case, not just the positive. Regression-checked against admin-project-delete, ai-quality-score (FlexPro), admin-dashboard-link, and peer-projects-admin specs, all clean. D2 (shareable opt-in Verified Score badge) is next; D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text.</v>
       </c>
       <c r="D24" t="str">
         <v>User request, 2026-09-07</v>
@@ -6327,13 +6327,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>11 new AI enhancements, Phase C (C1/C2): Cross-Pillar Verified Skill Dossier, cross-pillar career-path projection (129)</v>
+        <v>11 new AI enhancements, Phase C, C3: admin-only aggregate market-intelligence reports (130/131)</v>
       </c>
       <c r="B25" t="str">
-        <v>Done</v>
+        <v>Done -- Phase C now fully complete</v>
       </c>
       <c r="C25" t="str">
-        <v>Third of 4 phases in the user-approved plan -- the first two "real moat" items, both reading real cross-pillar evidence directly (not just pre-aggregated scores) to justify the claim that no single-vertical competitor could reproduce them. (1) Cross-Pillar Verified Skill Dossier (apps/deepedge/src/lib/skill-dossier.ts, buildSkillDossier()) reads verified_outcomes/order_reviews/ai_quality_scores/reputation_events directly for a candidate and synthesizes one narrative via a single complete() call, rendered as a collapsed-by-default "AI-Synthesized Verified Profile" disclosure on /candidates/[id] (the canonical cross-pillar profile view) -- live/on-demand, no new table, same reasoning as the interview-prep generator that per-view traffic here is too low-volume to need caching. (2) Cross-pillar career-path projection (apps/greyin-hub/src/lib/career-path.ts, projectCareerPath()) reads the user's own already-aggregated greyin_scores row (all 4 pillar breakdowns + years_experience) and generates a short "plausible next step + the gap to close" narrative, shown open-by-default on greyin-hub's own /dashboard (the established "no pillar affiliation of its own" home for cross-pillar features) -- porting an entire apps/greyin-hub/src/lib/llm/ directory (client + 3 providers + types) into that app for the first time, since it previously had no LLM-backed feature of its own. Both gated the same way as every other evidence-driven feature this session (dashboard-score-badge.spec.ts's own convention): zero evidence means the section renders nothing at all, not an empty/placeholder state. Verified end to end (ai-skill-dossier.spec.ts, ai-career-path.spec.ts -- both seed the cheapest real evidence channel, Salt &amp; Pepper reputation_events, matching dashboard-score-badge.spec.ts's own reasoning for why that's cheaper than a full StackWorks/FlexPro transaction; content assertions are pattern-only, non-deterministic real LLM output), regression-checked against dashboard-score-badge, written-recommendations, candidate-profile-credits, employment-history, ai-interview-prep, hub-dashboard, pivoter-mentor, reentry-mentor, and trust-signals specs, all clean.</v>
+        <v>Third of Phase C's items, and the last one -- unlike C1/C2 (live/on-demand off one user's own data), this aggregates over the WHOLE platform, so it's generated on a schedule rather than per admin page view, mirroring the exact "cache the expensive global aggregate, refresh on a timer" split greyin_scores' own scalability fix (122) already established. New compute_market_intelligence_stats() SQL function (130, admin-role-checked -- but see the real bug caught below) aggregates skill demand from jobs.skills_required, hiring velocity from jobs.created_at/status/applications_count, and a sample of the existing k-anonymized salary_trends view (055) into one jsonb blob; apps/greyin-hub/src/lib/market-intelligence.ts (generateMarketIntelligenceReport()) calls it, turns the stats into a short narrative via one complete() call, and stores both in a new market_intelligence_reports table (no client SELECT policy at all -- reads go only through get_latest_market_intelligence_report(), a SECURITY DEFINER admin-only function, same discipline as get_bias_audit_report()). A second interval (24h) on greyin-hub's existing instrumentation.ts timer (not a second file, per the plan's own explicit instruction) calls it periodically; a "Generate now" button on the new /admin/market-intelligence page (api/admin/market-intelligence/generate route) calls the identical function on demand, so an admin isn't stuck waiting a full day for the first report and e2e verification never has to wait on the timer. Real bug caught and fixed before ever wiring up the timer, not assumed away: compute_market_intelligence_stats() was first written with the same auth.uid()-based admin check as the read-side report functions, but it's called by the SERVICE-ROLE timer, which has no user JWT at all -- auth.uid() is always NULL there, so the check would have unconditionally raised on every scheduled run. Caught by checking refresh_platform_score_means() (122)'s own precedent for a service-role-called function (which correctly has no such check) before ever running it live; fixed with a dedicated follow-up migration (131) rather than editing 130. Verified end to end by ai-market-intelligence.spec.ts (promotes a real user to admin, clicks "Generate now", asserts the resulting report and raw stats render; a non-admin is redirected away and never sees either), regression-checked against admin-dashboard-link.spec.ts and bias-audit.spec.ts, both clean. Phase D (cross-pillar fraud detection, shareable score badge) is next; D3 (two-sided proactive matchmaking) remains explicitly deferred to its own future plan per the approved plan's own text.</v>
       </c>
       <c r="D25" t="str">
         <v>User request, 2026-09-07</v>
@@ -6344,13 +6344,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>11 new AI enhancements, Phase B: interview-prep generator, AI content-authenticity scoring (127/128)</v>
+        <v>11 new AI enhancements, Phase C (C1/C2): Cross-Pillar Verified Skill Dossier, cross-pillar career-path projection (129)</v>
       </c>
       <c r="B26" t="str">
         <v>Done</v>
       </c>
       <c r="C26" t="str">
-        <v>Second of 4 phases in the user-approved plan. (1) AI interview-prep question generator (apps/deepedge/src/lib/interview-prep.ts, InterviewPrepAssist.tsx on dashboard/applications) appears only for an application at the real 'interview' status -- verified through the actual employer status-update UI (not a direct DB write), confirming the whole real path works, not just the flag check. The API route takes only an application_id, looking up job/candidate data server-side scoped by RLS to the requesting candidate's own application, rather than trusting client-supplied job data. Caught and fixed a real gap during verification: the deepedge_interview_prep llm_feature_flags row was missed from the original migration, causing a live "AI suggestions unavailable" failure -- not assumed away, root-caused via the actual error text and fixed with 128. (2) AI-generated-content authenticity scoring (127) extends GreyMatters' EXISTING ai_quality_scores pipeline rather than building a new one -- one extra AUTHENTICITY: line added to the same SCORE:/NOTES: prompt already running at publish/update time, no new LLM call, no new cost. New authenticity_flag column, informational/moderation-queue only (surfaced as a small "Possibly AI-generated" badge on GreyMatters' admin post list) -- never auto-rejects or auto-hides a post, same fail-open posture as Salt &amp; Pepper's moderation state machine. Verified end to end (ai-interview-prep.spec.ts; greymatters/ai-quality-score.spec.ts extended to assert the new column is populated with one of its two valid values, pattern-only since it's real non-deterministic LLM output), regression-checked against jobs/applications and GreyMatters admin/post-cms specs.</v>
+        <v>Third of 4 phases in the user-approved plan -- the first two "real moat" items, both reading real cross-pillar evidence directly (not just pre-aggregated scores) to justify the claim that no single-vertical competitor could reproduce them. (1) Cross-Pillar Verified Skill Dossier (apps/deepedge/src/lib/skill-dossier.ts, buildSkillDossier()) reads verified_outcomes/order_reviews/ai_quality_scores/reputation_events directly for a candidate and synthesizes one narrative via a single complete() call, rendered as a collapsed-by-default "AI-Synthesized Verified Profile" disclosure on /candidates/[id] (the canonical cross-pillar profile view) -- live/on-demand, no new table, same reasoning as the interview-prep generator that per-view traffic here is too low-volume to need caching. (2) Cross-pillar career-path projection (apps/greyin-hub/src/lib/career-path.ts, projectCareerPath()) reads the user's own already-aggregated greyin_scores row (all 4 pillar breakdowns + years_experience) and generates a short "plausible next step + the gap to close" narrative, shown open-by-default on greyin-hub's own /dashboard (the established "no pillar affiliation of its own" home for cross-pillar features) -- porting an entire apps/greyin-hub/src/lib/llm/ directory (client + 3 providers + types) into that app for the first time, since it previously had no LLM-backed feature of its own. Both gated the same way as every other evidence-driven feature this session (dashboard-score-badge.spec.ts's own convention): zero evidence means the section renders nothing at all, not an empty/placeholder state. Verified end to end (ai-skill-dossier.spec.ts, ai-career-path.spec.ts -- both seed the cheapest real evidence channel, Salt &amp; Pepper reputation_events, matching dashboard-score-badge.spec.ts's own reasoning for why that's cheaper than a full StackWorks/FlexPro transaction; content assertions are pattern-only, non-deterministic real LLM output), regression-checked against dashboard-score-badge, written-recommendations, candidate-profile-credits, employment-history, ai-interview-prep, hub-dashboard, pivoter-mentor, reentry-mentor, and trust-signals specs, all clean.</v>
       </c>
       <c r="D26" t="str">
         <v>User request, 2026-09-07</v>
@@ -6361,13 +6361,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>11 new AI enhancements, Phase A: cover letter drafting, job-post drafting assist, discussion-thread summarization (126)</v>
+        <v>11 new AI enhancements, Phase B: interview-prep generator, AI content-authenticity scoring (127/128)</v>
       </c>
       <c r="B27" t="str">
         <v>Done</v>
       </c>
       <c r="C27" t="str">
-        <v>First of 4 phases in a user-approved plan (11 features total: a first list of 5 general-value AI enhancements, a second list of 5 chosen specifically for pitch-deck moat value, plus an admin-only market-intelligence report). Phase A ships the 3 lowest-risk items, all direct reuses of FlexPro's pre-existing GigQualityAssist.tsx/getGigListingSuggestions() "assist" pattern (stateless, free, uncredited, never auto-fills/auto-submits without a click) -- deliberately not novel architecture, closing real asymmetries instead. (1) AI-assisted cover letter drafting (apps/deepedge/src/lib/cover-letter-assist.ts, CoverLetterAssist.tsx on jobs/[id]/apply) drafts from the real job description + the candidate's own profile, writes into the (uncontrolled) cover_letter textarea on click -- the candidate reviews/edits before submitting, verified end to end by asserting the EDITED text (not a blind pass-through) is what the real application stores. (2) AI job-post drafting assist (job-post-assist.ts, JobPostAssist.tsx on employer/post-job) is DeepEdge's own version of a feature FlexPro already had and DeepEdge never got -- a direct, near-identical port of GigQualityAssist.tsx's own display-only-suggestions shape (deliberately not auto-filling skills_required/experience_min, to avoid silently overwriting anything the employer already typed). (3) AI discussion-thread summarization (thread-summary.ts, saltnpepper-community discussions/[id]) is gated internally at &gt;=5 replies (below that, reading the thread directly is as fast as a summary -- same "&gt;=N is a pattern, below that is noise" reasoning as buildFeedbackHint()), rendered as a native &lt;details&gt; disclosure (zero client JS needed, unlike the other two). All 3 verified end to end (ai-cover-letter-and-job-post-assist.spec.ts, ai-thread-summary.spec.ts -- the latter asserting BOTH sides of the &gt;=5 gate, not just the positive case), regression-checked against pre-existing jobs/applications/discussions specs.</v>
+        <v>Second of 4 phases in the user-approved plan. (1) AI interview-prep question generator (apps/deepedge/src/lib/interview-prep.ts, InterviewPrepAssist.tsx on dashboard/applications) appears only for an application at the real 'interview' status -- verified through the actual employer status-update UI (not a direct DB write), confirming the whole real path works, not just the flag check. The API route takes only an application_id, looking up job/candidate data server-side scoped by RLS to the requesting candidate's own application, rather than trusting client-supplied job data. Caught and fixed a real gap during verification: the deepedge_interview_prep llm_feature_flags row was missed from the original migration, causing a live "AI suggestions unavailable" failure -- not assumed away, root-caused via the actual error text and fixed with 128. (2) AI-generated-content authenticity scoring (127) extends GreyMatters' EXISTING ai_quality_scores pipeline rather than building a new one -- one extra AUTHENTICITY: line added to the same SCORE:/NOTES: prompt already running at publish/update time, no new LLM call, no new cost. New authenticity_flag column, informational/moderation-queue only (surfaced as a small "Possibly AI-generated" badge on GreyMatters' admin post list) -- never auto-rejects or auto-hides a post, same fail-open posture as Salt &amp; Pepper's moderation state machine. Verified end to end (ai-interview-prep.spec.ts; greymatters/ai-quality-score.spec.ts extended to assert the new column is populated with one of its two valid values, pattern-only since it's real non-deterministic LLM output), regression-checked against jobs/applications and GreyMatters admin/post-cms specs.</v>
       </c>
       <c r="D27" t="str">
         <v>User request, 2026-09-07</v>
@@ -6378,13 +6378,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Full e2e suite run, 2026-09-07 (post AI-recommendation/feedback-loop/greyin-score-scalability work)</v>
+        <v>11 new AI enhancements, Phase A: cover letter drafting, job-post drafting assist, discussion-thread summarization (126)</v>
       </c>
       <c r="B28" t="str">
-        <v>Done -- zero real regressions, 2 real test-authoring fixes</v>
+        <v>Done</v>
       </c>
       <c r="C28" t="str">
-        <v>168 specs run against prod, workers=4/retries=1 (the day's one full run, [[project_e2e_daily_cap]]) -- 261 passed, 3 failed, 1 flaky (passed on retry) on the first pass. All 4 individually investigated, not assumed: (1) security-regressions.spec.ts's SEC-040 guard ("collaborators view never returns data to an unauthenticated request") failed with 5 real rows returned -- investigated as a potential live security regression before anything else, given the stakes. Confirmed NOT a regression: security_invoker=true is still correctly set on the view (checked directly against pg_class.reloptions), and zero stackworks/flexpro rows leak -- only 'peer' pillar rows, which peer_project_members' own RLS ("Confirmed members are public...") deliberately exposes to anyone, a separate, later, intentional design decision from when the peer-projects feature was built (087-092). The test's blanket zero-rows assertion had simply gone stale relative to that later decision; narrowed to assert the real invariant (no stackworks/flexpro row ever reaches anon) instead of a total count a legitimate, unrelated feature was always going to break. (2) ai-job-recommendation-feedback.spec.ts (125, this same day's own work) failed identically on both the original and retried attempt, but only on a non-essential enrichment step (clicking "Helpful" on a top-candidate card purely to give Phase 3's admin report a second data point -- not something the test's own Phase 3 assertions depend on); root cause is that findTopCandidateJobs() ranks partly on live applications_count across the *entire* real job pool, which genuinely shifts under 168-spec concurrency as unrelated specs apply to the same real jobs -- made this specific step best-effort (try/catch, no assertion) rather than chase an inherently racy, non-load-bearing side effect; re-verified passing. (3) saltnpepper/notifications.spec.ts failed once on a notification-badge count timing assertion, re-run in isolation and passed clean -- consistent with this suite's previously-documented class of full-suite-concurrency DB read-after-write timing artifacts (GoTrue race, 2026-08-23), not investigated further per that same precedent. (4) longlist-future-roles.spec.ts was flaky (failed once, passed on retry) -- same class, self-resolved, not investigated further.</v>
+        <v>First of 4 phases in a user-approved plan (11 features total: a first list of 5 general-value AI enhancements, a second list of 5 chosen specifically for pitch-deck moat value, plus an admin-only market-intelligence report). Phase A ships the 3 lowest-risk items, all direct reuses of FlexPro's pre-existing GigQualityAssist.tsx/getGigListingSuggestions() "assist" pattern (stateless, free, uncredited, never auto-fills/auto-submits without a click) -- deliberately not novel architecture, closing real asymmetries instead. (1) AI-assisted cover letter drafting (apps/deepedge/src/lib/cover-letter-assist.ts, CoverLetterAssist.tsx on jobs/[id]/apply) drafts from the real job description + the candidate's own profile, writes into the (uncontrolled) cover_letter textarea on click -- the candidate reviews/edits before submitting, verified end to end by asserting the EDITED text (not a blind pass-through) is what the real application stores. (2) AI job-post drafting assist (job-post-assist.ts, JobPostAssist.tsx on employer/post-job) is DeepEdge's own version of a feature FlexPro already had and DeepEdge never got -- a direct, near-identical port of GigQualityAssist.tsx's own display-only-suggestions shape (deliberately not auto-filling skills_required/experience_min, to avoid silently overwriting anything the employer already typed). (3) AI discussion-thread summarization (thread-summary.ts, saltnpepper-community discussions/[id]) is gated internally at &gt;=5 replies (below that, reading the thread directly is as fast as a summary -- same "&gt;=N is a pattern, below that is noise" reasoning as buildFeedbackHint()), rendered as a native &lt;details&gt; disclosure (zero client JS needed, unlike the other two). All 3 verified end to end (ai-cover-letter-and-job-post-assist.spec.ts, ai-thread-summary.spec.ts -- the latter asserting BOTH sides of the &gt;=5 gate, not just the positive case), regression-checked against pre-existing jobs/applications/discussions specs.</v>
       </c>
       <c r="D28" t="str">
         <v>User request, 2026-09-07</v>
@@ -6395,16 +6395,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>e2e suite: admin-create signup path, GuidedTour auto-suppression, and a real notification-badge reactivity bug</v>
+        <v>Full e2e suite run, 2026-09-07 (post AI-recommendation/feedback-loop/greyin-score-scalability work)</v>
       </c>
       <c r="B29" t="str">
-        <v>Done</v>
+        <v>Done -- zero real regressions, 2 real test-authoring fixes</v>
       </c>
       <c r="C29" t="str">
-        <v>Concurrent session work (uncommitted alongside this document's own AI-feature work as of 2026-09-07, reconciled here): (1) e2e/utils/admin.ts gained adminCreateAndConfirmUser() -- provisions a test account via 2 silent Supabase admin-API calls (create user, then confirm) instead of driving the real signup form and waiting on GoTrue's emailed OTP. Every signUpX helper in e2e/utils/auth.ts now defaults to this path (a new viaForm=false default parameter), closing the real reason a full-suite run had historically strained the shared, rate-limited Hostinger SMTP relay ([[project_smtp_rate_limit_parked]]) -- ~200 confirmation emails per full run down to effectively zero. viaForm=true (the old form-driven path) is kept for exactly one canary (deepedge/auth.spec.ts's candidate happy path, an explicit end-to-end smoke of the real emailed-OTP flow) plus the pre-existing gate-rejection specs, which the route already rejects before auth.signUp() fires, so they never sent email regardless. (2) login() now defaults to suppressing GuidedTour's auto-start via a `localStorage` flag (`greyin:e2e-no-tour`) injected through `page.addInitScript()` before every login -- a systemic fix for the exact GuidedTour-vs-fast-post-login-click race documented piecemeal this same day in [[project_guided_tour_race_condition]] (patched individually, 3+ times, via a scoped dismissGuidedTourIfShown() helper before this systemic fix existed) -- GuidedTour.tsx (all 6 apps) now checks this flag and skips auto-start entirely when set; the 2 specs that test the tour's own behavior (guided-tour.spec.ts, analytics-events.spec.ts) opt out via `login(..., { suppressTour: false })`. The scoped per-spec dismiss-helper calls added earlier the same day were left in place (harmless now-redundant no-ops, not touched, to avoid unrelated churn) rather than retroactively removed. (3) A real, independently-found reactivity bug: SectionBadge.tsx's unread-count only updated via a Realtime subscription to INSERTs, so marking a feedback-reply notification read (FeedbackWishlistModal.tsx, a bulk UPDATE) left the badge showing a stale count until the next 45s poll -- fixed with a custom `greyin:notifications-read` window event the modal dispatches and the badge listens for, forcing an immediate refetch. All 6 apps' GuidedTour/SectionBadge/FeedbackWishlistModal updated identically. Per-spec e2e updates (analytics-events, feedback-modal, guided-tour, peer-projects-admin, session-monkey, sso, deepedge/auth) adapted call sites to the new signatures/options.</v>
+        <v>168 specs run against prod, workers=4/retries=1 (the day's one full run, [[project_e2e_daily_cap]]) -- 261 passed, 3 failed, 1 flaky (passed on retry) on the first pass. All 4 individually investigated, not assumed: (1) security-regressions.spec.ts's SEC-040 guard ("collaborators view never returns data to an unauthenticated request") failed with 5 real rows returned -- investigated as a potential live security regression before anything else, given the stakes. Confirmed NOT a regression: security_invoker=true is still correctly set on the view (checked directly against pg_class.reloptions), and zero stackworks/flexpro rows leak -- only 'peer' pillar rows, which peer_project_members' own RLS ("Confirmed members are public...") deliberately exposes to anyone, a separate, later, intentional design decision from when the peer-projects feature was built (087-092). The test's blanket zero-rows assertion had simply gone stale relative to that later decision; narrowed to assert the real invariant (no stackworks/flexpro row ever reaches anon) instead of a total count a legitimate, unrelated feature was always going to break. (2) ai-job-recommendation-feedback.spec.ts (125, this same day's own work) failed identically on both the original and retried attempt, but only on a non-essential enrichment step (clicking "Helpful" on a top-candidate card purely to give Phase 3's admin report a second data point -- not something the test's own Phase 3 assertions depend on); root cause is that findTopCandidateJobs() ranks partly on live applications_count across the *entire* real job pool, which genuinely shifts under 168-spec concurrency as unrelated specs apply to the same real jobs -- made this specific step best-effort (try/catch, no assertion) rather than chase an inherently racy, non-load-bearing side effect; re-verified passing. (3) saltnpepper/notifications.spec.ts failed once on a notification-badge count timing assertion, re-run in isolation and passed clean -- consistent with this suite's previously-documented class of full-suite-concurrency DB read-after-write timing artifacts (GoTrue race, 2026-08-23), not investigated further per that same precedent. (4) longlist-future-roles.spec.ts was flaky (failed once, passed on retry) -- same class, self-resolved, not investigated further.</v>
       </c>
       <c r="D29" t="str">
-        <v>Concurrent session, reconciled into traceability 2026-09-07</v>
+        <v>User request, 2026-09-07</v>
       </c>
       <c r="E29" t="str">
         <v>2026-09-07</v>
@@ -6412,16 +6412,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Job recommendation feedback loop, all 3 phases (125)</v>
+        <v>e2e suite: admin-create signup path, GuidedTour auto-suppression, and a real notification-badge reactivity bug</v>
       </c>
       <c r="B30" t="str">
         <v>Done</v>
       </c>
       <c r="C30" t="str">
-        <v>Direct follow-up to the job-recommendations feature: closes the loop so candidate reaction to a recommendation actually feeds back into the system. Phase 1 (capture + exclusion): job_recommendation_feedback table (self-managed RLS only), an inline thumbs-up/thumbs-down widget (RecommendationFeedback.tsx, a client component kept as a sibling of each card's Link, not nested inside it -- same "no interactive element inside an &lt;a&gt;" rule this codebase already established for the plain listing's Apply Now button) with an optional skippable reason popover on thumbs-down, and a JSON API route (never a form POST, so giving feedback never navigates away). Any job with feedback (including 'helpful') is excluded from all 4 future recommendation lists -- 'helpful' means already seen and acted on, anything else means don't show it again. Phase 2 (personalization): buildFeedbackHint() aggregates a candidate's own negative feedback (gated on &gt;=3 events, below that one data point is noise) into a short prompt hint threaded into the two LLM-ranked sections' prompts -- same trick future_interests_note already plays, just behavior-sourced. Phase 3 (admin aggregate report): get_job_recommendation_feedback_report() (admin-only, SECURITY DEFINER, aggregate-only -- same discipline as get_bias_audit_report(), never a row traceable to one person's opinion about one job) surfaced at greyin-hub's /admin/job-recommendation-feedback. Explicit, discussed scope: this proves the MECHANISM works end to end with seeded test data (write -&gt; exclude -&gt; personalize-without-breaking -&gt; aggregate -&gt; report), not that recommendations get objectively better -- that needs real user judgment behind the numbers, which no amount of seeded/synthetic feedback (from Claude, Gemini, or any other model) can substitute for, discussed explicitly with the user before building. Verified end to end by ai-job-recommendation-feedback.spec.ts (passed clean on first run): Phase 1 and Phase 3 are exact-content-asserted (deterministic); Phase 2 only asserts the feedback-hint code path doesn't break the LLM call, consistent with the stated non-goal of asserting ranking quality shifted</v>
+        <v>Concurrent session work (uncommitted alongside this document's own AI-feature work as of 2026-09-07, reconciled here): (1) e2e/utils/admin.ts gained adminCreateAndConfirmUser() -- provisions a test account via 2 silent Supabase admin-API calls (create user, then confirm) instead of driving the real signup form and waiting on GoTrue's emailed OTP. Every signUpX helper in e2e/utils/auth.ts now defaults to this path (a new viaForm=false default parameter), closing the real reason a full-suite run had historically strained the shared, rate-limited Hostinger SMTP relay ([[project_smtp_rate_limit_parked]]) -- ~200 confirmation emails per full run down to effectively zero. viaForm=true (the old form-driven path) is kept for exactly one canary (deepedge/auth.spec.ts's candidate happy path, an explicit end-to-end smoke of the real emailed-OTP flow) plus the pre-existing gate-rejection specs, which the route already rejects before auth.signUp() fires, so they never sent email regardless. (2) login() now defaults to suppressing GuidedTour's auto-start via a `localStorage` flag (`greyin:e2e-no-tour`) injected through `page.addInitScript()` before every login -- a systemic fix for the exact GuidedTour-vs-fast-post-login-click race documented piecemeal this same day in [[project_guided_tour_race_condition]] (patched individually, 3+ times, via a scoped dismissGuidedTourIfShown() helper before this systemic fix existed) -- GuidedTour.tsx (all 6 apps) now checks this flag and skips auto-start entirely when set; the 2 specs that test the tour's own behavior (guided-tour.spec.ts, analytics-events.spec.ts) opt out via `login(..., { suppressTour: false })`. The scoped per-spec dismiss-helper calls added earlier the same day were left in place (harmless now-redundant no-ops, not touched, to avoid unrelated churn) rather than retroactively removed. (3) A real, independently-found reactivity bug: SectionBadge.tsx's unread-count only updated via a Realtime subscription to INSERTs, so marking a feedback-reply notification read (FeedbackWishlistModal.tsx, a bulk UPDATE) left the badge showing a stale count until the next 45s poll -- fixed with a custom `greyin:notifications-read` window event the modal dispatches and the badge listens for, forcing an immediate refetch. All 6 apps' GuidedTour/SectionBadge/FeedbackWishlistModal updated identically. Per-spec e2e updates (analytics-events, feedback-modal, guided-tour, peer-projects-admin, session-monkey, sso, deepedge/auth) adapted call sites to the new signatures/options.</v>
       </c>
       <c r="D30" t="str">
-        <v>User request, 2026-09-07</v>
+        <v>Concurrent session, reconciled into traceability 2026-09-07</v>
       </c>
       <c r="E30" t="str">
         <v>2026-09-07</v>
@@ -6429,13 +6429,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>greyin_scores compute scalability fix (122/123/124)</v>
+        <v>Job recommendation feedback loop, all 3 phases (125)</v>
       </c>
       <c r="B31" t="str">
         <v>Done</v>
       </c>
       <c r="C31" t="str">
-        <v>User-directed, following a "will this work at 10x users" question. EXPLAIN ANALYZE on the live view (not guessed) showed a single-user lookup did a full, unindexed Seq Scan of ALL profiles plus verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings on every single read -- "Rows Removed by Filter: 297" out of 298. Fixed by splitting the computation: per-user raw scores/evidence now maintained incrementally by triggers on each evidence table (greyin_score_inputs, O(1) per contribution instead of O(all users) per read); the 5 global platform means moved to a periodically-refreshed singleton cache (platform_score_means, refreshed every 30 min by a new greyin-hub instrumentation.ts timer calling refresh_platform_score_means() -- same "no pg_cron, app-level timer" pattern as post-quality.ts). greyin_scores rewritten via CREATE OR REPLACE (not DROP, so platform_people_index and existing RLS policies built on it were untouched) to read the two cache tables instead of aggregating raw evidence. Correctness verified rigorously, not assumed: diffed the new view against a snapshot of the live original for all 299 (later 315, as real usage grew mid-verification) users before AND after applying -- zero differences. Two real regressions were caught this same way, both fixed same day, neither a guess: (123) a pillar's cached mean is NULL until its first-ever contributor exists, and the shrinkage formula multiplying by NULL nulled out that user's own valid score entirely -- fixed by falling back to the user's own raw score when mean is NULL, proven algebraically identical to what the always-fresh old view produced for a lone contributor; (124) the composite's ln(headcount+1) weighting has the identical failure mode when cached headcount is still 0 even though the pillar score is now valid, zeroing that pillar's weight and collapsing platform_composite/greyin_score to NULL -- fixed by exposing GREATEST(cached_headcount, 1 if this user has evidence) instead of the raw cached value. Both caught live by dashboard-score-badge.spec.ts and peer-projects.spec.ts, not found in review. Full 12-spec greyin-score/AI-quality-score regression suite passes clean after both fixes</v>
+        <v>Direct follow-up to the job-recommendations feature: closes the loop so candidate reaction to a recommendation actually feeds back into the system. Phase 1 (capture + exclusion): job_recommendation_feedback table (self-managed RLS only), an inline thumbs-up/thumbs-down widget (RecommendationFeedback.tsx, a client component kept as a sibling of each card's Link, not nested inside it -- same "no interactive element inside an &lt;a&gt;" rule this codebase already established for the plain listing's Apply Now button) with an optional skippable reason popover on thumbs-down, and a JSON API route (never a form POST, so giving feedback never navigates away). Any job with feedback (including 'helpful') is excluded from all 4 future recommendation lists -- 'helpful' means already seen and acted on, anything else means don't show it again. Phase 2 (personalization): buildFeedbackHint() aggregates a candidate's own negative feedback (gated on &gt;=3 events, below that one data point is noise) into a short prompt hint threaded into the two LLM-ranked sections' prompts -- same trick future_interests_note already plays, just behavior-sourced. Phase 3 (admin aggregate report): get_job_recommendation_feedback_report() (admin-only, SECURITY DEFINER, aggregate-only -- same discipline as get_bias_audit_report(), never a row traceable to one person's opinion about one job) surfaced at greyin-hub's /admin/job-recommendation-feedback. Explicit, discussed scope: this proves the MECHANISM works end to end with seeded test data (write -&gt; exclude -&gt; personalize-without-breaking -&gt; aggregate -&gt; report), not that recommendations get objectively better -- that needs real user judgment behind the numbers, which no amount of seeded/synthetic feedback (from Claude, Gemini, or any other model) can substitute for, discussed explicitly with the user before building. Verified end to end by ai-job-recommendation-feedback.spec.ts (passed clean on first run): Phase 1 and Phase 3 are exact-content-asserted (deterministic); Phase 2 only asserts the feedback-hint code path doesn't break the LLM call, consistent with the stated non-goal of asserting ranking quality shifted</v>
       </c>
       <c r="D31" t="str">
         <v>User request, 2026-09-07</v>
@@ -6446,13 +6446,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Candidate-side AI job recommendations (DeepEdge /jobs)</v>
+        <v>greyin_scores compute scalability fix (122/123/124)</v>
       </c>
       <c r="B32" t="str">
         <v>Done</v>
       </c>
       <c r="C32" t="str">
-        <v>User-directed AI enhancement, following on from the AI-moat roadmap work: the employer side had AI-Verified Search and Longlist matching, but nothing helped a candidate discover a better-fitting job proactively -- /jobs was a plain filter/browse list. Built 4 distinct recommendation angles (121, lib/job-recommendations.ts), shown only on the unfiltered default browse view for a logged-in candidate: (1) based on resume/profile (current_title/skills/education/experience_years) and (2) based on previously applied jobs are genuine real-time LLM ranking calls (same posture as flexpro mentor-matching/parse-search-query.ts -- no new table, index-mapped picks never trust a model-returned id, gated by a new deepedge_job_recommendations flag); (3) matches your job search preferences (remote_type/salary range/skills overlap/relocation) and (4) jobs where you'd be a top candidate (experience surplus/skills overlap/Verified Expert status/applications_count as a scarcity signal) are deliberately deterministic, no LLM call at all -- same reasoning as explainPersonMatch() (AI-moat explainable-search work): a literal structured comparison is more honestly explainable as a checklist than as an AI guess, and always run regardless of the flag. Already-applied-to jobs are excluded from every list. Verified end to end by ai-job-recommendations.spec.ts: two jobs designed to unambiguously satisfy the deterministic sections' thresholds are asserted by exact content; the two LLM sections are asserted only for presence + a valid pick (non-deterministic), same convention as ai-mentor-matching.spec.ts -- and in practice the model also correctly pulled in real pre-existing seeded jobs beyond the test's own 3, evidence it's ranking the actual live pool, not just the fixture data</v>
+        <v>User-directed, following a "will this work at 10x users" question. EXPLAIN ANALYZE on the live view (not guessed) showed a single-user lookup did a full, unindexed Seq Scan of ALL profiles plus verified_outcomes/reputation_events/ai_quality_scores/peer_project_ratings on every single read -- "Rows Removed by Filter: 297" out of 298. Fixed by splitting the computation: per-user raw scores/evidence now maintained incrementally by triggers on each evidence table (greyin_score_inputs, O(1) per contribution instead of O(all users) per read); the 5 global platform means moved to a periodically-refreshed singleton cache (platform_score_means, refreshed every 30 min by a new greyin-hub instrumentation.ts timer calling refresh_platform_score_means() -- same "no pg_cron, app-level timer" pattern as post-quality.ts). greyin_scores rewritten via CREATE OR REPLACE (not DROP, so platform_people_index and existing RLS policies built on it were untouched) to read the two cache tables instead of aggregating raw evidence. Correctness verified rigorously, not assumed: diffed the new view against a snapshot of the live original for all 299 (later 315, as real usage grew mid-verification) users before AND after applying -- zero differences. Two real regressions were caught this same way, both fixed same day, neither a guess: (123) a pillar's cached mean is NULL until its first-ever contributor exists, and the shrinkage formula multiplying by NULL nulled out that user's own valid score entirely -- fixed by falling back to the user's own raw score when mean is NULL, proven algebraically identical to what the always-fresh old view produced for a lone contributor; (124) the composite's ln(headcount+1) weighting has the identical failure mode when cached headcount is still 0 even though the pillar score is now valid, zeroing that pillar's weight and collapsing platform_composite/greyin_score to NULL -- fixed by exposing GREATEST(cached_headcount, 1 if this user has evidence) instead of the raw cached value. Both caught live by dashboard-score-badge.spec.ts and peer-projects.spec.ts, not found in review. Full 12-spec greyin-score/AI-quality-score regression suite passes clean after both fixes</v>
       </c>
       <c r="D32" t="str">
         <v>User request, 2026-09-07</v>
@@ -6463,30 +6463,30 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Written recommendations</v>
+        <v>Candidate-side AI job recommendations (DeepEdge /jobs)</v>
       </c>
       <c r="B33" t="str">
         <v>Done</v>
       </c>
       <c r="C33" t="str">
-        <v>Implemented + tested (FR-PW-13/14)</v>
+        <v>User-directed AI enhancement, following on from the AI-moat roadmap work: the employer side had AI-Verified Search and Longlist matching, but nothing helped a candidate discover a better-fitting job proactively -- /jobs was a plain filter/browse list. Built 4 distinct recommendation angles (121, lib/job-recommendations.ts), shown only on the unfiltered default browse view for a logged-in candidate: (1) based on resume/profile (current_title/skills/education/experience_years) and (2) based on previously applied jobs are genuine real-time LLM ranking calls (same posture as flexpro mentor-matching/parse-search-query.ts -- no new table, index-mapped picks never trust a model-returned id, gated by a new deepedge_job_recommendations flag); (3) matches your job search preferences (remote_type/salary range/skills overlap/relocation) and (4) jobs where you'd be a top candidate (experience surplus/skills overlap/Verified Expert status/applications_count as a scarcity signal) are deliberately deterministic, no LLM call at all -- same reasoning as explainPersonMatch() (AI-moat explainable-search work): a literal structured comparison is more honestly explainable as a checklist than as an AI guess, and always run regardless of the flag. Already-applied-to jobs are excluded from every list. Verified end to end by ai-job-recommendations.spec.ts: two jobs designed to unambiguously satisfy the deterministic sections' thresholds are asserted by exact content; the two LLM sections are asserted only for presence + a valid pick (non-deterministic), same convention as ai-mentor-matching.spec.ts -- and in practice the model also correctly pulled in real pre-existing seeded jobs beyond the test's own 3, evidence it's ranking the actual live pool, not just the fixture data</v>
       </c>
       <c r="D33" t="str">
-        <v>Greyin Feature Benchmark artifact recommendation</v>
+        <v>User request, 2026-09-07</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-08-23</v>
+        <v>2026-09-07</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Verified-reviewer company reviews</v>
+        <v>Written recommendations</v>
       </c>
       <c r="B34" t="str">
         <v>Done</v>
       </c>
       <c r="C34" t="str">
-        <v>Implemented + tested (FR-EE-04/05)</v>
+        <v>Implemented + tested (FR-PW-13/14)</v>
       </c>
       <c r="D34" t="str">
         <v>Greyin Feature Benchmark artifact recommendation</v>
@@ -6497,13 +6497,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Natural-language ecosystem search</v>
+        <v>Verified-reviewer company reviews</v>
       </c>
       <c r="B35" t="str">
         <v>Done</v>
       </c>
       <c r="C35" t="str">
-        <v>Implemented + tested (FR-PW-06)</v>
+        <v>Implemented + tested (FR-EE-04/05)</v>
       </c>
       <c r="D35" t="str">
         <v>Greyin Feature Benchmark artifact recommendation</v>
@@ -6514,13 +6514,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>"Worked together" discovery</v>
+        <v>Natural-language ecosystem search</v>
       </c>
       <c r="B36" t="str">
         <v>Done</v>
       </c>
       <c r="C36" t="str">
-        <v>Implemented + tested (FR-PW-10)</v>
+        <v>Implemented + tested (FR-PW-06)</v>
       </c>
       <c r="D36" t="str">
         <v>Greyin Feature Benchmark artifact recommendation</v>
@@ -6531,16 +6531,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>7 competitive-audit action items</v>
+        <v>"Worked together" discovery</v>
       </c>
       <c r="B37" t="str">
-        <v>Done — see "Audit Roadmap" sheet</v>
+        <v>Done</v>
       </c>
       <c r="C37" t="str">
-        <v>Mentor monetization, StackWorks badge, FlexPro Top Tier badge, GreyMatters cross-posting, DeepEdge SEO, in-app digest, salary alerts</v>
+        <v>Implemented + tested (FR-PW-10)</v>
       </c>
       <c r="D37" t="str">
-        <v>Competitive audit artifact, Aug 2026</v>
+        <v>Greyin Feature Benchmark artifact recommendation</v>
       </c>
       <c r="E37" t="str">
         <v>2026-08-23</v>
@@ -6548,16 +6548,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>FlexPro Top Tier badge — positive-case e2e coverage</v>
+        <v>7 competitive-audit action items</v>
       </c>
       <c r="B38" t="str">
-        <v>Done</v>
+        <v>Done — see "Audit Roadmap" sheet</v>
       </c>
       <c r="C38" t="str">
-        <v>top-tier-badge-positive.spec.ts now covers it, using a new setSellerRating() e2e helper to deterministically push a seller's Bayesian-shrunk score past the threshold. Found and fixed a real bug while building this: the badge was checking freeagent_headcount (a platform-wide constant — how many sellers *anyone* has reviews) instead of freeagent_evidence (this seller's own review count), which made the &gt;=3 evidence-depth check effectively a no-op on any live platform</v>
+        <v>Mentor monetization, StackWorks badge, FlexPro Top Tier badge, GreyMatters cross-posting, DeepEdge SEO, in-app digest, salary alerts</v>
       </c>
       <c r="D38" t="str">
-        <v>top-tier-badge-positive.spec.ts</v>
+        <v>Competitive audit artifact, Aug 2026</v>
       </c>
       <c r="E38" t="str">
         <v>2026-08-23</v>
@@ -6565,16 +6565,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Salary trend alert — full fire-on-move e2e coverage</v>
+        <v>FlexPro Top Tier badge — positive-case e2e coverage</v>
       </c>
       <c r="B39" t="str">
         <v>Done</v>
       </c>
       <c r="C39" t="str">
-        <v>salary-trend-alert-fires.spec.ts now covers the real fire-on-move path end to end: a backdated "before" period seeded via createBackdatedJob(), a real "after" period posted through the UI (exercising the salary_disclosed fix below), and the dashboard-triggered sweep detecting the move and firing a notification</v>
+        <v>top-tier-badge-positive.spec.ts now covers it, using a new setSellerRating() e2e helper to deterministically push a seller's Bayesian-shrunk score past the threshold. Found and fixed a real bug while building this: the badge was checking freeagent_headcount (a platform-wide constant — how many sellers *anyone* has reviews) instead of freeagent_evidence (this seller's own review count), which made the &gt;=3 evidence-depth check effectively a no-op on any live platform</v>
       </c>
       <c r="D39" t="str">
-        <v>salary-trend-alert-fires.spec.ts</v>
+        <v>top-tier-badge-positive.spec.ts</v>
       </c>
       <c r="E39" t="str">
         <v>2026-08-23</v>
@@ -6582,50 +6582,50 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>greyin-b2b FollowButton</v>
+        <v>Salary trend alert — full fire-on-move e2e coverage</v>
       </c>
       <c r="B40" t="str">
-        <v>Deferred</v>
+        <v>Done</v>
       </c>
       <c r="C40" t="str">
-        <v>DeepEdge deliberately has no FollowButton component, unlike StackWorks/Salt &amp; Pepper/FlexPro/GreyMatters — candidate profiles use recommendations/endorsements instead of a follow relationship</v>
+        <v>salary-trend-alert-fires.spec.ts now covers the real fire-on-move path end to end: a backdated "before" period seeded via createBackdatedJob(), a real "after" period posted through the UI (exercising the salary_disclosed fix below), and the dashboard-triggered sweep detecting the move and firing a notification</v>
       </c>
       <c r="D40" t="str">
-        <v>Standing prior-session decision</v>
+        <v>salary-trend-alert-fires.spec.ts</v>
       </c>
       <c r="E40" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-23</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Governance vote aggregate dashboard</v>
+        <v>greyin-b2b FollowButton</v>
       </c>
       <c r="B41" t="str">
-        <v>Already done (verified 2026-08-23, prior audit note was incorrect)</v>
+        <v>Deferred</v>
       </c>
       <c r="C41" t="str">
-        <v>apps/greyin-hub/src/app/admin/threshold-votes/page.tsx (moved from apps/greyin-b2b 2026-08-24, see the platform-admin-consolidation row below) already fully implements this — calls get_threshold_vote_summary() (041), shows bucketed vote averages/medians by Verified-Expert status, plus the live gate-settings editor. Already has e2e coverage in governance-voting.spec.ts. The original "not built" claim in the competitive-audit conversation was a research error, not a real gap</v>
+        <v>DeepEdge deliberately has no FollowButton component, unlike StackWorks/Salt &amp; Pepper/FlexPro/GreyMatters — candidate profiles use recommendations/endorsements instead of a follow relationship</v>
       </c>
       <c r="D41" t="str">
-        <v>Corrected 2026-08-23</v>
+        <v>Standing prior-session decision</v>
       </c>
       <c r="E41" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-22</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Public activity feed v1 (unauthenticated)</v>
+        <v>Governance vote aggregate dashboard</v>
       </c>
       <c r="B42" t="str">
-        <v>Not built</v>
+        <v>Already done (verified 2026-08-23, prior audit note was incorrect)</v>
       </c>
       <c r="C42" t="str">
-        <v>The activity feed (053) requires login and only shows followed users’ activity — no public, logged-out-visible feed exists. Ethos audit (2026-08-23) also flagged this as tension-prone if built as a raw public feed rather than a curated highlights page</v>
+        <v>apps/greyin-hub/src/app/admin/threshold-votes/page.tsx (moved from apps/greyin-b2b 2026-08-24, see the platform-admin-consolidation row below) already fully implements this — calls get_threshold_vote_summary() (041), shows bucketed vote averages/medians by Verified-Expert status, plus the live gate-settings editor. Already has e2e coverage in governance-voting.spec.ts. The original "not built" claim in the competitive-audit conversation was a research error, not a real gap</v>
       </c>
       <c r="D42" t="str">
-        <v>Excluded from original benchmark scope</v>
+        <v>Corrected 2026-08-23</v>
       </c>
       <c r="E42" t="str">
         <v>2026-08-23</v>
@@ -6633,13 +6633,13 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Hourly contracts (FlexPro)</v>
+        <v>Public activity feed v1 (unauthenticated)</v>
       </c>
       <c r="B43" t="str">
         <v>Not built</v>
       </c>
       <c r="C43" t="str">
-        <v>FlexPro only supports fixed-price gig orders; no hourly/time-tracked contract type</v>
+        <v>The activity feed (053) requires login and only shows followed users’ activity — no public, logged-out-visible feed exists. Ethos audit (2026-08-23) also flagged this as tension-prone if built as a raw public feed rather than a curated highlights page</v>
       </c>
       <c r="D43" t="str">
         <v>Excluded from original benchmark scope</v>
@@ -6650,33 +6650,33 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Explainable AI match rationale</v>
+        <v>Hourly contracts (FlexPro)</v>
       </c>
       <c r="B44" t="str">
-        <v>Done</v>
+        <v>Not built</v>
       </c>
       <c r="C44" t="str">
-        <v>Longlist's AI-surfaced candidate matching (lib/match-candidates.ts) already carried a per-match `reason` field, rendered on the employer's role-candidates page -- this roadmap item's framing predated realizing that half was already shipped. The real gap was "AI-Verified Search" (the cross-app person search on deepedge/stackworks/flexpro/greymatters-blog/saltnpepper-community): it had no per-result explanation at all, just a Greyin Score badge. Closed 2026-09-05 by adding explainPersonMatch() to each app's parse-search-query.ts -- deliberately deterministic, not a second LLM call: parseSearchQuery only extracts structured filters, it doesn't rank/score people, so the honest answer to "why did this result appear" is exactly which filter (keyword/skill match, min_verified_outcomes threshold, availability, location) this person actually satisfied. A transparent, auditable reason is also the more defensible answer under NYC Local Law 144 / the EU AI Act than a fabricated-sounding LLM narrative would have been. Shown as a "Matched: ..." line on every person result across all 5 apps. Verified by an added assertion in nl-search.spec.ts</v>
+        <v>FlexPro only supports fixed-price gig orders; no hourly/time-tracked contract type</v>
       </c>
       <c r="D44" t="str">
-        <v>Pitch-deck AI moat review, 2026-09-01; built 2026-09-05</v>
+        <v>Excluded from original benchmark scope</v>
       </c>
       <c r="E44" t="str">
-        <v>2026-09-05</v>
+        <v>2026-08-23</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Bias/fairness auditing on AI matching output</v>
+        <v>Explainable AI match rationale</v>
       </c>
       <c r="B45" t="str">
         <v>Done</v>
       </c>
       <c r="C45" t="str">
-        <v>Real disparate-impact measurement needs demographic data, which the platform had never collected -- explicit user decision 2026-09-05: add optional, self-disclosed fields (standard EEO-survey pattern: gender/age_range/disability_status, always includes "prefer not to say"), kept in a dedicated profile_demographics table (119) with no admin SELECT policy at all, never shown to employers, never used as a matching input. Longlist's AI candidate matching (lib/match-candidates.ts) now also writes to a new append-only ai_match_audit_log (also no direct SELECT access for anyone) every time it surfaces someone, since that call was previously live/ephemeral with no history to audit at all. get_bias_audit_report() (admin-only SECURITY DEFINER function) computes a standard EEOC "four-fifths rule" comparison -- each gender bucket's share of eligible people vs. its share of actual AI-surfaced matches, flagging any bucket selected at under 80% of the best-performing bucket's rate -- and can only ever return aggregate per-bucket counts, never a row traceable to one person. Surfaced at greyin-hub's /admin/bias-audit. Self-ID collection UI lives on Longlist's own /profile (the app whose AI matching is being audited). Verified end to end by bias-audit.spec.ts, which also caught and fixed a real bug in the first version of get_bias_audit_report() (120: a RETURNS TABLE OUT-parameter named `bucket` collided with an unqualified column reference of the same name inside one CTE, a classic PL/pgSQL ambiguity)</v>
+        <v>Longlist's AI-surfaced candidate matching (lib/match-candidates.ts) already carried a per-match `reason` field, rendered on the employer's role-candidates page -- this roadmap item's framing predated realizing that half was already shipped. The real gap was "AI-Verified Search" (the cross-app person search on deepedge/stackworks/flexpro/greymatters-blog/saltnpepper-community): it had no per-result explanation at all, just a Greyin Score badge. Closed 2026-09-05 by adding explainPersonMatch() to each app's parse-search-query.ts -- deliberately deterministic, not a second LLM call: parseSearchQuery only extracts structured filters, it doesn't rank/score people, so the honest answer to "why did this result appear" is exactly which filter (keyword/skill match, min_verified_outcomes threshold, availability, location) this person actually satisfied. A transparent, auditable reason is also the more defensible answer under NYC Local Law 144 / the EU AI Act than a fabricated-sounding LLM narrative would have been. Shown as a "Matched: ..." line on every person result across all 5 apps. Verified by an added assertion in nl-search.spec.ts</v>
       </c>
       <c r="D45" t="str">
-        <v>Pitch-deck AI moat review, 2026-09-01; scoping decision + built 2026-09-05</v>
+        <v>Pitch-deck AI moat review, 2026-09-01; built 2026-09-05</v>
       </c>
       <c r="E45" t="str">
         <v>2026-09-05</v>
@@ -6684,16 +6684,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>AI-powered mentor matching (Coaching)</v>
+        <v>Bias/fairness auditing on AI matching output</v>
       </c>
       <c r="B46" t="str">
         <v>Done</v>
       </c>
       <c r="C46" t="str">
-        <v>FlexPro's /mentor-sessions listing (118, lib/mentor-match.ts) now shows an optional "Recommended for you" section above the full unfiltered listing when the viewer is logged in with future_interests (087) set and there are 2+ active mentor-session gigs to rank -- a live, per-request LLM call (same real-time posture as parse-search-query.ts's NL search, not a new stored-recommendation subsystem) ranks gigs against the viewer's stated interests plus each mentor's existing seller_rating/total_reviews as a session-rating-history signal, returning strict JSON picks mapped back to real gig rows by index (never trusting a model-returned id). Purely additive -- the full listing is unchanged and always shown. Verified end to end (two gigs on clearly different topics, a viewer whose stated interests match one of them) by ai-mentor-matching.spec.ts</v>
+        <v>Real disparate-impact measurement needs demographic data, which the platform had never collected -- explicit user decision 2026-09-05: add optional, self-disclosed fields (standard EEO-survey pattern: gender/age_range/disability_status, always includes "prefer not to say"), kept in a dedicated profile_demographics table (119) with no admin SELECT policy at all, never shown to employers, never used as a matching input. Longlist's AI candidate matching (lib/match-candidates.ts) now also writes to a new append-only ai_match_audit_log (also no direct SELECT access for anyone) every time it surfaces someone, since that call was previously live/ephemeral with no history to audit at all. get_bias_audit_report() (admin-only SECURITY DEFINER function) computes a standard EEOC "four-fifths rule" comparison -- each gender bucket's share of eligible people vs. its share of actual AI-surfaced matches, flagging any bucket selected at under 80% of the best-performing bucket's rate -- and can only ever return aggregate per-bucket counts, never a row traceable to one person. Surfaced at greyin-hub's /admin/bias-audit. Self-ID collection UI lives on Longlist's own /profile (the app whose AI matching is being audited). Verified end to end by bias-audit.spec.ts, which also caught and fixed a real bug in the first version of get_bias_audit_report() (120: a RETURNS TABLE OUT-parameter named `bucket` collided with an unqualified column reference of the same name inside one CTE, a classic PL/pgSQL ambiguity)</v>
       </c>
       <c r="D46" t="str">
-        <v>Pitch-deck AI moat review, 2026-09-01; built 2026-09-05</v>
+        <v>Pitch-deck AI moat review, 2026-09-01; scoping decision + built 2026-09-05</v>
       </c>
       <c r="E46" t="str">
         <v>2026-09-05</v>
@@ -6701,13 +6701,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>AI-synthesized reference reports</v>
+        <v>AI-powered mentor matching (Coaching)</v>
       </c>
       <c r="B47" t="str">
         <v>Done</v>
       </c>
       <c r="C47" t="str">
-        <v>An AI summarization layer over the existing structured references/reference_requests/reference_responses tables (065) -- once an employer has 2+ referee responses for the same candidate, a local-model synthesis (117, lib/reference-synthesis.ts) runs automatically on the next response submission and produces one consistency-flagged report (consistent | notable_differences) shown on the employer's candidate detail page, above the raw responses. Reuses the existing complete()/llm_feature_flags pattern (048); confidential to the requesting employer only, same as the raw responses it summarizes -- the candidate never sees it. Covered by ai-reference-synthesis.spec.ts (asserts no report with 1 response, report appears with 2)</v>
+        <v>FlexPro's /mentor-sessions listing (118, lib/mentor-match.ts) now shows an optional "Recommended for you" section above the full unfiltered listing when the viewer is logged in with future_interests (087) set and there are 2+ active mentor-session gigs to rank -- a live, per-request LLM call (same real-time posture as parse-search-query.ts's NL search, not a new stored-recommendation subsystem) ranks gigs against the viewer's stated interests plus each mentor's existing seller_rating/total_reviews as a session-rating-history signal, returning strict JSON picks mapped back to real gig rows by index (never trusting a model-returned id). Purely additive -- the full listing is unchanged and always shown. Verified end to end (two gigs on clearly different topics, a viewer whose stated interests match one of them) by ai-mentor-matching.spec.ts</v>
       </c>
       <c r="D47" t="str">
         <v>Pitch-deck AI moat review, 2026-09-01; built 2026-09-05</v>
@@ -6718,33 +6718,33 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Referral bonus tracking</v>
+        <v>AI-synthesized reference reports</v>
       </c>
       <c r="B48" t="str">
-        <v>Not built</v>
+        <v>Done</v>
       </c>
       <c r="C48" t="str">
-        <v>Referral notifications exist (040) but no monetary bonus/payout tracking for successful referrals. Ethos audit (2026-08-23) recommends a hire-and-tenure gate before building — every other monetized signal on the platform requires a verified transaction, and a naive referral bonus would be the first exception</v>
+        <v>An AI summarization layer over the existing structured references/reference_requests/reference_responses tables (065) -- once an employer has 2+ referee responses for the same candidate, a local-model synthesis (117, lib/reference-synthesis.ts) runs automatically on the next response submission and produces one consistency-flagged report (consistent | notable_differences) shown on the employer's candidate detail page, above the raw responses. Reuses the existing complete()/llm_feature_flags pattern (048); confidential to the requesting employer only, same as the raw responses it summarizes -- the candidate never sees it. Covered by ai-reference-synthesis.spec.ts (asserts no report with 1 response, report appears with 2)</v>
       </c>
       <c r="D48" t="str">
-        <v>Excluded from original benchmark scope</v>
+        <v>Pitch-deck AI moat review, 2026-09-01; built 2026-09-05</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-08-23</v>
+        <v>2026-09-05</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>jobs.salary_disclosed never set by the post-job UI</v>
+        <v>Referral bonus tracking</v>
       </c>
       <c r="B49" t="str">
-        <v>Fixed</v>
+        <v>Not built</v>
       </c>
       <c r="C49" t="str">
-        <v>Added a "publicly disclose this range" checkbox to both the post-job and edit-job forms, wired through both API routes (create + update). Real jobs posted through the UI now feed the salary_trends view's market source, and salary-trend-alert-fires.spec.ts exercises the full path end to end</v>
+        <v>Referral notifications exist (040) but no monetary bonus/payout tracking for successful referrals. Ethos audit (2026-08-23) recommends a hire-and-tenure gate before building — every other monetized signal on the platform requires a verified transaction, and a naive referral bonus would be the first exception</v>
       </c>
       <c r="D49" t="str">
-        <v>Discovered this session, fixed 2026-08-23</v>
+        <v>Excluded from original benchmark scope</v>
       </c>
       <c r="E49" t="str">
         <v>2026-08-23</v>
@@ -6752,30 +6752,30 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Skill endorsements are the one open/ungated social-proof signal</v>
+        <v>jobs.salary_disclosed never set by the post-job UI</v>
       </c>
       <c r="B50" t="str">
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="C50" t="str">
-        <v>Identified 2026-08-23, fixed 2026-08-24 per explicit user direction. Gated via a new RLS policy on skill_endorsements (064) requiring the endorser+endorsee pair to appear in the collaborators view (059, real accepted StackWorks collaboration or completed FlexPro order) — the same evidence already used for "worked together" discovery. apps/greyin-b2b/src/app/candidates/[id]/page.tsx now only renders the Endorse button when eligible, with an explanatory note otherwise; the endorse API route surfaces a real error banner instead of silently swallowing RLS failures. Found and fixed a real UX bug along the way: the endorsement count was only ever shown inside the button, so it disappeared entirely for ineligible viewers once the button got hidden — now shown as an always-visible "N endorsements" line, matching how the rating count already works. Covered end to end (positive + negative case, including a direct API bypass attempt) by skill-endorsements.spec.ts</v>
+        <v>Added a "publicly disclose this range" checkbox to both the post-job and edit-job forms, wired through both API routes (create + update). Real jobs posted through the UI now feed the salary_trends view's market source, and salary-trend-alert-fires.spec.ts exercises the full path end to end</v>
       </c>
       <c r="D50" t="str">
-        <v>Ethos audit, 2026-08-23; fixed 2026-08-24</v>
+        <v>Discovered this session, fixed 2026-08-23</v>
       </c>
       <c r="E50" t="str">
-        <v>2026-08-24</v>
+        <v>2026-08-23</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Salt &amp; Pepper karma feeds Greyin Score without a verification gate</v>
+        <v>Skill endorsements are the one open/ungated social-proof signal</v>
       </c>
       <c r="B51" t="str">
         <v>Done</v>
       </c>
       <c r="C51" t="str">
-        <v>Identified 2026-08-23, fixed 2026-08-24 per explicit user direction. The Greyin Score view's saltnpepper_raw CTE (064) now filters reputation_events to event_type='project_upvoted' only — the one reputation event type that requires another real person's action (a genuine, per-user-deduped upvote), excluding the three self-generated event types (discussion_created, reply_given, project_created) that previously counted toward a hiring-relevant score just for a user posting their own content. reputation_scores (Salt &amp; Pepper's own /members display) is untouched — posting activity is still legitimate community standing there, just no longer evidence for the cross-pillar composite. Verified via direct SQL and by saltnpepper-karma-gate.spec.ts, which confirms a builder's own project post does not move their score but a real upvote from a different account does</v>
+        <v>Identified 2026-08-23, fixed 2026-08-24 per explicit user direction. Gated via a new RLS policy on skill_endorsements (064) requiring the endorser+endorsee pair to appear in the collaborators view (059, real accepted StackWorks collaboration or completed FlexPro order) — the same evidence already used for "worked together" discovery. apps/greyin-b2b/src/app/candidates/[id]/page.tsx now only renders the Endorse button when eligible, with an explanatory note otherwise; the endorse API route surfaces a real error banner instead of silently swallowing RLS failures. Found and fixed a real UX bug along the way: the endorsement count was only ever shown inside the button, so it disappeared entirely for ineligible viewers once the button got hidden — now shown as an always-visible "N endorsements" line, matching how the rating count already works. Covered end to end (positive + negative case, including a direct API bypass attempt) by skill-endorsements.spec.ts</v>
       </c>
       <c r="D51" t="str">
         <v>Ethos audit, 2026-08-23; fixed 2026-08-24</v>
@@ -6786,50 +6786,50 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SMTP rate limiting under e2e load</v>
+        <v>Salt &amp; Pepper karma feeds Greyin Score without a verification gate</v>
       </c>
       <c r="B52" t="str">
-        <v>Parked</v>
+        <v>Done</v>
       </c>
       <c r="C52" t="str">
-        <v>Hostinger’s 500/hr SMTP cap can be hit by heavy e2e signup volume; recommended fix is swapping to a dedicated provider (Resend/SES) — not yet actioned. This is also why FR-RM-06 shipped as an in-app digest instead of a real weekly email</v>
+        <v>Identified 2026-08-23, fixed 2026-08-24 per explicit user direction. The Greyin Score view's saltnpepper_raw CTE (064) now filters reputation_events to event_type='project_upvoted' only — the one reputation event type that requires another real person's action (a genuine, per-user-deduped upvote), excluding the three self-generated event types (discussion_created, reply_given, project_created) that previously counted toward a hiring-relevant score just for a user posting their own content. reputation_scores (Salt &amp; Pepper's own /members display) is untouched — posting activity is still legitimate community standing there, just no longer evidence for the cross-pillar composite. Verified via direct SQL and by saltnpepper-karma-gate.spec.ts, which confirms a builder's own project post does not move their score but a real upvote from a different account does</v>
       </c>
       <c r="D52" t="str">
-        <v>project_smtp_rate_limit_parked.md (session memory)</v>
+        <v>Ethos audit, 2026-08-23; fixed 2026-08-24</v>
       </c>
       <c r="E52" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-24</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Full-suite run, 2026-08-23 (post-audit-deploy)</v>
+        <v>SMTP rate limiting under e2e load</v>
       </c>
       <c r="B53" t="str">
-        <v>Done — zero real regressions</v>
+        <v>Parked</v>
       </c>
       <c r="C53" t="str">
-        <v>166 tests run against prod, workers=4/retries=1. First-pass: 157 passed, 8 failed, 1 flaky (passed on retry). All 8 failures individually re-verified after fixes: 2 were real pre-existing bugs (see next 2 rows), 5 were a GoTrue read-after-write race under full-suite concurrency (not a regression — see next row), 1 was a genuine one-off ERR_NETWORK_CHANGED network blip. Every one of the 8 now passes in isolation.</v>
+        <v>Hostinger’s 500/hr SMTP cap can be hit by heavy e2e signup volume; recommended fix is swapping to a dedicated provider (Resend/SES) — not yet actioned. This is also why FR-RM-06 shipped as an in-app digest instead of a real weekly email</v>
       </c>
       <c r="D53" t="str">
-        <v>Full-suite run requested after competitive-audit deploy</v>
+        <v>project_smtp_rate_limit_parked.md (session memory)</v>
       </c>
       <c r="E53" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-21</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>GoTrue read-after-write race under full-suite load</v>
+        <v>Full-suite run, 2026-08-23 (post-audit-deploy)</v>
       </c>
       <c r="B54" t="str">
-        <v>Hardened, not a functional bug</v>
+        <v>Done — zero real regressions</v>
       </c>
       <c r="C54" t="str">
-        <v>e2e/utils/admin.ts's confirmTestUserEmail already retried a paginated admin-API user lookup for exactly this race (documented in its own comments), but the existing budget (15 pages deep, 10 retries) was sized for single-feature verification runs, not a genuine 166-test full run's signup volume. Hit 5 times in the 2026-08-23 full run (pivoter-mentor, referral-cross-app, session-persistence, sso, trust-signals — all cross-platform). Hardened to 25 pages / 15 retries; all 5 confirmed passing individually afterward, proving the underlying app features were never broken</v>
+        <v>166 tests run against prod, workers=4/retries=1. First-pass: 157 passed, 8 failed, 1 flaky (passed on retry). All 8 failures individually re-verified after fixes: 2 were real pre-existing bugs (see next 2 rows), 5 were a GoTrue read-after-write race under full-suite concurrency (not a regression — see next row), 1 was a genuine one-off ERR_NETWORK_CHANGED network blip. Every one of the 8 now passes in isolation.</v>
       </c>
       <c r="D54" t="str">
-        <v>Found during 2026-08-23 full-suite run</v>
+        <v>Full-suite run requested after competitive-audit deploy</v>
       </c>
       <c r="E54" t="str">
         <v>2026-08-23</v>
@@ -6837,33 +6837,33 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>weekly-digest.spec.ts assumed the recommendation form is always visible</v>
+        <v>GoTrue read-after-write race under full-suite load</v>
       </c>
       <c r="B55" t="str">
-        <v>Fixed</v>
+        <v>Hardened, not a functional bug</v>
       </c>
       <c r="C55" t="str">
-        <v>Found during the pre-full-run audit: the test wrote a recommendation between two strangers with no real collaboration, which written_recommendations' new gate (065, same day) now blocks — the form is hidden for ineligible viewers. Fixed by seeding a real completed FlexPro order first, same pattern as written-recommendations.spec.ts/skill-endorsements.spec.ts. Verified passing individually before the full run</v>
+        <v>e2e/utils/admin.ts's confirmTestUserEmail already retried a paginated admin-API user lookup for exactly this race (documented in its own comments), but the existing budget (15 pages deep, 10 retries) was sized for single-feature verification runs, not a genuine 166-test full run's signup volume. Hit 5 times in the 2026-08-23 full run (pivoter-mentor, referral-cross-app, session-persistence, sso, trust-signals — all cross-platform). Hardened to 25 pages / 15 retries; all 5 confirmed passing individually afterward, proving the underlying app features were never broken</v>
       </c>
       <c r="D55" t="str">
-        <v>Found during pre-full-run audit, 2026-08-24</v>
+        <v>Found during 2026-08-23 full-suite run</v>
       </c>
       <c r="E55" t="str">
-        <v>2026-08-24</v>
+        <v>2026-08-23</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Full-suite run, 2026-08-24 (post feature-batch: middleware fix, ethos gates, worked-together surfacing, reference checks, admin consolidation)</v>
+        <v>weekly-digest.spec.ts assumed the recommendation form is always visible</v>
       </c>
       <c r="B56" t="str">
-        <v>Done — zero real regressions</v>
+        <v>Fixed</v>
       </c>
       <c r="C56" t="str">
-        <v>First full run of the day (once/day cap). 172 tests run against prod, workers=4/retries=1. First-pass: 159 passed, 3 flaky (passed on retry), 10 failed even after retry — all 13 in the cross-platform project, and all 13 shared one identical root error ("Could not find newly-created test user... to confirm"), the same class of issue as the 2026-08-23 GoTrue race (see previous row), just recurring worse as the cross-platform project grew today (5 specs moved/added: session-refresh-middleware, worked-together-surfacing, admin-llm, governance-voting, gate-settings-update). None were regressions in today's actual feature work — every touched feature (middleware, skill-endorsement/recommendation/karma gates, worked-together surfacing, reference checks, admin-panel move) had already passed its own dedicated spec individually earlier in the day</v>
+        <v>Found during the pre-full-run audit: the test wrote a recommendation between two strangers with no real collaboration, which written_recommendations' new gate (065, same day) now blocks — the form is hidden for ineligible viewers. Fixed by seeding a real completed FlexPro order first, same pattern as written-recommendations.spec.ts/skill-endorsements.spec.ts. Verified passing individually before the full run</v>
       </c>
       <c r="D56" t="str">
-        <v>Full-suite run requested by user, 2026-08-24</v>
+        <v>Found during pre-full-run audit, 2026-08-24</v>
       </c>
       <c r="E56" t="str">
         <v>2026-08-24</v>
@@ -6871,16 +6871,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>GoTrue admin-lookup congestion, properly fixed (not just re-hardened)</v>
+        <v>Full-suite run, 2026-08-24 (post feature-batch: middleware fix, ethos gates, worked-together surfacing, reference checks, admin consolidation)</v>
       </c>
       <c r="B57" t="str">
-        <v>Fixed</v>
+        <v>Done — zero real regressions</v>
       </c>
       <c r="C57" t="str">
-        <v>Root-caused via direct API testing against prod (curl, service-role key): findUserIdByEmail (e2e/utils/admin.ts) was paginating GoTrue's admin users list 20-at-a-time, up to 25 sequential requests per lookup attempt, retried up to 15 times by confirmTestUserEmail — up to 375 sequential HTTP requests to the same admin endpoint per single user confirmation. Confirmed the endpoint accepts a single per_page=2000 request instead (returned all 200 then-current users in one call, matching x-total-count exactly, no truncation) -- with workers=4 running dozens of concurrent signups each doing the old 25-request dance, this was self-inflicted congestion on the admin API, not multi-second replication lag. Rewrote findUserIdByEmail to fetch in one request (~25x fewer requests per lookup); the outer retry loop is unchanged as a safety net, now far cheaper per attempt. Validated by re-running the entire cross-platform project (42 tests, not the full suite — the once/day cap applies to the full ~172-test run, already used today) under the same workers=4 concurrency: 42/42 passed, zero retries needed</v>
+        <v>First full run of the day (once/day cap). 172 tests run against prod, workers=4/retries=1. First-pass: 159 passed, 3 flaky (passed on retry), 10 failed even after retry — all 13 in the cross-platform project, and all 13 shared one identical root error ("Could not find newly-created test user... to confirm"), the same class of issue as the 2026-08-23 GoTrue race (see previous row), just recurring worse as the cross-platform project grew today (5 specs moved/added: session-refresh-middleware, worked-together-surfacing, admin-llm, governance-voting, gate-settings-update). None were regressions in today's actual feature work — every touched feature (middleware, skill-endorsement/recommendation/karma gates, worked-together surfacing, reference checks, admin-panel move) had already passed its own dedicated spec individually earlier in the day</v>
       </c>
       <c r="D57" t="str">
-        <v>Fixed and validated same day, 2026-08-24</v>
+        <v>Full-suite run requested by user, 2026-08-24</v>
       </c>
       <c r="E57" t="str">
         <v>2026-08-24</v>
@@ -6888,30 +6888,30 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>mentor-sessions.spec.ts input[name="title"] collision</v>
+        <v>GoTrue admin-lookup congestion, properly fixed (not just re-hardened)</v>
       </c>
       <c r="B58" t="str">
         <v>Fixed</v>
       </c>
       <c r="C58" t="str">
-        <v>The pre-existing spec broke once mentor-monetization.spec.ts's new "Add package" mini-form (062) was added to the same manage page — a bare input[name="title"] locator started matching 2 elements. Same fix pattern as mentor-monetization.spec.ts itself: scoped to form[action="/api/mentor-sessions/gigs"]</v>
+        <v>Root-caused via direct API testing against prod (curl, service-role key): findUserIdByEmail (e2e/utils/admin.ts) was paginating GoTrue's admin users list 20-at-a-time, up to 25 sequential requests per lookup attempt, retried up to 15 times by confirmTestUserEmail — up to 375 sequential HTTP requests to the same admin endpoint per single user confirmation. Confirmed the endpoint accepts a single per_page=2000 request instead (returned all 200 then-current users in one call, matching x-total-count exactly, no truncation) -- with workers=4 running dozens of concurrent signups each doing the old 25-request dance, this was self-inflicted congestion on the admin API, not multi-second replication lag. Rewrote findUserIdByEmail to fetch in one request (~25x fewer requests per lookup); the outer retry loop is unchanged as a safety net, now far cheaper per attempt. Validated by re-running the entire cross-platform project (42 tests, not the full suite — the once/day cap applies to the full ~172-test run, already used today) under the same workers=4 concurrency: 42/42 passed, zero retries needed</v>
       </c>
       <c r="D58" t="str">
-        <v>Found during 2026-08-23 full-suite run</v>
+        <v>Fixed and validated same day, 2026-08-24</v>
       </c>
       <c r="E58" t="str">
-        <v>2026-08-23</v>
+        <v>2026-08-24</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>jobs-and-applications.spec.ts / notifications.spec.ts waitForURL regex</v>
+        <v>mentor-sessions.spec.ts input[name="title"] collision</v>
       </c>
       <c r="B59" t="str">
         <v>Fixed</v>
       </c>
       <c r="C59" t="str">
-        <v>waitForURL(/\/applications$/) never matched the real redirect target /employer/jobs/[id]/applications?success=1 (confirmed via page snapshot that the actual status-update feature worked correctly the whole time) — a latent, pre-existing test bug unrelated to any change this session, just never previously triggered/noticed. Fixed to waitForURL(/\/applications\?success=1/) in both files</v>
+        <v>The pre-existing spec broke once mentor-monetization.spec.ts's new "Add package" mini-form (062) was added to the same manage page — a bare input[name="title"] locator started matching 2 elements. Same fix pattern as mentor-monetization.spec.ts itself: scoped to form[action="/api/mentor-sessions/gigs"]</v>
       </c>
       <c r="D59" t="str">
         <v>Found during 2026-08-23 full-suite run</v>
@@ -6922,33 +6922,33 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Login/logout not working reliably across pillars</v>
+        <v>jobs-and-applications.spec.ts / notifications.spec.ts waitForURL regex</v>
       </c>
       <c r="B60" t="str">
         <v>Fixed</v>
       </c>
       <c r="C60" t="str">
-        <v>Live bug reported directly by the user: logging in on Greyin Hub, staying logged in, then navigating to another pillar or logging out didn't reliably work. Root cause: every app's lib/supabase/server.ts cookie code has a comment saying failures there "can be ignored if you have middleware refreshing user sessions" — but only greyin-b2b actually had that middleware.ts (src/middleware.ts calling supabase.auth.getUser() on every request so a refreshed access token's Set-Cookie persists back to the browser). The other 5 apps, including Greyin Hub itself, had none — so a session open a while, or navigated across the shared .greyin.net cookie domain, could silently go stale, reading exactly as "login/logout isn't working" to a real user. The existing sso.spec.ts/logout-flow.spec.ts both do an immediate login-then-single-action flow too short-lived to ever need a token refresh, so neither caught it. Fixed by adding the same middleware.ts to all 5 remaining apps (greyin-hub, greymatters-blog, saltnpepper-community, freeagent-marketplace, stackedge); deployed to prod and confirmed with a new spec (session-refresh-middleware.spec.ts) that chains several real cross-pillar navigations starting from Greyin Hub before checking the session still holds, then verifies logout actually clears the shared cookie (not just redirects) and that the logout propagates to a second pillar too. sso.spec.ts and logout-flow.spec.ts re-run individually against prod with no regressions</v>
+        <v>waitForURL(/\/applications$/) never matched the real redirect target /employer/jobs/[id]/applications?success=1 (confirmed via page snapshot that the actual status-update feature worked correctly the whole time) — a latent, pre-existing test bug unrelated to any change this session, just never previously triggered/noticed. Fixed to waitForURL(/\/applications\?success=1/) in both files</v>
       </c>
       <c r="D60" t="str">
-        <v>User bug report, 2026-08-24; fixed same day</v>
+        <v>Found during 2026-08-23 full-suite run</v>
       </c>
       <c r="E60" t="str">
-        <v>2026-08-24</v>
+        <v>2026-08-23</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Written recommendations open to any authenticated user, no interaction gate</v>
+        <v>Login/logout not working reliably across pillars</v>
       </c>
       <c r="B61" t="str">
         <v>Fixed</v>
       </c>
       <c r="C61" t="str">
-        <v>Left open when 064 gated skill_endorsements and the Greyin Score's saltnpepper input — same self-report gap, just missed in that pass. Flagged by the user while discussing whether a "references" feature would add value; fixed the same day (2026-08-24) via the identical collaborators-view gate skill_endorsements already uses (065). The "Write a recommendation" form on candidates/[id] is now hidden for ineligible viewers (with an explanatory note), matching the endorsement UI pattern; the create route surfaces an honest error instead of a generic one. Verified end to end by written-recommendations.spec.ts (rewrote to seed a real collaboration first; added a negative case for a stranger)</v>
+        <v>Live bug reported directly by the user: logging in on Greyin Hub, staying logged in, then navigating to another pillar or logging out didn't reliably work. Root cause: every app's lib/supabase/server.ts cookie code has a comment saying failures there "can be ignored if you have middleware refreshing user sessions" — but only greyin-b2b actually had that middleware.ts (src/middleware.ts calling supabase.auth.getUser() on every request so a refreshed access token's Set-Cookie persists back to the browser). The other 5 apps, including Greyin Hub itself, had none — so a session open a while, or navigated across the shared .greyin.net cookie domain, could silently go stale, reading exactly as "login/logout isn't working" to a real user. The existing sso.spec.ts/logout-flow.spec.ts both do an immediate login-then-single-action flow too short-lived to ever need a token refresh, so neither caught it. Fixed by adding the same middleware.ts to all 5 remaining apps (greyin-hub, greymatters-blog, saltnpepper-community, freeagent-marketplace, stackedge); deployed to prod and confirmed with a new spec (session-refresh-middleware.spec.ts) that chains several real cross-pillar navigations starting from Greyin Hub before checking the session still holds, then verifies logout actually clears the shared cookie (not just redirects) and that the logout propagates to a second pillar too. sso.spec.ts and logout-flow.spec.ts re-run individually against prod with no regressions</v>
       </c>
       <c r="D61" t="str">
-        <v>User conversation, 2026-08-24</v>
+        <v>User bug report, 2026-08-24; fixed same day</v>
       </c>
       <c r="E61" t="str">
         <v>2026-08-24</v>
@@ -6956,13 +6956,13 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Employer-initiated private reference checks</v>
+        <v>Written recommendations open to any authenticated user, no interaction gate</v>
       </c>
       <c r="B62" t="str">
-        <v>Done</v>
+        <v>Fixed</v>
       </c>
       <c r="C62" t="str">
-        <v>Follow-up to the LinkedIn "connection request" discussion below: user asked whether a reference-check feature (distinct from recommendations) would add value. Assessed as a genuinely different, stronger signal — employer asks directly, candidate never sees or edits the answer — and, per explicit user direction, deliberately NOT gated to a verified interaction the way endorsements/recommendations are, since a reference is often corroborating something outside Greyin entirely (a past job). Instead: the candidate tags the relationship from a dropdown (in-platform task, ex-colleague, current colleague, other) plus free text, and any real in-platform tie is shown as additional verified context (a "Greyin-verified: worked together via X" badge, computed once at insert time via a trigger since collaborators' own RLS correctly won't let a non-participant employer query it live). New tables professional_references/reference_requests/reference_responses (065); reference_requests has no INSERT policy at all — the eligibility check spans 4 tables, so create_reference_request() (SECURITY DEFINER) is the only legitimate write path, verified directly via a blocked-bypass SQL test. Employer eligibility mirrors company_reviews: a real application at that employer's company. New UI: "Add as reference" on candidates/[id], "Your references" management + pending-request count on /profile, and /references/respond for the referee to answer privately. Verified end to end by reference-checks.spec.ts: a candidate lists two references (one plain, one with a real FlexPro order behind it), an employer requests a check tied to a real job application, the referee answers privately, the employer sees the response, and the candidate never does, anywhere</v>
+        <v>Left open when 064 gated skill_endorsements and the Greyin Score's saltnpepper input — same self-report gap, just missed in that pass. Flagged by the user while discussing whether a "references" feature would add value; fixed the same day (2026-08-24) via the identical collaborators-view gate skill_endorsements already uses (065). The "Write a recommendation" form on candidates/[id] is now hidden for ineligible viewers (with an explanatory note), matching the endorsement UI pattern; the create route surfaces an honest error instead of a generic one. Verified end to end by written-recommendations.spec.ts (rewrote to seed a real collaboration first; added a negative case for a stranger)</v>
       </c>
       <c r="D62" t="str">
         <v>User conversation, 2026-08-24</v>
@@ -6973,16 +6973,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Platform-wide admin consolidated onto Greyin Hub</v>
+        <v>Employer-initiated private reference checks</v>
       </c>
       <c r="B63" t="str">
         <v>Done</v>
       </c>
       <c r="C63" t="str">
-        <v>Two admin panels were living on pillar-specific apps despite being genuinely platform-wide: the LLM provider/feature-flag panel (apps/*/admin/llm, llm_providers/llm_feature_flags feed AI scoring across GreyMatters/Salt &amp; Pepper/FlexPro) was on StackWorks, and the eligibility-threshold governance summary + live gate-settings editor (apps/*/admin/threshold-votes, affects Verified Expert status across all four marketplace apps) was on greyin-b2b. Per explicit user direction ("move all platform-wide admin to one location"), both moved to Greyin Hub 2026-08-24 — the one app with no pillar affiliation of its own — under a new shared /admin index. The old locations on StackWorks/greyin-b2b now point to the new ones via absolute cross-app links rather than just disappearing. Member voting on the eligibility threshold itself stays on greyin-b2b/governance/threshold — only the admin-facing summary/editor moved. All API routes carried over unchanged (self-contained via each app's own absoluteUrl()). Verified end to end by 3 specs moved into e2e/tests/cross-platform/ (admin-llm.spec.ts, governance-voting.spec.ts, gate-settings-update.spec.ts), all passing against prod</v>
+        <v>Follow-up to the LinkedIn "connection request" discussion below: user asked whether a reference-check feature (distinct from recommendations) would add value. Assessed as a genuinely different, stronger signal — employer asks directly, candidate never sees or edits the answer — and, per explicit user direction, deliberately NOT gated to a verified interaction the way endorsements/recommendations are, since a reference is often corroborating something outside Greyin entirely (a past job). Instead: the candidate tags the relationship from a dropdown (in-platform task, ex-colleague, current colleague, other) plus free text, and any real in-platform tie is shown as additional verified context (a "Greyin-verified: worked together via X" badge, computed once at insert time via a trigger since collaborators' own RLS correctly won't let a non-participant employer query it live). New tables professional_references/reference_requests/reference_responses (065); reference_requests has no INSERT policy at all — the eligibility check spans 4 tables, so create_reference_request() (SECURITY DEFINER) is the only legitimate write path, verified directly via a blocked-bypass SQL test. Employer eligibility mirrors company_reviews: a real application at that employer's company. New UI: "Add as reference" on candidates/[id], "Your references" management + pending-request count on /profile, and /references/respond for the referee to answer privately. Verified end to end by reference-checks.spec.ts: a candidate lists two references (one plain, one with a real FlexPro order behind it), an employer requests a check tied to a real job application, the referee answers privately, the employer sees the response, and the candidate never does, anywhere</v>
       </c>
       <c r="D63" t="str">
-        <v>User direction, 2026-08-24</v>
+        <v>User conversation, 2026-08-24</v>
       </c>
       <c r="E63" t="str">
         <v>2026-08-24</v>
@@ -6990,47 +6990,47 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Longlist — 7th pillar, future roles posted anonymously</v>
+        <v>Platform-wide admin consolidated onto Greyin Hub</v>
       </c>
       <c r="B64" t="str">
-        <v>Done, live and e2e-covered</v>
+        <v>Done</v>
       </c>
       <c r="C64" t="str">
-        <v>User-directed: "future roles to be hired down the line (3/6/9/12 months)" as a separate pillar, not a feature bolted onto DeepEdge. Shipped as apps/longlist (own domain, own Docker service, own middleware/SSO), migrations 087 (schema + RLS) and 088 (a real bug found by direct RLS verification: the subscription INSERT check queried the base future_roles table, which members have no SELECT grant on, so even subscribing to your own future-interest was unconditionally rejected until fixed to check future_roles_public instead). Anonymity is structural (a column-filtered view, no company_id/posted_by ever exposed), not a UI convention -- verified directly via SET LOCAL role authenticated + request.jwt.claims. AI-matching second candidate set rides the existing llm_feature_flags registry, defaulted OFF. Cross-linked into all 6 existing apps' nav + notification-link.ts, greyin-hub's landing page, and greyin-b2b's /about page. DNS (longlist.greyin.net, configured by the user on the Hostinger panel) resolved and a real Let's Encrypt cert issued after force-restarting the shared Traefik service to pick up the new router -- confirmed live over HTTPS. E2E: 4 specs in tests/longlist/ + 2 in tests/cross-platform/longlist-future-roles.spec.ts (the full anonymized-post -&gt; subscribe -&gt; employer-sees-candidate flow, and a stranger-gets-404 negative case), 6/6 passing. Two real bugs found and fixed while getting these green, neither caught by the earlier direct-SQL-only verification: (1) PostgREST's schema cache was stale for the new future_roles table/profiles columns (PGRST204 "column does not exist" on every write through the Supabase JS client, even though direct psql worked fine) -- another instance of the same class NFR-OPS-01 already documents (NOTIFY pgrst alone doesn't reliably propagate through this deployment), fixed with docker service update --force supabase_rest; (2) a test-authoring bug in profile-future-interests.spec.ts assumed login() would land on an arbitrary expectedUrl, when it only ever waits for wherever the login route actually redirects (always /dashboard for Longlist, no role branching) -- fixed by navigating separately after login instead of asserting through it. Also hit and cleared this session's own SEC-017 signup rate limit (10/hour/IP, shared across all 6 apps' signup routes since they key on the same rate_limit_attempts table and this session's test traffic all shares one IP) -- expected behavior working as designed, not a bug, just self-inflicted by the volume of same-day testing. FR-LL-04/05 (AI-matching, role-filled notification) remain uncovered by e2e -- flagged as a follow-up, not silently skipped.</v>
+        <v>Two admin panels were living on pillar-specific apps despite being genuinely platform-wide: the LLM provider/feature-flag panel (apps/*/admin/llm, llm_providers/llm_feature_flags feed AI scoring across GreyMatters/Salt &amp; Pepper/FlexPro) was on StackWorks, and the eligibility-threshold governance summary + live gate-settings editor (apps/*/admin/threshold-votes, affects Verified Expert status across all four marketplace apps) was on greyin-b2b. Per explicit user direction ("move all platform-wide admin to one location"), both moved to Greyin Hub 2026-08-24 — the one app with no pillar affiliation of its own — under a new shared /admin index. The old locations on StackWorks/greyin-b2b now point to the new ones via absolute cross-app links rather than just disappearing. Member voting on the eligibility threshold itself stays on greyin-b2b/governance/threshold — only the admin-facing summary/editor moved. All API routes carried over unchanged (self-contained via each app's own absoluteUrl()). Verified end to end by 3 specs moved into e2e/tests/cross-platform/ (admin-llm.spec.ts, governance-voting.spec.ts, gate-settings-update.spec.ts), all passing against prod</v>
       </c>
       <c r="D64" t="str">
-        <v>User request, 2026-08-31</v>
+        <v>User direction, 2026-08-24</v>
       </c>
       <c r="E64" t="str">
-        <v>2026-08-31</v>
+        <v>2026-08-24</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Three pillars rebranded: ExpertEdge -&gt; DeepEdge, FreeAgent -&gt; FlexPro, StackEdge -&gt; StackWorks</v>
+        <v>Longlist — 7th pillar, future roles posted anonymously</v>
       </c>
       <c r="B65" t="str">
-        <v>Done -- migrated and redeployed</v>
+        <v>Done, live and e2e-covered</v>
       </c>
       <c r="C65" t="str">
-        <v>User-directed naming pass, following on from the deck/traceability naming discussion this same session. Domains cut over (Hostinger A-records for flexpro/deepedge/stackworks.greyin.net added by the user, old expertedge/freeagent/stackedge A-records already repointed to localhost -- confirmed dead before this migration touched anything). FreeAgent specifically fixes a real trademark-collision risk (an existing UK accounting SaaS company already uses that name), not just a style preference. Scope deliberately limited to the brand/domain layer, matching the precedent already set by ExpertEdge itself (which has run as apps/greyin-b2b, branded differently from its folder, since the app was built) and by StackEdge's own earlier rename from Prolab (047): app folder names, Docker image names, Compose service keys, Traefik router/service IDs, e2e test directory names, and e2e helper function names (signUpFreeAgent, signUpGreyinB2B, signUpStackEdgeBuilder/Supporter) all kept as internal codenames -- renaming those would touch dozens of files for zero user-facing benefit and meaningfully risk the 125-spec e2e suite. What changed: deployment/.env + .env.example (domain env vars renamed and repointed), frontend-stack.yml (Host() rules + NEXT_PUBLIC_SITE_URL, plus updated section-header comments), every app's displayed brand text (SiteHeader wordmarks, page titles/metadata, hero/terms/privacy copy), the shared PILLARS array in all 7 apps' EcosystemWidget.tsx (label + url, key left unchanged), the FeedCard.tsx/EcosystemSearchResults.tsx pillar-label maps duplicated across 5 apps, notification-link.ts's PILLAR_DOMAINS in 6 apps, and every literal cross-app mention (greyin-hub's pivoting/reentry/dashboard/admin pages, longlist's employer-onboarding links, greyin-b2b/about, greymatters/about). Caught via a full domain-string sweep (26 files still had lowercase href="https://expertedge.greyin.net"-style literals the brand-name text replace didn't touch) and a separate e2e sweep that found real breaking assertions -- most importantly playwright.config.ts's own baseURLs for the greyin-b2b/freeagent/stackedge projects, which would have pointed the entire e2e suite at now-dead domains if missed, plus specific getByText/name: assertions in navigation.spec.ts, homepage.spec.ts, greyin-score.spec.ts, trust-signals.spec.ts, freeagent-trust-signal.spec.ts, worked-together-surfacing.spec.ts, logout-flow.spec.ts, and reference-checks.spec.ts checking literal old brand text that the app no longer renders. All 7 apps typecheck clean post-rename.</v>
+        <v>User-directed: "future roles to be hired down the line (3/6/9/12 months)" as a separate pillar, not a feature bolted onto DeepEdge. Shipped as apps/longlist (own domain, own Docker service, own middleware/SSO), migrations 087 (schema + RLS) and 088 (a real bug found by direct RLS verification: the subscription INSERT check queried the base future_roles table, which members have no SELECT grant on, so even subscribing to your own future-interest was unconditionally rejected until fixed to check future_roles_public instead). Anonymity is structural (a column-filtered view, no company_id/posted_by ever exposed), not a UI convention -- verified directly via SET LOCAL role authenticated + request.jwt.claims. AI-matching second candidate set rides the existing llm_feature_flags registry, defaulted OFF. Cross-linked into all 6 existing apps' nav + notification-link.ts, greyin-hub's landing page, and greyin-b2b's /about page. DNS (longlist.greyin.net, configured by the user on the Hostinger panel) resolved and a real Let's Encrypt cert issued after force-restarting the shared Traefik service to pick up the new router -- confirmed live over HTTPS. E2E: 4 specs in tests/longlist/ + 2 in tests/cross-platform/longlist-future-roles.spec.ts (the full anonymized-post -&gt; subscribe -&gt; employer-sees-candidate flow, and a stranger-gets-404 negative case), 6/6 passing. Two real bugs found and fixed while getting these green, neither caught by the earlier direct-SQL-only verification: (1) PostgREST's schema cache was stale for the new future_roles table/profiles columns (PGRST204 "column does not exist" on every write through the Supabase JS client, even though direct psql worked fine) -- another instance of the same class NFR-OPS-01 already documents (NOTIFY pgrst alone doesn't reliably propagate through this deployment), fixed with docker service update --force supabase_rest; (2) a test-authoring bug in profile-future-interests.spec.ts assumed login() would land on an arbitrary expectedUrl, when it only ever waits for wherever the login route actually redirects (always /dashboard for Longlist, no role branching) -- fixed by navigating separately after login instead of asserting through it. Also hit and cleared this session's own SEC-017 signup rate limit (10/hour/IP, shared across all 6 apps' signup routes since they key on the same rate_limit_attempts table and this session's test traffic all shares one IP) -- expected behavior working as designed, not a bug, just self-inflicted by the volume of same-day testing. FR-LL-04/05 (AI-matching, role-filled notification) remain uncovered by e2e -- flagged as a follow-up, not silently skipped.</v>
       </c>
       <c r="D65" t="str">
-        <v>User request, 2026-09-01</v>
+        <v>User request, 2026-08-31</v>
       </c>
       <c r="E65" t="str">
-        <v>2026-09-01</v>
+        <v>2026-08-31</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Full code sweep for untracked-but-shipped features</v>
+        <v>Three pillars rebranded: ExpertEdge -&gt; DeepEdge, FreeAgent -&gt; FlexPro, StackEdge -&gt; StackWorks</v>
       </c>
       <c r="B66" t="str">
-        <v>Done -- 6 documentation gaps found and closed, zero implementation or test gaps found</v>
+        <v>Done -- migrated and redeployed</v>
       </c>
       <c r="C66" t="str">
-        <v>User-directed, prompted by discovering Outplacement had zero FR row despite being real and tested. Method: diffed every migration (001-088) against every migration number actually cited anywhere in this file, then read the ones that came back genuinely uncited (046, 049, 052) plus a few with only passing prose mentions (025, 032-034, 044) to judge whether each was a real distinct feature or a pure fix. Also ran a blunt route-path-fragment grep across all 127 API routes against every spec file to surface untested candidates -- noisy (most hits were false positives; specs test via UI flows, not literal route strings, e.g. jobs/create genuinely is tested by jobs-and-applications.spec.ts despite not string-matching) but useful for triage. Four real, shipped, already-e2e-tested features had no FR row at all: Fractional Leadership Placement and Outplacement (both sales-led enterprise offerings, migration 044, tested by enterprise-solutions.spec.ts -- now FR-EE-12/13, and Outplacement is one of Greyin's three Primary/revenue tiers per the pitch deck's tier restructuring this same request), the personal cross-pillar activity calendar on Greyin Hub's dashboard (migrations 046/047, tested by hub-dashboard.spec.ts -- now FR-PW-23), and GreyMatters' admin-triggered real-email newsletter digest send (migration 052, tested by admin-digest-send.spec.ts -- now FR-GM-06, and worth noting it sends real email despite FR-RM-06's cross-pillar digest deliberately avoiding email over the known SMTP rate-limit constraint; different scope, different volume, both correct). Two existing FR rows had incomplete migration citations, fixed rather than left: FR-SP-01 (Salt &amp; Pepper karma) was missing 025, the migration that actually creates reputation_events; FR-SE-03 (StackWorks verification) was missing 032-034, which close a self-review hole and enable a Builder's own project_shipped self-submission -- a real workflow variant beyond what the row's original text described. No new engineering or test-writing was needed for any of the six -- every one was already correctly implemented and already had real e2e coverage; the gap was purely in this document, not in the product.</v>
+        <v>User-directed naming pass, following on from the deck/traceability naming discussion this same session. Domains cut over (Hostinger A-records for flexpro/deepedge/stackworks.greyin.net added by the user, old expertedge/freeagent/stackedge A-records already repointed to localhost -- confirmed dead before this migration touched anything). FreeAgent specifically fixes a real trademark-collision risk (an existing UK accounting SaaS company already uses that name), not just a style preference. Scope deliberately limited to the brand/domain layer, matching the precedent already set by ExpertEdge itself (which has run as apps/greyin-b2b, branded differently from its folder, since the app was built) and by StackEdge's own earlier rename from Prolab (047): app folder names, Docker image names, Compose service keys, Traefik router/service IDs, e2e test directory names, and e2e helper function names (signUpFreeAgent, signUpGreyinB2B, signUpStackEdgeBuilder/Supporter) all kept as internal codenames -- renaming those would touch dozens of files for zero user-facing benefit and meaningfully risk the 125-spec e2e suite. What changed: deployment/.env + .env.example (domain env vars renamed and repointed), frontend-stack.yml (Host() rules + NEXT_PUBLIC_SITE_URL, plus updated section-header comments), every app's displayed brand text (SiteHeader wordmarks, page titles/metadata, hero/terms/privacy copy), the shared PILLARS array in all 7 apps' EcosystemWidget.tsx (label + url, key left unchanged), the FeedCard.tsx/EcosystemSearchResults.tsx pillar-label maps duplicated across 5 apps, notification-link.ts's PILLAR_DOMAINS in 6 apps, and every literal cross-app mention (greyin-hub's pivoting/reentry/dashboard/admin pages, longlist's employer-onboarding links, greyin-b2b/about, greymatters/about). Caught via a full domain-string sweep (26 files still had lowercase href="https://expertedge.greyin.net"-style literals the brand-name text replace didn't touch) and a separate e2e sweep that found real breaking assertions -- most importantly playwright.config.ts's own baseURLs for the greyin-b2b/freeagent/stackedge projects, which would have pointed the entire e2e suite at now-dead domains if missed, plus specific getByText/name: assertions in navigation.spec.ts, homepage.spec.ts, greyin-score.spec.ts, trust-signals.spec.ts, freeagent-trust-signal.spec.ts, worked-together-surfacing.spec.ts, logout-flow.spec.ts, and reference-checks.spec.ts checking literal old brand text that the app no longer renders. All 7 apps typecheck clean post-rename.</v>
       </c>
       <c r="D66" t="str">
         <v>User request, 2026-09-01</v>
@@ -7041,47 +7041,47 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>LinkedIn-style "connection request" — considered, rejected in favor of surfacing real collaborators</v>
+        <v>Full code sweep for untracked-but-shipped features</v>
       </c>
       <c r="B67" t="str">
-        <v>Done (alternative shipped)</v>
+        <v>Done -- 6 documentation gaps found and closed, zero implementation or test gaps found</v>
       </c>
       <c r="C67" t="str">
-        <v>User asked whether Greyin had a LinkedIn-style mutual connect-request feature; it didn't. Assessed against the platform ethos and rejected: a request/accept graph is, by construction, two strangers mutually self-declaring a relationship with zero verification — the same class of gap the skill-endorsement and Salt &amp; Pepper karma gates (064) were built to close, not reopen. DMs are already open to any authenticated user and profiles are already unpaywalled, so a connection wouldn't even unlock anything LinkedIn-equivalent. Shipped the on-ethos alternative instead: surfaced the collaborators view (059, real accepted StackWorks collaborations + completed FlexPro orders) properly rather than adding a new unverified signal. (A) the existing "people you've worked with" pill widgets on StackWorks /people and Salt &amp; Pepper /members now link to the person's profile and show which pillar via; (B) individual profile pages (greyin-b2b/candidates/[id], freeagent/sellers/[id]) now show an inline "You've worked together via X" note when the viewer and the profile actually share a collaborators row — freeagent/sellers/[id] had zero collaborators awareness before; (C) Greyin Hub's dashboard now has one canonical cross-pillar "People you've worked with" section, rather than duplicating a per-app module (the same "5 independently-drifting copies" pattern that caused the login/logout middleware bug above). Verified end to end by worked-together-surfacing.spec.ts: a real completed FlexPro order makes the collaborator show up correctly on Hub and on the seller profile, and confirms a stranger with no real interaction sees neither</v>
+        <v>User-directed, prompted by discovering Outplacement had zero FR row despite being real and tested. Method: diffed every migration (001-088) against every migration number actually cited anywhere in this file, then read the ones that came back genuinely uncited (046, 049, 052) plus a few with only passing prose mentions (025, 032-034, 044) to judge whether each was a real distinct feature or a pure fix. Also ran a blunt route-path-fragment grep across all 127 API routes against every spec file to surface untested candidates -- noisy (most hits were false positives; specs test via UI flows, not literal route strings, e.g. jobs/create genuinely is tested by jobs-and-applications.spec.ts despite not string-matching) but useful for triage. Four real, shipped, already-e2e-tested features had no FR row at all: Fractional Leadership Placement and Outplacement (both sales-led enterprise offerings, migration 044, tested by enterprise-solutions.spec.ts -- now FR-EE-12/13, and Outplacement is one of Greyin's three Primary/revenue tiers per the pitch deck's tier restructuring this same request), the personal cross-pillar activity calendar on Greyin Hub's dashboard (migrations 046/047, tested by hub-dashboard.spec.ts -- now FR-PW-23), and GreyMatters' admin-triggered real-email newsletter digest send (migration 052, tested by admin-digest-send.spec.ts -- now FR-GM-06, and worth noting it sends real email despite FR-RM-06's cross-pillar digest deliberately avoiding email over the known SMTP rate-limit constraint; different scope, different volume, both correct). Two existing FR rows had incomplete migration citations, fixed rather than left: FR-SP-01 (Salt &amp; Pepper karma) was missing 025, the migration that actually creates reputation_events; FR-SE-03 (StackWorks verification) was missing 032-034, which close a self-review hole and enable a Builder's own project_shipped self-submission -- a real workflow variant beyond what the row's original text described. No new engineering or test-writing was needed for any of the six -- every one was already correctly implemented and already had real e2e coverage; the gap was purely in this document, not in the product.</v>
       </c>
       <c r="D67" t="str">
-        <v>User request, 2026-08-24</v>
+        <v>User request, 2026-09-01</v>
       </c>
       <c r="E67" t="str">
-        <v>2026-08-24</v>
+        <v>2026-09-01</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Peer-confirmed projects (off-platform work history) + anonymous peer ratings + employer reciprocity detection + admin moderation</v>
+        <v>LinkedIn-style "connection request" — considered, rejected in favor of surfacing real collaborators</v>
       </c>
       <c r="B68" t="str">
-        <v>Done, live and e2e-covered -- admin moderation UI added same day, remaining gaps flagged below, not yet closed</v>
+        <v>Done (alternative shipped)</v>
       </c>
       <c r="C68" t="str">
-        <v>User proposed the use case (add off-platform projects, tag real teammates, rate contribution) and asked for a business-value assessment before building. Assessed as solving a real cold-start gap (every existing trust signal requires an on-platform transaction; a senior member's entire pre-Greyin career contributes nothing) with a real viral-acquisition angle (tagging a non-member is an invite hook), conditioned on three things the initial assessment flagged as required, not optional: (1) never call it "verified" -- reserved for transaction-backed evidence elsewhere on the platform, this is "peer-confirmed" throughout; (2) mutual confirmation as a real gate, not a courtesy -- a tag stays private until the tagged member actively confirms; (3) ratings anonymous by default. User then explicitly asked for the peer_score to be a fully separate number from the platform-verified Greyin Score, never blended -- built that way (089): platform_composite/greyin_score/is_verified_expert still compute only from StackWorks/FlexPro/Salt&amp;Pepper/GreyMatters, peer_score is a sibling column nobody's gate reads. User then raised the sharpest requirement: ratings must be genuinely anonymous at the RLS layer (not just an app convention) for regular members, but employers specifically need to see a given rater's rating-giving PATTERN, to catch reciprocal quid-pro-quo grade-inflation between colluding peers. Initially shipped following company_reviews' (058) "anonymity is an app convention" precedent, USING(true) -- caught as insufficient against this specific requirement before rollout and tightened (090) to real row-level restriction (self-caught, logged as SEC-039). Two new employer/admin-gated aggregate views followed: peer_rater_reliability (a rater's overall pattern -- avg rating given, % top-rating, % of ratings that are part of a mutual pair where both sides rated each other 4+) and peer_project_reciprocity_flags (090, 091 -- the same detection at per-project granularity, surfaced as a "⚠ Possible reciprocal rating" badge on the specific flagged project, added after the user asked for project-level flagging specifically rather than only an aggregate rater-level number). Schema: peer_projects/peer_project_members/peer_project_ratings (089), collaborators view extended with a third 'peer' source (mutually-confirmed pairs only), greyin_scores extended with peer_score/peer_evidence/peer_headcount as trailing columns (CREATE OR REPLACE VIEW's column-position constraint required restructuring the query into a `gated` CTE to append them after is_verified_expert rather than before years_experience -- caught by the DB itself rejecting the first attempt, not found via review). UI: greyin-hub/dashboard (add project, tag via a platform_people_index-backed live search, confirm/decline pending tags, rate confirmed teammates using performance-review-style labels -- 1="Did not meet expectations" through 5="Exceeded expectations" -- rather than a bare number) and greyin-b2b/candidates/[id] (employer-only rating-pattern panel + per-project reciprocity flag; the peer-confirmed project list itself is public to any viewer, only the pattern/flag are employer-gated). Verified via direct RLS simulation as rater/non-rater/employer/non-employer (mutual-pair reciprocity math confirmed correct: a rater with one reciprocal + one one-directional rating correctly shows 50%, a rater with only a reciprocal rating shows 100%) and end to end via peer-projects.spec.ts (real signups, real UI tag/confirm/rate flow across two browser contexts, employer sees the flag, a regular member does not). One real app-layer bug found and fixed during e2e verification that had nothing to do with the schema: a locator matching on displayed name text picked up the dashboard's unrelated "People you've worked with" module (which independently renders the same names) instead of the intended rating form -- fixed by scoping the test locator to the rating form's own ratee_id hidden input instead of name text; several rebuild/redeploy cycles and live server-side debug logging were needed to isolate this from a false "stale data" hypothesis before finding the real cause. GAPS/IMPROVEMENTS RECOMMENDED BEFORE WIDER ROLLOUT, not yet built: (a) reciprocity detection is pairwise only -- a 3+-account round-robin ring (A rates B, B rates C, C rates A, never a direct mutual pair) evades both peer_rater_reliability and peer_project_reciprocity_flags entirely; (b) no rate limiting on peer_projects/peer_project_members/peer_project_ratings creation -- unlike signup (SEC-017), nothing stops spamming fake projects/tags/ratings; (c) no path for a CONFIRMED member to later withdraw their confirmation (only a still-pending tag can be removed, by the creator) -- worth a considered decision on what should happen to any ratings already given if a withdrawal were added; (d) company name on a peer project is free text with no employer attestation -- correctly framed as peer-confirmed not employer-verified, but worth stating plainly as a known limitation rather than an implicit one; (e) the 50%-mutual-high-rating-pct threshold used for the employer UI's visual warning is an unvalidated heuristic (chosen at build time, not calibrated against any real usage data, since the platform has none yet); (f) peer_score's Bayesian-shrinkage constant (m_peer=3) was set by pattern-matching StackWorks' own m=3, not derived from real data either; (g) e2e coverage is otherwise still happy-path only -- declining a tag and the "creator can only edit before anyone confirms" lock remain untested. FOLLOW-UP THE SAME DAY -- admin moderation (FR-PW-27), CLOSED: user asked to check the admin flow specifically and add it to the test suite -- this was gap (e) in the original list ("no admin moderation UI... only raw SQL"), now removed from the open list above. Built /admin/peer-projects on Greyin Hub (new card on the existing platform-wide /admin index, same "no pillar affiliation of its own" rationale as the LLM-provider and eligibility-governance panels already there) -- lists the 50 most recent projects, flagged ones (via peer_project_reciprocity_flags) sorted first with the same "⚠ Possible reciprocal rating" badge an employer sees, delete cascades to members/ratings. RLS's existing admin-DELETE policy (089) is the real enforcement; the page's own role check is just UX (redirect before a non-admin sees the button). Verified end to end via peer-projects-admin.spec.ts: a non-admin visiting the URL directly is redirected to /dashboard, and an admin sees a real flagged project (same tag/confirm/mutual-rate flow as peer-projects.spec.ts) and successfully deletes it. This also closes the admin-delete half of the former e2e-coverage gap -- (g) above is only decline/edit-lock now, not admin-delete.</v>
+        <v>User asked whether Greyin had a LinkedIn-style mutual connect-request feature; it didn't. Assessed against the platform ethos and rejected: a request/accept graph is, by construction, two strangers mutually self-declaring a relationship with zero verification — the same class of gap the skill-endorsement and Salt &amp; Pepper karma gates (064) were built to close, not reopen. DMs are already open to any authenticated user and profiles are already unpaywalled, so a connection wouldn't even unlock anything LinkedIn-equivalent. Shipped the on-ethos alternative instead: surfaced the collaborators view (059, real accepted StackWorks collaborations + completed FlexPro orders) properly rather than adding a new unverified signal. (A) the existing "people you've worked with" pill widgets on StackWorks /people and Salt &amp; Pepper /members now link to the person's profile and show which pillar via; (B) individual profile pages (greyin-b2b/candidates/[id], freeagent/sellers/[id]) now show an inline "You've worked together via X" note when the viewer and the profile actually share a collaborators row — freeagent/sellers/[id] had zero collaborators awareness before; (C) Greyin Hub's dashboard now has one canonical cross-pillar "People you've worked with" section, rather than duplicating a per-app module (the same "5 independently-drifting copies" pattern that caused the login/logout middleware bug above). Verified end to end by worked-together-surfacing.spec.ts: a real completed FlexPro order makes the collaborator show up correctly on Hub and on the seller profile, and confirms a stranger with no real interaction sees neither</v>
       </c>
       <c r="D68" t="str">
-        <v>User request, 2026-09-02</v>
+        <v>User request, 2026-08-24</v>
       </c>
       <c r="E68" t="str">
-        <v>2026-09-02</v>
+        <v>2026-08-24</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>FlexPro revenue model rebuild: client-posted jobs, subscription-gated posting, 2% both-sides service fee, bidirectional disputes</v>
+        <v>Peer-confirmed projects (off-platform work history) + anonymous peer ratings + employer reciprocity detection + admin moderation</v>
       </c>
       <c r="B69" t="str">
-        <v>Done, live and e2e-covered</v>
+        <v>Done, live and e2e-covered -- admin moderation UI added same day, remaining gaps flagged below, not yet closed</v>
       </c>
       <c r="C69" t="str">
-        <v>Started from a chain of user questions rather than a single spec: (1) asked to check whether FreeAgent had any "expert posts a gig, others apply" mechanism -- confirmed it did not (only seller-lists-a-listing, buyer-purchases-directly existed); (2) user then specified the real intended model -- experts can ALSO post as a client (not just offer services as a freelancer), both sides pay a subscription to post, plus a service fee per accepted transaction, and if that means "0%-commission" is no longer accurate, retire the wording; explicitly asked for a red-flag/dispute mechanism for both sides ("to avoid pay conflicts/bad deliverables upon breach of trust"); confirmed StackWorks stays a free crowdwork model, unaffected. This surfaced a real pre-existing discrepancy before any of it was built: the "0%-commission" claim (PILLARS description, signup/terms/gigs-new copy, pitch deck) was already false in the OPPOSITE direction -- posting was free but the freelancer was already being charged a real 2% platform fee at payout. Two architectural decisions confirmed with the user before writing schema: one unified subscription (not two) covering both post-as-freelancer and post-as-client, matching the platform's existing "one identity, many roles" pattern; and the service fee split both sides rather than one, smaller each. The 2% rate itself was NOT invented for this feature -- it's the exact rate the existing gig-purchase checkout/payout flow already used on both sides (buyer-side fee shown at checkout, seller-side deduction at payout), so this pass just named and extended an already-real number rather than picking a new one. Schema (093): freeagent_subscriptions (mirrors 039's company_subscriptions design exactly, user-scoped since FreeAgent has no company concept), client_jobs + client_job_applications (free to apply, no subscription needed -- only posting either kind of listing is gated), and gig_orders extended with a nullable gig_id + client_job_application_id as an alternate origin so client-job engagements reuse the ENTIRE existing escrow/delivery/dispute/refund/Razorpay machinery wholesale rather than duplicating a ~35-column table -- confirmed safe before writing by reading every existing gig_orders RLS policy first: all of them key off buyer_id/seller_id directly, never gig_id, so zero RLS changes were needed there. 094 gates the pre-existing gigs INSERT policy the same way (posting a gig was never gated before, despite the old "0%" claim implying some model existed). Two real pre-existing bugs found only because this feature exercised gig_orders in a genuinely new way, both fixed in 095, and neither specific to this feature -- a pre-claim-then-attach-Razorpay-order pattern (api/orders/create's own "preClaimedOrderId" path, already used by mentor-session bookings) was silently broken by 068/073's immutable-fields trigger, which blocked razorpay_order_id's legitimate first-time NULL-to-value transition, not just later tampering -- caught immediately by e2e (mockRazorpayCheckout succeeding, then the DB update failing with the trigger's own exception), and very likely a live, if less-exercised, gap in mentor-session checkout too, not something newly introduced; separately, the DB trigger enforcing the 'disputed' transition was ALSO still buyer-only underneath the app-layer route fix below, which alone would not have been sufficient. Full pg_get_functiondef of the original trigger was read before writing the replacement, to guarantee every existing transition rule (revision requests, admin dispute resolution, buyer cancellation, seller delivery) was preserved verbatim and not accidentally dropped. api/orders/dispute/route.ts's buyer-only restriction was lifted (either buyer_id or seller_id can now raise a dispute, disputed_by records who) with matching UI added to orders/[id]/page.tsx for the seller's own waiting/revision states, which previously showed the seller nothing at all once they'd delivered. UI: /subscribe (mirrors greyin-b2b's own subscription checkout page, Razorpay Subscriptions), /client-jobs (browse/post/detail with apply form + owner accept/reject), /client-jobs/[id]/pay/[orderId] (a job-engagement-specific checkout, no package selection since the accepted application already fixed one price) reusing api/orders/create/verify with a new clientJobEngagement branch rather than a parallel payment flow. All "0%-commission" wording retired platform-wide (PILLARS.description in all 7 apps, FreeAgent's signup/terms/gigs-new copy, and the pitch deck's customer-opportunity and pillar-summary slides) in favor of accurately describing the real model. Verified end to end via client-jobs.spec.ts (real subscription grant, gate correctly blocks/allows posting, free application, accept creates a real gig_orders row via the real UI + mocked Razorpay checkout.js, stored amount/service_fee_buyer/service_fee_seller read back and confirmed exactly correct -- 9000/180/180 for a 9000 proposed price) plus re-running the pre-existing payment-critical suite after the shared-infrastructure changes: checkout-payment.spec.ts and all 3 escrow-workflow.spec.ts cases (revision/redelivery, buyer cancel+refund, admin dispute resolution) pass clean, confirming 095's trigger rewrite preserved every existing transition rule. The new subscription gate on gig-posting is a real, deliberate breaking change to 14 pre-existing e2e specs that post a gig as a normal part of their own setup (checkout-payment, escrow-workflow, gigs-filters, earnings-and-payouts, webhook-payment-captured, order-lifecycle, notifications, auth-and-gigs, admin, ai-quality-score, image-upload, top-tier-badge, top-tier-badge-positive, activity-feed) -- all 14 updated (grantFreeagentSubscription called before posting, same "grant directly, don't drive the real subscription-checkout UI in e2e" precedent already established for greyin-b2b's own enterprise subscriptions) and 5 of the 14 re-run clean (checkout-payment, all 3 escrow-workflow cases, order-lifecycle, gigs-filters); the remaining 9 (webhook-payment-captured, notifications, auth-and-gigs, admin, ai-quality-score, image-upload, top-tier-badge, top-tier-badge-positive, activity-feed) were re-run individually in a follow-up pass per explicit user request ("re-run the remaining 9 as well") -- 8 of 9 passed clean (one file, admin.spec.ts, needed a direct fix first: its pre-existing multi-line import statement wasn't matched by the earlier batch-fix script's single-line regex, producing a duplicate conflicting import; fixed by hand). image-upload.spec.ts failed, investigated, and confirmed unrelated to this feature -- the only edit to api/gigs/create/route.ts was a purely additive subscription check inserted before all pre-existing image/gig-insert logic, and no gig row persisted in the DB (cleaned up by test teardown before it could be inspected further), consistent with a pre-existing flake in the image-upload pipeline itself, not a regression from this work. Reported honestly as a known, separate, unresolved issue rather than claimed fixed.</v>
+        <v>User proposed the use case (add off-platform projects, tag real teammates, rate contribution) and asked for a business-value assessment before building. Assessed as solving a real cold-start gap (every existing trust signal requires an on-platform transaction; a senior member's entire pre-Greyin career contributes nothing) with a real viral-acquisition angle (tagging a non-member is an invite hook), conditioned on three things the initial assessment flagged as required, not optional: (1) never call it "verified" -- reserved for transaction-backed evidence elsewhere on the platform, this is "peer-confirmed" throughout; (2) mutual confirmation as a real gate, not a courtesy -- a tag stays private until the tagged member actively confirms; (3) ratings anonymous by default. User then explicitly asked for the peer_score to be a fully separate number from the platform-verified Greyin Score, never blended -- built that way (089): platform_composite/greyin_score/is_verified_expert still compute only from StackWorks/FlexPro/Salt&amp;Pepper/GreyMatters, peer_score is a sibling column nobody's gate reads. User then raised the sharpest requirement: ratings must be genuinely anonymous at the RLS layer (not just an app convention) for regular members, but employers specifically need to see a given rater's rating-giving PATTERN, to catch reciprocal quid-pro-quo grade-inflation between colluding peers. Initially shipped following company_reviews' (058) "anonymity is an app convention" precedent, USING(true) -- caught as insufficient against this specific requirement before rollout and tightened (090) to real row-level restriction (self-caught, logged as SEC-039). Two new employer/admin-gated aggregate views followed: peer_rater_reliability (a rater's overall pattern -- avg rating given, % top-rating, % of ratings that are part of a mutual pair where both sides rated each other 4+) and peer_project_reciprocity_flags (090, 091 -- the same detection at per-project granularity, surfaced as a "⚠ Possible reciprocal rating" badge on the specific flagged project, added after the user asked for project-level flagging specifically rather than only an aggregate rater-level number). Schema: peer_projects/peer_project_members/peer_project_ratings (089), collaborators view extended with a third 'peer' source (mutually-confirmed pairs only), greyin_scores extended with peer_score/peer_evidence/peer_headcount as trailing columns (CREATE OR REPLACE VIEW's column-position constraint required restructuring the query into a `gated` CTE to append them after is_verified_expert rather than before years_experience -- caught by the DB itself rejecting the first attempt, not found via review). UI: greyin-hub/dashboard (add project, tag via a platform_people_index-backed live search, confirm/decline pending tags, rate confirmed teammates using performance-review-style labels -- 1="Did not meet expectations" through 5="Exceeded expectations" -- rather than a bare number) and greyin-b2b/candidates/[id] (employer-only rating-pattern panel + per-project reciprocity flag; the peer-confirmed project list itself is public to any viewer, only the pattern/flag are employer-gated). Verified via direct RLS simulation as rater/non-rater/employer/non-employer (mutual-pair reciprocity math confirmed correct: a rater with one reciprocal + one one-directional rating correctly shows 50%, a rater with only a reciprocal rating shows 100%) and end to end via peer-projects.spec.ts (real signups, real UI tag/confirm/rate flow across two browser contexts, employer sees the flag, a regular member does not). One real app-layer bug found and fixed during e2e verification that had nothing to do with the schema: a locator matching on displayed name text picked up the dashboard's unrelated "People you've worked with" module (which independently renders the same names) instead of the intended rating form -- fixed by scoping the test locator to the rating form's own ratee_id hidden input instead of name text; several rebuild/redeploy cycles and live server-side debug logging were needed to isolate this from a false "stale data" hypothesis before finding the real cause. GAPS/IMPROVEMENTS RECOMMENDED BEFORE WIDER ROLLOUT, not yet built: (a) reciprocity detection is pairwise only -- a 3+-account round-robin ring (A rates B, B rates C, C rates A, never a direct mutual pair) evades both peer_rater_reliability and peer_project_reciprocity_flags entirely; (b) no rate limiting on peer_projects/peer_project_members/peer_project_ratings creation -- unlike signup (SEC-017), nothing stops spamming fake projects/tags/ratings; (c) no path for a CONFIRMED member to later withdraw their confirmation (only a still-pending tag can be removed, by the creator) -- worth a considered decision on what should happen to any ratings already given if a withdrawal were added; (d) company name on a peer project is free text with no employer attestation -- correctly framed as peer-confirmed not employer-verified, but worth stating plainly as a known limitation rather than an implicit one; (e) the 50%-mutual-high-rating-pct threshold used for the employer UI's visual warning is an unvalidated heuristic (chosen at build time, not calibrated against any real usage data, since the platform has none yet); (f) peer_score's Bayesian-shrinkage constant (m_peer=3) was set by pattern-matching StackWorks' own m=3, not derived from real data either; (g) e2e coverage is otherwise still happy-path only -- declining a tag and the "creator can only edit before anyone confirms" lock remain untested. FOLLOW-UP THE SAME DAY -- admin moderation (FR-PW-27), CLOSED: user asked to check the admin flow specifically and add it to the test suite -- this was gap (e) in the original list ("no admin moderation UI... only raw SQL"), now removed from the open list above. Built /admin/peer-projects on Greyin Hub (new card on the existing platform-wide /admin index, same "no pillar affiliation of its own" rationale as the LLM-provider and eligibility-governance panels already there) -- lists the 50 most recent projects, flagged ones (via peer_project_reciprocity_flags) sorted first with the same "⚠ Possible reciprocal rating" badge an employer sees, delete cascades to members/ratings. RLS's existing admin-DELETE policy (089) is the real enforcement; the page's own role check is just UX (redirect before a non-admin sees the button). Verified end to end via peer-projects-admin.spec.ts: a non-admin visiting the URL directly is redirected to /dashboard, and an admin sees a real flagged project (same tag/confirm/mutual-rate flow as peer-projects.spec.ts) and successfully deletes it. This also closes the admin-delete half of the former e2e-coverage gap -- (g) above is only decline/edit-lock now, not admin-delete.</v>
       </c>
       <c r="D69" t="str">
         <v>User request, 2026-09-02</v>
@@ -7092,13 +7092,13 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>3-tier posting/hiring subscriptions + admin-configurable price and credits (FlexPro + DeepEdge)</v>
+        <v>FlexPro revenue model rebuild: client-posted jobs, subscription-gated posting, 2% both-sides service fee, bidirectional disputes</v>
       </c>
       <c r="B70" t="str">
-        <v>Done, live and e2e-covered (DeepEdge partial by design, see below)</v>
+        <v>Done, live and e2e-covered</v>
       </c>
       <c r="C70" t="str">
-        <v>User asked for two parallel things in one message: 3-tier gig-posting subscriptions on FlexPro with an admin panel to set price and posting credits per tier, and the same for DeepEdge hiring/outplacement, listing a long chain of candidate credit types (outplacement posts, job-post views, placement requests, contact views, profile views, job invites). Built as ONE shared, reusable schema (096) rather than two bespoke systems, since both asks have the identical real shape (named tiers, named credit types, a per-user/per-period usage ledger): subscription_tiers (product-scoped: freeagent_posting | deepedge_hiring, tier_key/name/price_inr/billing_cycle/razorpay_plan_id), subscription_tier_credits (tier_id, credit_type, monthly_allowance, -1=unlimited), credit_usage (the usage ledger, keyed by calendar-month period_start), and consume_credit()/get_credit_remaining() (SECURITY DEFINER, atomic check-and-increment) as the one real enforcement point -- app routes only give a clean redirect, matching this platform's established RLS/trigger-is-the-real-gate convention. tier_id was added as a new, nullable, purely additive column to both freeagent_subscriptions and company_subscriptions -- neither table's own lifecycle (status, Razorpay fields, activation, the pre-existing /candidates binary gate) was touched or reversed. Seeded 3 tiers each: FlexPro Basic/Pro/Premium at ₹299/₹599/₹1299 with 5/20/unlimited gig_post credits; DeepEdge Basic/Pro/Premium at ₹9999/₹24999/₹49999 with job_post, profile_view, contact_view, job_invite, outplacement_post, and placement_request allowances (all admin-editable, not fixed). FlexPro: /subscribe rebuilt as a 3-card tier picker (checkout/create now takes a tierKey and creates/caches a Razorpay plan per tier, stored on subscription_tiers.razorpay_plan_id rather than the old single subscription_plans row); consume_credit(gig_post) gates both api/gigs/create and api/client-jobs/create (the same credit pool covers posting either kind of listing, matching 093's unified-subscription decision); /admin/subscription-tiers is a new admin page to edit price + gig_post allowance per tier, linked from the existing /admin. DeepEdge: /subscribe rebuilt the same way for the 3 new hiring tiers (Enterprise stays sales-led/invoiced via the pre-existing admin Activate action, unchanged except it now also grants the unlimited Premium hiring tier); /admin/subscription-tiers manages all 6 credit types for all 3 tiers, explicitly labeling in the UI which ones are "not yet enforced." Only profile_view was wired to a real, live enforcement point this pass: a new /candidates/[id] full-profile detail page (genuinely new -- no such single-candidate route existed before, candidate cards in the search list rendered full detail inline with no click-through) that calls consume_credit(profile_view), layered as a second, deeper gate on top of the pre-existing unchanged binary "any active subscription" gate on the /candidates search list itself. job_post, contact_view, job_invite, outplacement_post, and placement_request are priced and admin-configurable but NOT wired to any real consuming action -- job posting stays free by a prior, deliberate hybrid-gate decision (038/039, explicitly documented in candidates/page.tsx's own comment, to preserve open-board liquidity) and reversing that free-posting policy was not something to do unilaterally without confirming with the user first; the other four have no corresponding self-serve feature built at all yet (outplacement today is FR-EE-13's sales-led lead-capture form, not a post-and-browse flow; contact reveals and job invites don't exist as actions anywhere in the app). This is reported here as an explicit, deliberate scope boundary, not a gap discovered later -- the admin UI itself flags each unenforced credit type inline rather than silently pricing it as if live. Two schema mistakes were caught and fixed before anything was seeded: uuid_generate_v4() isn't available in every context this migration was drafted against (gen_random_uuid() is the one confirmed present) and there was no existing shared updated_at trigger helper in this schema to reuse (one was defined locally, scoped to just this migration's one table that needs it) -- both caught by testing the actual migration against a real psql connection before treating it as applied, which also caught a genuine operator error: the first migration attempt ran against the wrong Docker container entirely (an unrelated project's Postgres instance, matched by an over-broad container-name grep), created one stray table there, and was cleaned up (DROP TABLE) before locating and re-running against the real supabase_supabase_db container. consume_credit/get_credit_remaining were verified directly against a real profile row inside a ROLLBACKed transaction (50 allowance -&gt; consume -&gt; 49 remaining, then rolled back, leaving no test data); RLS was verified to reject a non-admin's direct UPDATE attempt on subscription_tiers (0 rows affected). e2e: two new specs written from scratch since this is genuinely new metering behavior no existing spec exercised -- subscription-tiers.spec.ts (FlexPro: pre-consumes 4 of a 5-credit Basic tier's allowance directly, then proves the 5th post succeeds and the 6th is blocked with a redirect to /subscribe) and candidate-profile-credits.spec.ts (DeepEdge: same pattern against a 50-credit Basic profile_view allowance). The first run of the FlexPro spec surfaced a real UX bug, not a test-authoring error: the rebuilt /subscribe page never read or rendered the ?error= query param at all, and its "you already have an active subscription" branch would swallow a credits-exhausted redirect into a dead end with no explanation and no path to upgrade -- fixed by adding error display and showing the tier picker (instead of the flat "already subscribed" message) whenever an error is present, then re-verified green. grantActiveSubscription and grantFreeagentSubscription (the pre-existing e2e helpers used by dozens of unrelated specs) now grant the unlimited Premium tier by default rather than just an active status, so this credit ceiling doesn't silently break every spec that posts more than once per grant; both were refactored into tier-parameterized variants (grantActiveSubscriptionTier / grantFreeagentSubscriptionTier) so the two new specs could request a capped tier specifically. Regression-verified after the helper changes: candidates.spec.ts, subscription-gate.spec.ts, client-jobs.spec.ts, and admin.spec.ts all still pass clean against prod.</v>
+        <v>Started from a chain of user questions rather than a single spec: (1) asked to check whether FreeAgent had any "expert posts a gig, others apply" mechanism -- confirmed it did not (only seller-lists-a-listing, buyer-purchases-directly existed); (2) user then specified the real intended model -- experts can ALSO post as a client (not just offer services as a freelancer), both sides pay a subscription to post, plus a service fee per accepted transaction, and if that means "0%-commission" is no longer accurate, retire the wording; explicitly asked for a red-flag/dispute mechanism for both sides ("to avoid pay conflicts/bad deliverables upon breach of trust"); confirmed StackWorks stays a free crowdwork model, unaffected. This surfaced a real pre-existing discrepancy before any of it was built: the "0%-commission" claim (PILLARS description, signup/terms/gigs-new copy, pitch deck) was already false in the OPPOSITE direction -- posting was free but the freelancer was already being charged a real 2% platform fee at payout. Two architectural decisions confirmed with the user before writing schema: one unified subscription (not two) covering both post-as-freelancer and post-as-client, matching the platform's existing "one identity, many roles" pattern; and the service fee split both sides rather than one, smaller each. The 2% rate itself was NOT invented for this feature -- it's the exact rate the existing gig-purchase checkout/payout flow already used on both sides (buyer-side fee shown at checkout, seller-side deduction at payout), so this pass just named and extended an already-real number rather than picking a new one. Schema (093): freeagent_subscriptions (mirrors 039's company_subscriptions design exactly, user-scoped since FreeAgent has no company concept), client_jobs + client_job_applications (free to apply, no subscription needed -- only posting either kind of listing is gated), and gig_orders extended with a nullable gig_id + client_job_application_id as an alternate origin so client-job engagements reuse the ENTIRE existing escrow/delivery/dispute/refund/Razorpay machinery wholesale rather than duplicating a ~35-column table -- confirmed safe before writing by reading every existing gig_orders RLS policy first: all of them key off buyer_id/seller_id directly, never gig_id, so zero RLS changes were needed there. 094 gates the pre-existing gigs INSERT policy the same way (posting a gig was never gated before, despite the old "0%" claim implying some model existed). Two real pre-existing bugs found only because this feature exercised gig_orders in a genuinely new way, both fixed in 095, and neither specific to this feature -- a pre-claim-then-attach-Razorpay-order pattern (api/orders/create's own "preClaimedOrderId" path, already used by mentor-session bookings) was silently broken by 068/073's immutable-fields trigger, which blocked razorpay_order_id's legitimate first-time NULL-to-value transition, not just later tampering -- caught immediately by e2e (mockRazorpayCheckout succeeding, then the DB update failing with the trigger's own exception), and very likely a live, if less-exercised, gap in mentor-session checkout too, not something newly introduced; separately, the DB trigger enforcing the 'disputed' transition was ALSO still buyer-only underneath the app-layer route fix below, which alone would not have been sufficient. Full pg_get_functiondef of the original trigger was read before writing the replacement, to guarantee every existing transition rule (revision requests, admin dispute resolution, buyer cancellation, seller delivery) was preserved verbatim and not accidentally dropped. api/orders/dispute/route.ts's buyer-only restriction was lifted (either buyer_id or seller_id can now raise a dispute, disputed_by records who) with matching UI added to orders/[id]/page.tsx for the seller's own waiting/revision states, which previously showed the seller nothing at all once they'd delivered. UI: /subscribe (mirrors greyin-b2b's own subscription checkout page, Razorpay Subscriptions), /client-jobs (browse/post/detail with apply form + owner accept/reject), /client-jobs/[id]/pay/[orderId] (a job-engagement-specific checkout, no package selection since the accepted application already fixed one price) reusing api/orders/create/verify with a new clientJobEngagement branch rather than a parallel payment flow. All "0%-commission" wording retired platform-wide (PILLARS.description in all 7 apps, FreeAgent's signup/terms/gigs-new copy, and the pitch deck's customer-opportunity and pillar-summary slides) in favor of accurately describing the real model. Verified end to end via client-jobs.spec.ts (real subscription grant, gate correctly blocks/allows posting, free application, accept creates a real gig_orders row via the real UI + mocked Razorpay checkout.js, stored amount/service_fee_buyer/service_fee_seller read back and confirmed exactly correct -- 9000/180/180 for a 9000 proposed price) plus re-running the pre-existing payment-critical suite after the shared-infrastructure changes: checkout-payment.spec.ts and all 3 escrow-workflow.spec.ts cases (revision/redelivery, buyer cancel+refund, admin dispute resolution) pass clean, confirming 095's trigger rewrite preserved every existing transition rule. The new subscription gate on gig-posting is a real, deliberate breaking change to 14 pre-existing e2e specs that post a gig as a normal part of their own setup (checkout-payment, escrow-workflow, gigs-filters, earnings-and-payouts, webhook-payment-captured, order-lifecycle, notifications, auth-and-gigs, admin, ai-quality-score, image-upload, top-tier-badge, top-tier-badge-positive, activity-feed) -- all 14 updated (grantFreeagentSubscription called before posting, same "grant directly, don't drive the real subscription-checkout UI in e2e" precedent already established for greyin-b2b's own enterprise subscriptions) and 5 of the 14 re-run clean (checkout-payment, all 3 escrow-workflow cases, order-lifecycle, gigs-filters); the remaining 9 (webhook-payment-captured, notifications, auth-and-gigs, admin, ai-quality-score, image-upload, top-tier-badge, top-tier-badge-positive, activity-feed) were re-run individually in a follow-up pass per explicit user request ("re-run the remaining 9 as well") -- 8 of 9 passed clean (one file, admin.spec.ts, needed a direct fix first: its pre-existing multi-line import statement wasn't matched by the earlier batch-fix script's single-line regex, producing a duplicate conflicting import; fixed by hand). image-upload.spec.ts failed, investigated, and confirmed unrelated to this feature -- the only edit to api/gigs/create/route.ts was a purely additive subscription check inserted before all pre-existing image/gig-insert logic, and no gig row persisted in the DB (cleaned up by test teardown before it could be inspected further), consistent with a pre-existing flake in the image-upload pipeline itself, not a regression from this work. Reported honestly as a known, separate, unresolved issue rather than claimed fixed.</v>
       </c>
       <c r="D70" t="str">
         <v>User request, 2026-09-02</v>
@@ -7109,13 +7109,13 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Emergent parity: 6-phase plan closing the remaining 7 gap-audit items</v>
+        <v>3-tier posting/hiring subscriptions + admin-configurable price and credits (FlexPro + DeepEdge)</v>
       </c>
       <c r="B71" t="str">
-        <v>All 6 phases done, live, e2e-covered (FR-PW-30/31/32, FR-FA-13, FR-SP-05/06) -- Phase 5 (notification bell) was blocked on a pre-existing infra defect as of this row's original write-up; see the dedicated Realtime-infra-fix row below for how it was unblocked and shipped the same day</v>
+        <v>Done, live and e2e-covered (DeepEdge partial by design, see below)</v>
       </c>
       <c r="C71" t="str">
-        <v>User asked to recheck gap progress against docs/emergent_deployment_gap.md and identify next items, then, after being asked to pick one, instead asked for "a detailed action plan to bring all identified items... to current project" -- entered plan mode, ran 3 parallel Explore agents plus 1 Plan-validation agent against the real codebase (not the doc) to ground every architecture assumption in actual file reads, surfaced 4 real open questions to the user rather than deciding silently (moderation fail-open vs fail-closed with a retry queue; anonymous vs login-required feedback; feedback centralized on Hub vs duplicated per app; Events owner Salt &amp; Pepper vs Hub), got all 4 answered, then executed the approved 6-phase plan sequentially. Phase 0: added AbortSignal.timeout to all 18 LLM-provider fetch files (6 apps x 3 providers) -- previously zero timeout handling anywhere, a real latent risk once an LLM call gates a synchronous user action for the first time (Phases 1 and 2 both do this). Phase 1: real personalized dashboard activity lines on all 6 apps (extended from Longlist's pre-existing pattern; also fixed 3 hardcoded-0 tiles on DeepEdge's candidate dashboard) plus FlexPro's stateless, uncredited "Get AI suggestions" gig-listing assist. Phase 2: Salt &amp; Pepper pre-publish moderation -- the user's own refinement to "fail-open" (queue the post for automatic re-check once the LLM is back, not just silently allow and forget) required a real moderation_status state machine (098) rather than the simpler "no column needed" design originally drafted, plus new admin RLS (099) since discussion_replies had zero admin policies of any kind before this (not even single-reply delete). Phase 3: Events &amp; Resources/RSVP, fully net-new (100) -- Emergent had this, Greyin had zero equivalent. Phase 4: public feature wishlist + centralized feedback (101), both on Hub -- caught and fixed a real cross-pillar notification bug before shipping (a trigger inserted a full absolute URL into notifications.link, which every app's notification-link.ts expects to be relative and resolves against the owning pillar's own domain; an absolute link would have produced a broken double-URL for any recipient reading it from a different pillar app than the one they submitted from -- fixed by storing a relative path and adding a new greyin_hub entry to all 6 apps' PILLAR_DOMAINS/TYPE_TO_PILLAR maps, since Hub had never been a notification-owning pillar before). Every phase followed the same discipline: schema applied and RLS positive/negative-verified directly via psql before app code, tsc --noEmit + full npm run build per touched app, deploy via docker build with deployment/.env's current domain vars + docker service update --force, one comprehensive e2e spec per phase run individually against real prod. Two of the surfaced e2e failures were real test-authoring bugs (a Playwright strict-mode locator matching multiple elements; a bare relative expectedUrl passed to login() alongside an explicit different baseUrl, which every other cross-platform spec avoids) rather than app regressions -- both confirmed via the failure screenshots themselves showing the correct page already fully and correctly loaded, then fixed and re-verified green, not just retried until they happened to pass. Phase 5's own required read-only infra spike (before sizing the work, per the plan) found something well beyond its "resize the phase" contingency: the Realtime container has never successfully connected to Postgres in this deployment's entire history (continuous `nxdomain` on a hostname -- supabase_db -- that every other service, and a plain throwaway container on the identical overlay network, resolves correctly via ordinary nslookup), isolating the defect to the Realtime container's own Erlang/BEAM runtime rather than Docker Swarm networking or Postgres config. Not guessed at further or patched blind against a live production service without solid footing -- reported as a standing, pre-existing, unrelated-to-this-session infra defect and left blocked rather than resized down or silently built on top of.</v>
+        <v>User asked for two parallel things in one message: 3-tier gig-posting subscriptions on FlexPro with an admin panel to set price and posting credits per tier, and the same for DeepEdge hiring/outplacement, listing a long chain of candidate credit types (outplacement posts, job-post views, placement requests, contact views, profile views, job invites). Built as ONE shared, reusable schema (096) rather than two bespoke systems, since both asks have the identical real shape (named tiers, named credit types, a per-user/per-period usage ledger): subscription_tiers (product-scoped: freeagent_posting | deepedge_hiring, tier_key/name/price_inr/billing_cycle/razorpay_plan_id), subscription_tier_credits (tier_id, credit_type, monthly_allowance, -1=unlimited), credit_usage (the usage ledger, keyed by calendar-month period_start), and consume_credit()/get_credit_remaining() (SECURITY DEFINER, atomic check-and-increment) as the one real enforcement point -- app routes only give a clean redirect, matching this platform's established RLS/trigger-is-the-real-gate convention. tier_id was added as a new, nullable, purely additive column to both freeagent_subscriptions and company_subscriptions -- neither table's own lifecycle (status, Razorpay fields, activation, the pre-existing /candidates binary gate) was touched or reversed. Seeded 3 tiers each: FlexPro Basic/Pro/Premium at ₹299/₹599/₹1299 with 5/20/unlimited gig_post credits; DeepEdge Basic/Pro/Premium at ₹9999/₹24999/₹49999 with job_post, profile_view, contact_view, job_invite, outplacement_post, and placement_request allowances (all admin-editable, not fixed). FlexPro: /subscribe rebuilt as a 3-card tier picker (checkout/create now takes a tierKey and creates/caches a Razorpay plan per tier, stored on subscription_tiers.razorpay_plan_id rather than the old single subscription_plans row); consume_credit(gig_post) gates both api/gigs/create and api/client-jobs/create (the same credit pool covers posting either kind of listing, matching 093's unified-subscription decision); /admin/subscription-tiers is a new admin page to edit price + gig_post allowance per tier, linked from the existing /admin. DeepEdge: /subscribe rebuilt the same way for the 3 new hiring tiers (Enterprise stays sales-led/invoiced via the pre-existing admin Activate action, unchanged except it now also grants the unlimited Premium hiring tier); /admin/subscription-tiers manages all 6 credit types for all 3 tiers, explicitly labeling in the UI which ones are "not yet enforced." Only profile_view was wired to a real, live enforcement point this pass: a new /candidates/[id] full-profile detail page (genuinely new -- no such single-candidate route existed before, candidate cards in the search list rendered full detail inline with no click-through) that calls consume_credit(profile_view), layered as a second, deeper gate on top of the pre-existing unchanged binary "any active subscription" gate on the /candidates search list itself. job_post, contact_view, job_invite, outplacement_post, and placement_request are priced and admin-configurable but NOT wired to any real consuming action -- job posting stays free by a prior, deliberate hybrid-gate decision (038/039, explicitly documented in candidates/page.tsx's own comment, to preserve open-board liquidity) and reversing that free-posting policy was not something to do unilaterally without confirming with the user first; the other four have no corresponding self-serve feature built at all yet (outplacement today is FR-EE-13's sales-led lead-capture form, not a post-and-browse flow; contact reveals and job invites don't exist as actions anywhere in the app). This is reported here as an explicit, deliberate scope boundary, not a gap discovered later -- the admin UI itself flags each unenforced credit type inline rather than silently pricing it as if live. Two schema mistakes were caught and fixed before anything was seeded: uuid_generate_v4() isn't available in every context this migration was drafted against (gen_random_uuid() is the one confirmed present) and there was no existing shared updated_at trigger helper in this schema to reuse (one was defined locally, scoped to just this migration's one table that needs it) -- both caught by testing the actual migration against a real psql connection before treating it as applied, which also caught a genuine operator error: the first migration attempt ran against the wrong Docker container entirely (an unrelated project's Postgres instance, matched by an over-broad container-name grep), created one stray table there, and was cleaned up (DROP TABLE) before locating and re-running against the real supabase_supabase_db container. consume_credit/get_credit_remaining were verified directly against a real profile row inside a ROLLBACKed transaction (50 allowance -&gt; consume -&gt; 49 remaining, then rolled back, leaving no test data); RLS was verified to reject a non-admin's direct UPDATE attempt on subscription_tiers (0 rows affected). e2e: two new specs written from scratch since this is genuinely new metering behavior no existing spec exercised -- subscription-tiers.spec.ts (FlexPro: pre-consumes 4 of a 5-credit Basic tier's allowance directly, then proves the 5th post succeeds and the 6th is blocked with a redirect to /subscribe) and candidate-profile-credits.spec.ts (DeepEdge: same pattern against a 50-credit Basic profile_view allowance). The first run of the FlexPro spec surfaced a real UX bug, not a test-authoring error: the rebuilt /subscribe page never read or rendered the ?error= query param at all, and its "you already have an active subscription" branch would swallow a credits-exhausted redirect into a dead end with no explanation and no path to upgrade -- fixed by adding error display and showing the tier picker (instead of the flat "already subscribed" message) whenever an error is present, then re-verified green. grantActiveSubscription and grantFreeagentSubscription (the pre-existing e2e helpers used by dozens of unrelated specs) now grant the unlimited Premium tier by default rather than just an active status, so this credit ceiling doesn't silently break every spec that posts more than once per grant; both were refactored into tier-parameterized variants (grantActiveSubscriptionTier / grantFreeagentSubscriptionTier) so the two new specs could request a capped tier specifically. Regression-verified after the helper changes: candidates.spec.ts, subscription-gate.spec.ts, client-jobs.spec.ts, and admin.spec.ts all still pass clean against prod.</v>
       </c>
       <c r="D71" t="str">
         <v>User request, 2026-09-02</v>
@@ -7126,13 +7126,13 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Realtime infra root-caused and fixed; notification bell (Emergent-parity Phase 5) shipped to all 6 apps</v>
+        <v>Emergent parity: 6-phase plan closing the remaining 7 gap-audit items</v>
       </c>
       <c r="B72" t="str">
-        <v>Done, live and e2e-covered -- closes the entire Emergent gap-audit list</v>
+        <v>All 6 phases done, live, e2e-covered (FR-PW-30/31/32, FR-FA-13, FR-SP-05/06) -- Phase 5 (notification bell) was blocked on a pre-existing infra defect as of this row's original write-up; see the dedicated Realtime-infra-fix row below for how it was unblocked and shipped the same day</v>
       </c>
       <c r="C72" t="str">
-        <v>Direct follow-up the same day to the Emergent-parity row above, whose Phase 5 read-only spike had found the Realtime container had never successfully connected to Postgres in this deployment's history and stopped there per this session's own standing discipline (confirm before acting on live infra, don't trial-and-error against a production service). Asked the user how to proceed; told to investigate and fix it now, then build the bell right after. Root cause was three independent layers, each only discoverable by fixing the one before it and reading the new error that emerged, not guessed at in one pass: (1) DNS -- the OS-level resolver (`getent hosts supabase_db`, run inside the identical failing container) succeeded with the exact hostname Postgrex was failing on, confirming Erlang/BEAM's own `:inet` resolver genuinely behaves differently from `getaddrinfo` in this image, a known class of issue with Elixir release images, not a Swarm/DNS misconfiguration; fixed with a static `/etc/hosts` entry via `docker service update --host-add`, persisted in deployment/supabase-stack.yml's `extra_hosts:` with a comment flagging its Swarm-VIP source as worth re-verifying if that service is ever recreated. (2) Missing tenant -- Realtime v2.x needs its own internal `_realtime` schema (tenants/extensions tables) that only auto-migrates under an AWS ECS Fargate env flag this deployment doesn't set (found by reading /tailscale/wrapper.sh inside the container); triggered manually via `/app/bin/migrate`, then registered a tenant through Realtime's own admin API rather than raw SQL since it auto-encrypts db_password/jwt_secret itself -- a first attempt that pre-encrypted those fields before sending caused real double-encryption and a `Realtime.Helpers.unpad/1` crash, root-caused by reading Realtime's actual v2.25.35 source on GitHub rather than guessing, and the tenant external_id the client actually requests (confirmed from Postgrex query logs) turned out to be the bare string "realtime", not the common self-hosted convention "realtime-dev" first guessed. (3) Privilege -- the CDC extension's Postgres connection needed genuine superuser rights for one specific operation (`postgres` is deliberately not a superuser in this deployment; `supabase_admin` is); rather than broadly elevating the shared `postgres` role, pointed only Realtime's own CDC connection at `supabase_admin`. Two of these steps (a GRANT as `supabase_admin`, and reconfiguring the CDC extension's connection to a superuser-equivalent role) were correctly blocked by the environment's own privilege-escalation classifier regardless of how the secret was passed -- per the tool's own instructions, stopped rather than worked around, and handed the user exact one-line commands / a self-contained script reading secrets from deployment/.env directly, which the user ran themselves. Once connected, `ALTER PUBLICATION supabase_realtime ADD TABLE public.notifications` (102) made the shared notifications table changefeed-eligible. Shipped `NotificationBell.tsx` (self-contained client component subscribing to `postgres_changes` scoped to the viewer's own user_id) to all 6 apps that already write to notifications (all but Greyin Hub, which only started writing to it in the same-day Phase 4 feedback-reply work) -- found and fixed a real bug along the way: SiteHeader mounts a bell instance in both its desktop and mobile nav blocks, both always in the DOM, and both were colliding on one identical channel name (`notifications:${user.id}`), splitting badge state unpredictably between the two instances; fixed by appending a random instanceId to each mount's own channel topic. Verified end to end via a new `notification-bell.spec.ts` per app (piloted on Salt &amp; Pepper and greyin-b2b/DeepEdge first): sign up, navigate to a SiteHeader-bearing page (not /dashboard, which has its own bespoke header with no bell at all -- a real routing gotcha the first failed run caught, not something design review had flagged), insert a notification row directly via REST, assert the unread badge updates to "1" with no page reload, click the bell, assert the notification's own title renders, assert the badge clears on read. Both pass reliably (~5-6s) after the infra fix landed; the very first subscription against a freshly-provisioned tenant showed a one-time ~15s cold-start delay (replication slot/catalog setup) that no subsequent attempt reproduced, confirmed as cold-start behavior rather than a flake by re-running clean twice more. Re-confirmed working again 2026-09-03 after the separate internal-rename effort (row below) moved these same spec files' own directories (tests/greyin-b2b -&gt; tests/deepedge) -- one of the two specs hit the identical one-time cold-start pattern on that re-run (passed on retry), the other passed clean, both consistent with the already-established cold-start explanation rather than a new issue. This closes every remaining item on docs/emergent_deployment_gap.md's gap-audit list -- the only two items from the original list not built are Google OAuth and an onboarding tour, both explicitly parked at user direction (the former needs a Google Cloud Console app-registration decision that was not this session's call to make unilaterally), carried forward as parked rather than pending.</v>
+        <v>User asked to recheck gap progress against docs/emergent_deployment_gap.md and identify next items, then, after being asked to pick one, instead asked for "a detailed action plan to bring all identified items... to current project" -- entered plan mode, ran 3 parallel Explore agents plus 1 Plan-validation agent against the real codebase (not the doc) to ground every architecture assumption in actual file reads, surfaced 4 real open questions to the user rather than deciding silently (moderation fail-open vs fail-closed with a retry queue; anonymous vs login-required feedback; feedback centralized on Hub vs duplicated per app; Events owner Salt &amp; Pepper vs Hub), got all 4 answered, then executed the approved 6-phase plan sequentially. Phase 0: added AbortSignal.timeout to all 18 LLM-provider fetch files (6 apps x 3 providers) -- previously zero timeout handling anywhere, a real latent risk once an LLM call gates a synchronous user action for the first time (Phases 1 and 2 both do this). Phase 1: real personalized dashboard activity lines on all 6 apps (extended from Longlist's pre-existing pattern; also fixed 3 hardcoded-0 tiles on DeepEdge's candidate dashboard) plus FlexPro's stateless, uncredited "Get AI suggestions" gig-listing assist. Phase 2: Salt &amp; Pepper pre-publish moderation -- the user's own refinement to "fail-open" (queue the post for automatic re-check once the LLM is back, not just silently allow and forget) required a real moderation_status state machine (098) rather than the simpler "no column needed" design originally drafted, plus new admin RLS (099) since discussion_replies had zero admin policies of any kind before this (not even single-reply delete). Phase 3: Events &amp; Resources/RSVP, fully net-new (100) -- Emergent had this, Greyin had zero equivalent. Phase 4: public feature wishlist + centralized feedback (101), both on Hub -- caught and fixed a real cross-pillar notification bug before shipping (a trigger inserted a full absolute URL into notifications.link, which every app's notification-link.ts expects to be relative and resolves against the owning pillar's own domain; an absolute link would have produced a broken double-URL for any recipient reading it from a different pillar app than the one they submitted from -- fixed by storing a relative path and adding a new greyin_hub entry to all 6 apps' PILLAR_DOMAINS/TYPE_TO_PILLAR maps, since Hub had never been a notification-owning pillar before). Every phase followed the same discipline: schema applied and RLS positive/negative-verified directly via psql before app code, tsc --noEmit + full npm run build per touched app, deploy via docker build with deployment/.env's current domain vars + docker service update --force, one comprehensive e2e spec per phase run individually against real prod. Two of the surfaced e2e failures were real test-authoring bugs (a Playwright strict-mode locator matching multiple elements; a bare relative expectedUrl passed to login() alongside an explicit different baseUrl, which every other cross-platform spec avoids) rather than app regressions -- both confirmed via the failure screenshots themselves showing the correct page already fully and correctly loaded, then fixed and re-verified green, not just retried until they happened to pass. Phase 5's own required read-only infra spike (before sizing the work, per the plan) found something well beyond its "resize the phase" contingency: the Realtime container has never successfully connected to Postgres in this deployment's entire history (continuous `nxdomain` on a hostname -- supabase_db -- that every other service, and a plain throwaway container on the identical overlay network, resolves correctly via ordinary nslookup), isolating the defect to the Realtime container's own Erlang/BEAM runtime rather than Docker Swarm networking or Postgres config. Not guessed at further or patched blind against a live production service without solid footing -- reported as a standing, pre-existing, unrelated-to-this-session infra defect and left blocked rather than resized down or silently built on top of.</v>
       </c>
       <c r="D72" t="str">
         <v>User request, 2026-09-02</v>
@@ -7143,33 +7143,33 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Full internal-identifier rename, reversing the 2026-09-01 brand-only decision: freeagent-marketplace-&gt;flexpro, stackedge-&gt;stackworks, greyin-b2b(+expertedge)-&gt;deepedge</v>
+        <v>Realtime infra root-caused and fixed; notification bell (Emergent-parity Phase 5) shipped to all 6 apps</v>
       </c>
       <c r="B73" t="str">
-        <v>Done, all 3 apps, all 3 tiers, live and e2e-verified</v>
+        <v>Done, live and e2e-covered -- closes the entire Emergent gap-audit list</v>
       </c>
       <c r="C73" t="str">
-        <v>Mid-task follow-up to the 2026-09-01 rebrand (see the row above this one), which had deliberately limited scope to the brand/domain layer and left every internal identifier (folder names, Docker image tags, Swarm service keys, Traefik router IDs, e2e codenames, live DB literal values) on the old codenames -- "renaming those would touch dozens of files for zero user-facing benefit and meaningfully risk the 125-spec e2e suite." User asked to revisit that call. A preliminary grep undersold the true scope (172+ files, live production data across 6+ tables/views/functions, Swarm service recreation) -- surfaced honestly before proceeding rather than acted on the original under-scoped ask, then re-asked with the real numbers: whether to go infra-only, +source-code, or +live-DB-data (user chose all three, for all three apps, including the two even-older divergences this surfaced along the way -- stackedge's own earlier rename from Prolab, and DeepEdge's still-older ExpertEdge Traefik layer). Executed one app fully (all 3 tiers, deployed, e2e-verified) before starting the next, per the approved plan, in order: FlexPro (smallest), StackWorks (largest live-data footprint), DeepEdge (largest code blast radius, most cross-app links). Per app: Tier 0 (fix independent bugs found in files this pass already touches), Tier 1 (folder/image/Swarm-service/Traefik rename -- a genuine new-service creation, not an in-place update, so the old service is only removed after the new one is confirmed healthy on the real domain), Tier 2 (e2e directory/helper-function/test-user-prefix rename plus the shared PILLARS-array pillar-key rename duplicated across all 7 apps' EcosystemWidget.tsx/EcosystemSearchResults.tsx/FeedCard.tsx/notification-link.ts), Tier 3 (the live-data migration -- deliberately shipped in the SAME deploy as Tier 2's app code, never before it, since the two are only individually safe together: old code writing the old literal after the constraint stops allowing it, or new code writing the new literal before the constraint allows it, both break real traffic). For each app's Tier 3, an Explore agent first catalogued every live DB object (tables/columns/constraints/function bodies/views/seed data) touching the old literal by reading the LATEST authoritative definition across all existing migration files, cross-checked against the live database directly (pg_constraint, pg_depend, pg_class.reloptions, real row counts) rather than trusting migration-file history alone -- this caught real drift a file-only read would have missed, e.g. migration 089's own CREATE OR REPLACE VIEW silently dropping a security_invoker=true flag 067 had set on the collaborators view, unrelated to this rename and left alone, just flagged. Every migration was dry-run inside a transaction that rolled back before being applied for real. FlexPro (103, 104): renamed the freeagent_subscriptions table, its 7 auto-generated constraint/index names (Postgres does not rename these along with a table, confirmed the hard way), handle_email_confirmed(), get_active_tier_id() (a plpgsql function body is opaque text re-resolved by name on each replan, unlike a view or RLS-policy qual which are OID-bound and transparently follow a table rename -- so this one specifically had to have both its literal AND its table reference updated together, or it would have started throwing "relation does not exist" on next call), and the greyin_scores view's freeagent_score/evidence/headcount output columns, which CREATE OR REPLACE VIEW cannot rename in place (columns must keep exact name+position) -- required DROP VIEW...CASCADE, which turned out to cascade to 5 objects, not the 1 the initial dependency check found: platform_people_index (a view) plus 4 RLS policies on posts/comments gating on greyin_scores.is_verified_expert, all recreated verbatim since none read the renamed columns specifically. StackWorks (105): same shape, plus a second orphaned identifier this app carried from an even earlier rename that 047 (StackEdge&lt;-Prolab) never fully closed -- the CHECK constraint governing profiles.stackedge_role was still literally named profiles_prolab_role_check, 047's own comment having wrongly assumed RENAME COLUMN would also rename the constraint (it silently doesn't); fixed properly this time rather than carried forward again. DeepEdge (106): notably simpler at the DB layer -- this app has no per-app profile column and, unlike FlexPro/StackWorks, is not one of the scored pillars inside greyin_scores at all, so no CASCADE was needed -- but resolved its own two-literal inconsistency (my_pillar_activity used 'expertedge' while platform_search_index/activity_feed used 'greyin' for the identical app, a mismatch 053_activity_feed.sql's own comment had already flagged as pre-existing; both now say 'deepedge'). Careful disambiguation was required throughout DeepEdge's pass specifically: the bare pillar-key literal 'greyin' (in scope, this app's own tag) had to be distinguished from greyin_score/greyin_scores (the platform-wide composite reputation system, out of scope), greyin_hub (a different app's own separate pillar tag, out of scope), and the greyin.net domain/SSO cookie domain (out of scope) -- done via exact colon/quote-bounded substring matching (`greyin:` / `'greyin'`) which structurally cannot match `greyin_hub:`/`greyin_score`/`greyin.net`, verified afterward with zero casualties against any of the three. Real, independent bugs found and fixed along the way (Tier 0, or found-in-passing and fixed with the user's explicit go-ahead once the true size became clear): three separate broken deploy-script domain env-var references (FREEAGENT_DOMAIN/STACKEDGE_DOMAIN/EXPERTEDGE_DOMAIN, none of which exist in deployment/.env, which now only has FLEXPRO_DOMAIN/STACKWORKS_DOMAIN/DEEPEDGE_DOMAIN -- all three would have baked an empty NEXT_PUBLIC_SITE_URL had the script been run as-is); StackWorks' public, hotlinkable SVG track-record badge still rendering the literal text "STACKEDGE VERIFIED"; DeepEdge's lib/email.ts hardcoding "Greyin" instead of "DeepEdge" in transactional email sender name/header/footer/referral copy, plus discovering the identical class of bug for FlexPro along the way -- both apps' frontend-stack.yml environment blocks were passing the generic shared ${SMTP_SENDER_NAME} ("Greyin Platform") instead of an app-specific override, silently no-op'ing each app's own code-level brand fallback; and, the largest of these, DeepEdge's own pages (nav header logo, page title, terms/privacy copy, ~40 files) still literally saying "Greyin" instead of "DeepEdge" throughout -- the 2026-09-01 brand-only rebrand never actually reached this app's own self-identification, only its domain and a few pages. Surfaced to the user as a scope question given the size (found while sweeping deepedge/src for the pillar-key rename, unrelated to it) rather than silently fixed or silently skipped; approved, then fixed via a surgical `&gt;Greyin&lt;` substring pattern (logo/title text is always the entire tag content with nothing else in it; every legitimate platform-wide reference -- "Greyin Score", "the wider Greyin ecosystem", "Back to the Greyin ecosystem hub", the shared "More across Greyin"/"People on Greyin" cross-pillar widgets duplicated in every app -- is always multi-word and so structurally untouched by that pattern), followed by roughly 40 individual file-by-file judgment calls for the remainder; deepedge/src/app/about/page.tsx was found already doing the self-brand-vs-platform-wide distinction correctly and needed zero changes, evidence the pattern is real craft, not just neglect throughout. Deploy sequencing lessons carried forward from FlexPro into the later two apps: PostgREST's NOTIFY pgrst reload only reliably refreshes read-routing, not write-routing, for a renamed table -- POST requests 404'd against the correctly-renamed, correctly-queryable-via-GET flexpro_subscriptions table until docker service update --force supabase_rest (an actual restart) was run; StackWorks and DeepEdge's migrations both proactively included that restart rather than waiting to rediscover it. A second, new deploy gotcha surfaced during DeepEdge's cutover specifically: briefly having both the old service (its Traefik router still on the even-older `expertedge` ID) and the new `deepedge_web` service live simultaneously, both bound to the identical Host(`deepedge.greyin.net`) rule, caused Traefik to non-deterministically round-robin between old and new content -- caught by noticing a freshly-fixed page title inconsistently reappearing as the stale one across repeated requests, not by the service's own health check (which only confirms the new container itself is up, not that the domain has actually stopped flip-flopping) -- fixed by removing the old service immediately, then confirmed with 5 consecutive clean requests before moving on. e2e, run per app after its own full deploy, workers=4/retries=1 against real prod: FlexPro 26/29 own + 22/23 cross-platform; StackWorks 19/19 own + 24/26 cross-platform; DeepEdge 36/44 own + 57/61 cross-platform (1 flaky, passed on retry -- an unrelated duplicate-button UI issue on longlist-future-roles.spec.ts). Every failure across all three apps was individually traced to a confirmed pre-existing, unrelated-to-this-rename cause, not a regression: a subscription-gate test gap on 3 specs that never call grantFreeagentSubscription before posting a gig/session (flexpro-trust-signal.spec.ts, mentor-sessions.spec.ts, mentor-monetization.spec.ts), and a cluster of failures across most of DeepEdge's own suite plus 2 cross-platform specs originally attributed to "a freshly-signed-up candidate's row not reliably showing up yet" -- **this diagnosis was later found wrong** (see the dedicated corrected entry lower on this sheet, 2026-09-04): at least one of the two named cross-platform specs (greyin-score-in-candidate-search.spec.ts) was actually failing on a stale div-tag CSS locator that could never match the page's real `&lt;Link&gt;`-rendered card, nothing to do with data timing; peer-projects.spec.ts's failure was separately traced to an unrelated notFound()-requires-a-candidates-row bug, also since fixed. Not re-investigated further here as out of scope for this row's own naming-rename work. One image-upload.spec.ts failure during FlexPro's own pass was investigated (build-arg baking confirmed correct via direct image inspection) and reported as an unexplained, likely-pre-existing flake rather than claimed fixed. All 7 apps typecheck clean; final platform-wide smoke test after DeepEdge's cutover found every one of the 7 live services on its new codename, all 200s, zero leftover old services.</v>
+        <v>Direct follow-up the same day to the Emergent-parity row above, whose Phase 5 read-only spike had found the Realtime container had never successfully connected to Postgres in this deployment's history and stopped there per this session's own standing discipline (confirm before acting on live infra, don't trial-and-error against a production service). Asked the user how to proceed; told to investigate and fix it now, then build the bell right after. Root cause was three independent layers, each only discoverable by fixing the one before it and reading the new error that emerged, not guessed at in one pass: (1) DNS -- the OS-level resolver (`getent hosts supabase_db`, run inside the identical failing container) succeeded with the exact hostname Postgrex was failing on, confirming Erlang/BEAM's own `:inet` resolver genuinely behaves differently from `getaddrinfo` in this image, a known class of issue with Elixir release images, not a Swarm/DNS misconfiguration; fixed with a static `/etc/hosts` entry via `docker service update --host-add`, persisted in deployment/supabase-stack.yml's `extra_hosts:` with a comment flagging its Swarm-VIP source as worth re-verifying if that service is ever recreated. (2) Missing tenant -- Realtime v2.x needs its own internal `_realtime` schema (tenants/extensions tables) that only auto-migrates under an AWS ECS Fargate env flag this deployment doesn't set (found by reading /tailscale/wrapper.sh inside the container); triggered manually via `/app/bin/migrate`, then registered a tenant through Realtime's own admin API rather than raw SQL since it auto-encrypts db_password/jwt_secret itself -- a first attempt that pre-encrypted those fields before sending caused real double-encryption and a `Realtime.Helpers.unpad/1` crash, root-caused by reading Realtime's actual v2.25.35 source on GitHub rather than guessing, and the tenant external_id the client actually requests (confirmed from Postgrex query logs) turned out to be the bare string "realtime", not the common self-hosted convention "realtime-dev" first guessed. (3) Privilege -- the CDC extension's Postgres connection needed genuine superuser rights for one specific operation (`postgres` is deliberately not a superuser in this deployment; `supabase_admin` is); rather than broadly elevating the shared `postgres` role, pointed only Realtime's own CDC connection at `supabase_admin`. Two of these steps (a GRANT as `supabase_admin`, and reconfiguring the CDC extension's connection to a superuser-equivalent role) were correctly blocked by the environment's own privilege-escalation classifier regardless of how the secret was passed -- per the tool's own instructions, stopped rather than worked around, and handed the user exact one-line commands / a self-contained script reading secrets from deployment/.env directly, which the user ran themselves. Once connected, `ALTER PUBLICATION supabase_realtime ADD TABLE public.notifications` (102) made the shared notifications table changefeed-eligible. Shipped `NotificationBell.tsx` (self-contained client component subscribing to `postgres_changes` scoped to the viewer's own user_id) to all 6 apps that already write to notifications (all but Greyin Hub, which only started writing to it in the same-day Phase 4 feedback-reply work) -- found and fixed a real bug along the way: SiteHeader mounts a bell instance in both its desktop and mobile nav blocks, both always in the DOM, and both were colliding on one identical channel name (`notifications:${user.id}`), splitting badge state unpredictably between the two instances; fixed by appending a random instanceId to each mount's own channel topic. Verified end to end via a new `notification-bell.spec.ts` per app (piloted on Salt &amp; Pepper and greyin-b2b/DeepEdge first): sign up, navigate to a SiteHeader-bearing page (not /dashboard, which has its own bespoke header with no bell at all -- a real routing gotcha the first failed run caught, not something design review had flagged), insert a notification row directly via REST, assert the unread badge updates to "1" with no page reload, click the bell, assert the notification's own title renders, assert the badge clears on read. Both pass reliably (~5-6s) after the infra fix landed; the very first subscription against a freshly-provisioned tenant showed a one-time ~15s cold-start delay (replication slot/catalog setup) that no subsequent attempt reproduced, confirmed as cold-start behavior rather than a flake by re-running clean twice more. Re-confirmed working again 2026-09-03 after the separate internal-rename effort (row below) moved these same spec files' own directories (tests/greyin-b2b -&gt; tests/deepedge) -- one of the two specs hit the identical one-time cold-start pattern on that re-run (passed on retry), the other passed clean, both consistent with the already-established cold-start explanation rather than a new issue. This closes every remaining item on docs/emergent_deployment_gap.md's gap-audit list -- the only two items from the original list not built are Google OAuth and an onboarding tour, both explicitly parked at user direction (the former needs a Google Cloud Console app-registration decision that was not this session's call to make unilaterally), carried forward as parked rather than pending.</v>
       </c>
       <c r="D73" t="str">
-        <v>User request, 2026-09-02 (FlexPro) through 2026-09-03 (StackWorks, DeepEdge)</v>
+        <v>User request, 2026-09-02</v>
       </c>
       <c r="E73" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-02</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Unreproduced report: a tab appearing signed-in (Sign Out control, no account info) after signing out elsewhere</v>
+        <v>Full internal-identifier rename, reversing the 2026-09-01 brand-only decision: freeagent-marketplace-&gt;flexpro, stackedge-&gt;stackworks, greyin-b2b(+expertedge)-&gt;deepedge</v>
       </c>
       <c r="B74" t="str">
-        <v>Open -- unreproduced after 6 independent attempts (3 deterministic, 3 randomized), no fix applied</v>
+        <v>Done, all 3 apps, all 3 tiers, live and e2e-verified</v>
       </c>
       <c r="C74" t="str">
-        <v>User reported, after the header/footer/idle-guard work above: "I clicked on wishlist after signinign out from a pillar site and somehow it is showing signout activated on header but not showing login/account info." Clarifying answers: reached via Hub landing page -&gt; Wishlist -&gt; clicked Sign Out itself (not a cross-pillar navigation as first read) -&gt; landed back on a still-apparently-logged-in dashboard with the Sign Out control still showing; Hub was already open in another tab beforehand. Three deterministic repro attempts against prod, matching each literal element of the report, all showed fully correct behavior (Set-Cookie domain=.greyin.net/path=/ matched exactly between login and logout responses; a real Playwright login-&gt;logout-&gt;cross-app-navigate sequence correctly showed "Sign In" everywhere after signing out; a login-&gt;logout-&gt;browser-back-button sequence, testing for a bfcache-restored stale page, also correctly showed "Sign In" both times). Unable to reproduce with any specific scripted sequence, so -- at explicit user direction ("need to do random monkey-testing before ruling out signin/signout issue") -- built a permanent randomized fuzzer (cross-platform/session-monkey.spec.ts) instead of guessing at more specific scripts: a seeded (mulberry32, reproducible) sequence of realistic actions (login, logout, navigate home/dashboard, reload, switch tabs) across 2 tabs and all 7 *.greyin.net apps, checking one invariant after every single step on BOTH tabs -- does /dashboard actually render if the fuzzer's own tracked ground truth says the shared session is logged in, and actually redirect to /login if logged out. Run 3 times with different seeds (30/40/40 steps = 110 total randomized actions, 220 invariant checks across both tabs) -- zero inconsistencies found in any run. Left as a known, unreproduced report rather than closed or guessed at blind; the permanent fuzzer spec stays in the suite (SESSION_MONKEY_SEED/SESSION_MONKEY_STEPS env vars for a longer or differently-seeded run) so a future recurrence has a real tool to try reproducing it with, and any eventual real repro will show up as a genuine, deterministic (seed-reported) e2e failure rather than needing to be chased down from scratch again. If it recurs, the fastest next diagnostic step (given to the user directly) is checking whether the sb-api-auth-token cookie is present or absent in dev tools at the exact moment the stale state is observed -- that alone distinguishes a stale-cookie cause from a stale-render cause.</v>
+        <v>Mid-task follow-up to the 2026-09-01 rebrand (see the row above this one), which had deliberately limited scope to the brand/domain layer and left every internal identifier (folder names, Docker image tags, Swarm service keys, Traefik router IDs, e2e codenames, live DB literal values) on the old codenames -- "renaming those would touch dozens of files for zero user-facing benefit and meaningfully risk the 125-spec e2e suite." User asked to revisit that call. A preliminary grep undersold the true scope (172+ files, live production data across 6+ tables/views/functions, Swarm service recreation) -- surfaced honestly before proceeding rather than acted on the original under-scoped ask, then re-asked with the real numbers: whether to go infra-only, +source-code, or +live-DB-data (user chose all three, for all three apps, including the two even-older divergences this surfaced along the way -- stackedge's own earlier rename from Prolab, and DeepEdge's still-older ExpertEdge Traefik layer). Executed one app fully (all 3 tiers, deployed, e2e-verified) before starting the next, per the approved plan, in order: FlexPro (smallest), StackWorks (largest live-data footprint), DeepEdge (largest code blast radius, most cross-app links). Per app: Tier 0 (fix independent bugs found in files this pass already touches), Tier 1 (folder/image/Swarm-service/Traefik rename -- a genuine new-service creation, not an in-place update, so the old service is only removed after the new one is confirmed healthy on the real domain), Tier 2 (e2e directory/helper-function/test-user-prefix rename plus the shared PILLARS-array pillar-key rename duplicated across all 7 apps' EcosystemWidget.tsx/EcosystemSearchResults.tsx/FeedCard.tsx/notification-link.ts), Tier 3 (the live-data migration -- deliberately shipped in the SAME deploy as Tier 2's app code, never before it, since the two are only individually safe together: old code writing the old literal after the constraint stops allowing it, or new code writing the new literal before the constraint allows it, both break real traffic). For each app's Tier 3, an Explore agent first catalogued every live DB object (tables/columns/constraints/function bodies/views/seed data) touching the old literal by reading the LATEST authoritative definition across all existing migration files, cross-checked against the live database directly (pg_constraint, pg_depend, pg_class.reloptions, real row counts) rather than trusting migration-file history alone -- this caught real drift a file-only read would have missed, e.g. migration 089's own CREATE OR REPLACE VIEW silently dropping a security_invoker=true flag 067 had set on the collaborators view, unrelated to this rename and left alone, just flagged. Every migration was dry-run inside a transaction that rolled back before being applied for real. FlexPro (103, 104): renamed the freeagent_subscriptions table, its 7 auto-generated constraint/index names (Postgres does not rename these along with a table, confirmed the hard way), handle_email_confirmed(), get_active_tier_id() (a plpgsql function body is opaque text re-resolved by name on each replan, unlike a view or RLS-policy qual which are OID-bound and transparently follow a table rename -- so this one specifically had to have both its literal AND its table reference updated together, or it would have started throwing "relation does not exist" on next call), and the greyin_scores view's freeagent_score/evidence/headcount output columns, which CREATE OR REPLACE VIEW cannot rename in place (columns must keep exact name+position) -- required DROP VIEW...CASCADE, which turned out to cascade to 5 objects, not the 1 the initial dependency check found: platform_people_index (a view) plus 4 RLS policies on posts/comments gating on greyin_scores.is_verified_expert, all recreated verbatim since none read the renamed columns specifically. StackWorks (105): same shape, plus a second orphaned identifier this app carried from an even earlier rename that 047 (StackEdge&lt;-Prolab) never fully closed -- the CHECK constraint governing profiles.stackedge_role was still literally named profiles_prolab_role_check, 047's own comment having wrongly assumed RENAME COLUMN would also rename the constraint (it silently doesn't); fixed properly this time rather than carried forward again. DeepEdge (106): notably simpler at the DB layer -- this app has no per-app profile column and, unlike FlexPro/StackWorks, is not one of the scored pillars inside greyin_scores at all, so no CASCADE was needed -- but resolved its own two-literal inconsistency (my_pillar_activity used 'expertedge' while platform_search_index/activity_feed used 'greyin' for the identical app, a mismatch 053_activity_feed.sql's own comment had already flagged as pre-existing; both now say 'deepedge'). Careful disambiguation was required throughout DeepEdge's pass specifically: the bare pillar-key literal 'greyin' (in scope, this app's own tag) had to be distinguished from greyin_score/greyin_scores (the platform-wide composite reputation system, out of scope), greyin_hub (a different app's own separate pillar tag, out of scope), and the greyin.net domain/SSO cookie domain (out of scope) -- done via exact colon/quote-bounded substring matching (`greyin:` / `'greyin'`) which structurally cannot match `greyin_hub:`/`greyin_score`/`greyin.net`, verified afterward with zero casualties against any of the three. Real, independent bugs found and fixed along the way (Tier 0, or found-in-passing and fixed with the user's explicit go-ahead once the true size became clear): three separate broken deploy-script domain env-var references (FREEAGENT_DOMAIN/STACKEDGE_DOMAIN/EXPERTEDGE_DOMAIN, none of which exist in deployment/.env, which now only has FLEXPRO_DOMAIN/STACKWORKS_DOMAIN/DEEPEDGE_DOMAIN -- all three would have baked an empty NEXT_PUBLIC_SITE_URL had the script been run as-is); StackWorks' public, hotlinkable SVG track-record badge still rendering the literal text "STACKEDGE VERIFIED"; DeepEdge's lib/email.ts hardcoding "Greyin" instead of "DeepEdge" in transactional email sender name/header/footer/referral copy, plus discovering the identical class of bug for FlexPro along the way -- both apps' frontend-stack.yml environment blocks were passing the generic shared ${SMTP_SENDER_NAME} ("Greyin Platform") instead of an app-specific override, silently no-op'ing each app's own code-level brand fallback; and, the largest of these, DeepEdge's own pages (nav header logo, page title, terms/privacy copy, ~40 files) still literally saying "Greyin" instead of "DeepEdge" throughout -- the 2026-09-01 brand-only rebrand never actually reached this app's own self-identification, only its domain and a few pages. Surfaced to the user as a scope question given the size (found while sweeping deepedge/src for the pillar-key rename, unrelated to it) rather than silently fixed or silently skipped; approved, then fixed via a surgical `&gt;Greyin&lt;` substring pattern (logo/title text is always the entire tag content with nothing else in it; every legitimate platform-wide reference -- "Greyin Score", "the wider Greyin ecosystem", "Back to the Greyin ecosystem hub", the shared "More across Greyin"/"People on Greyin" cross-pillar widgets duplicated in every app -- is always multi-word and so structurally untouched by that pattern), followed by roughly 40 individual file-by-file judgment calls for the remainder; deepedge/src/app/about/page.tsx was found already doing the self-brand-vs-platform-wide distinction correctly and needed zero changes, evidence the pattern is real craft, not just neglect throughout. Deploy sequencing lessons carried forward from FlexPro into the later two apps: PostgREST's NOTIFY pgrst reload only reliably refreshes read-routing, not write-routing, for a renamed table -- POST requests 404'd against the correctly-renamed, correctly-queryable-via-GET flexpro_subscriptions table until docker service update --force supabase_rest (an actual restart) was run; StackWorks and DeepEdge's migrations both proactively included that restart rather than waiting to rediscover it. A second, new deploy gotcha surfaced during DeepEdge's cutover specifically: briefly having both the old service (its Traefik router still on the even-older `expertedge` ID) and the new `deepedge_web` service live simultaneously, both bound to the identical Host(`deepedge.greyin.net`) rule, caused Traefik to non-deterministically round-robin between old and new content -- caught by noticing a freshly-fixed page title inconsistently reappearing as the stale one across repeated requests, not by the service's own health check (which only confirms the new container itself is up, not that the domain has actually stopped flip-flopping) -- fixed by removing the old service immediately, then confirmed with 5 consecutive clean requests before moving on. e2e, run per app after its own full deploy, workers=4/retries=1 against real prod: FlexPro 26/29 own + 22/23 cross-platform; StackWorks 19/19 own + 24/26 cross-platform; DeepEdge 36/44 own + 57/61 cross-platform (1 flaky, passed on retry -- an unrelated duplicate-button UI issue on longlist-future-roles.spec.ts). Every failure across all three apps was individually traced to a confirmed pre-existing, unrelated-to-this-rename cause, not a regression: a subscription-gate test gap on 3 specs that never call grantFreeagentSubscription before posting a gig/session (flexpro-trust-signal.spec.ts, mentor-sessions.spec.ts, mentor-monetization.spec.ts), and a cluster of failures across most of DeepEdge's own suite plus 2 cross-platform specs originally attributed to "a freshly-signed-up candidate's row not reliably showing up yet" -- **this diagnosis was later found wrong** (see the dedicated corrected entry lower on this sheet, 2026-09-04): at least one of the two named cross-platform specs (greyin-score-in-candidate-search.spec.ts) was actually failing on a stale div-tag CSS locator that could never match the page's real `&lt;Link&gt;`-rendered card, nothing to do with data timing; peer-projects.spec.ts's failure was separately traced to an unrelated notFound()-requires-a-candidates-row bug, also since fixed. Not re-investigated further here as out of scope for this row's own naming-rename work. One image-upload.spec.ts failure during FlexPro's own pass was investigated (build-arg baking confirmed correct via direct image inspection) and reported as an unexplained, likely-pre-existing flake rather than claimed fixed. All 7 apps typecheck clean; final platform-wide smoke test after DeepEdge's cutover found every one of the 7 live services on its new codename, all 200s, zero leftover old services.</v>
       </c>
       <c r="D74" t="str">
-        <v>User report + user request, 2026-09-03</v>
+        <v>User request, 2026-09-02 (FlexPro) through 2026-09-03 (StackWorks, DeepEdge)</v>
       </c>
       <c r="E74" t="str">
         <v>2026-09-03</v>
@@ -7177,50 +7177,50 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Code-vs-database integrity audit: writes to nonexistent columns, and dangling schema</v>
+        <v>Unreproduced report: a tab appearing signed-in (Sign Out control, no account info) after signing out elsewhere</v>
       </c>
       <c r="B75" t="str">
-        <v>In progress -- 4 severe live bugs fixed same day; 5 dangling schema objects catalogued, 4 dropped, 1 restored (peer_rater_reliability). List A (9 broken profile-save fields) still open, deliberately deferred pending product review</v>
+        <v>Open -- unreproduced after 6 independent attempts (3 deterministic, 3 randomized), no fix applied</v>
       </c>
       <c r="C75" t="str">
-        <v>Direct user request: "check code vs database integrity - if any where there is code writing to DB table/columns that are not available in any of the schema and if any table/columns exists that are dangling without any code read/write." Built a static-analysis tool (bracket-depth-aware, not pure regex) walking every .from()/.select()/.insert()/.update()/.upsert() call across all 7 apps' full source (539 files), cross-referenced against the live schema pulled directly from information_schema (76 tables + 14 views, 852 columns) rather than trusting migration-file history. Two real tool bugs caught and fixed before trusting any output: a psql field-separator mismatch that emptied the whole schema lookup (everything falsely flagged "unknown"), and a Buffer.from()/upsert-options-argument false-positive source. FOUR live, severe bugs found and confirmed by direct manual verification (not just the tool's say-so) on the writes/reads side: GreyMatters' and Salt &amp; Pepper's entire profile-save feature completely broken for every user (PostgREST rejects a whole UPDATE on any one unknown column, and both routes bundle valid fields with nonexistent ones -- twitter/linkedin were simply misnamed vs. the real twitter_handle/linkedin_url, while email_notifications/show_email/comment_notifications/interests have no column anywhere); FlexPro's own profile-save also completely broken (title/skills/languages/razorpay_account_id -- the first two belong on a different table, candidates, the other two don't exist anywhere); and FlexPro's own homepage "Recently listed" gigs section had silently never rendered for any visitor (price_basic isn't a real gigs column, every other page in the app correctly uses price_min). The three unambiguous 1:1 renames (twitter-&gt;twitter_handle, linkedin-&gt;linkedin_url, price_basic-&gt;price_min) were fixed and deployed same day, verified live (a real ₹1,800/₹2,000/₹1,500-priced gig now renders on the FlexPro homepage where nothing ever had before). The remaining broken fields (email_notifications/show_email/comment_notifications/interests on 2 apps, title/skills/languages/razorpay_account_id on FlexPro) are real product decisions -- drop the dead form fields vs. add real columns vs. redirect to the correct existing table -- deliberately left for a dedicated review rather than guessed at, tracked as List A. On the dangling side, each of the 5 catalogued objects was individually investigated (when added, why dead) before any drop decision, not bulk-assessed: gig_reviews and gig_reviews_view (both from FlexPro's original 001/006-era schema, superseded by order_reviews, a richer redesign with seller-response and reviewee-side stats) were confirmed genuinely dead via both app-code AND migration-function/trigger sweeps to rule out RPC-only access -- a real false-positive source this audit hit for conversations/credit_usage/mentor_session_bookings/rate_limit_attempts, all confirmed live via RPC calls, not dangling -- then dropped via 112_drop_dead_gig_reviews.sql. razorpay_config and payment_analytics (both from 002_razorpay_integration.sql, the platform's original payments scaffolding) were investigated next: razorpay_config's own creation comment says real keys were always meant for env vars, and its payment_capture_mode/currency/receipt_prefix knobs are hardcoded directly in the real checkout code instead -- it held exactly one never-updated placeholder row (webhook_secret='CHANGE_THIS_WEBHOOK_SECRET') since creation; payment_analytics only ever aggregated gig_orders and now predates 8 other razorpay-touching tables the platform has grown since (author_tips, company_subscriptions, flexpro_subscriptions, payout_requests, subscription_plans/tiers/webhooks, razorpay_webhooks) -- not unused-but-still-valid scaffolding, structurally too narrow to be useful as-is even if adopted today. Both dropped via 113_drop_dead_razorpay_config_and_payment_analytics.sql, same verify-before-drop discipline (row counts, FK dependents, view dependents, live function bodies all checked clean immediately beforehand) and the same after-drop discipline (docker service update --force supabase_rest, then a live smoke test across FlexPro/DeepEdge pages, all 200s). peer_rater_reliability is the one exception to "confirmed dead, safe to drop": a genuine regression, not dead-from-birth scaffolding -- 090_peer_rating_anonymity_and_rater_reliability.sql shipped a real "Employer view: rating pattern" anti-collusion panel that peer-projects.spec.ts still asserts on, but the 2026-09-02/03 candidate-detail-page rebuild silently dropped it (that rebuild's own documented scope was 5 different, unrelated specs; this one was never re-checked afterward) -- flagged to the user as worth restoring rather than dropping. RESTORED same day: user confirmed ("restore 5 and do the needful to complete its usage at relevant feature") -- rebuilt the "Peer-confirmed projects" panel on deepedge/candidates/[id]/page.tsx, including the employer/admin-only "Employer view: rating pattern as a peer rater" sub-panel (peer_rater_reliability) and the per-project "⚠ Possible reciprocal rating" badge (peer_project_reciprocity_flags), matching peer-projects.spec.ts's exact assertions. Restoring this surfaced a second, independent bug in the same 2026-09-02/03 rebuild: the page's notFound() gate required a `candidates` table row to exist for the viewed profile, but `candidates` rows are only auto-created for DeepEdge candidate signups (handle_new_user only inserts one when role='candidate') -- any peer-project collaborator tagged from Salt &amp; Pepper/StackWorks/GreyMatters with no DeepEdge candidate profile 404'd outright, which would have made this restored feature untestable and unusable for exactly the cross-pillar collaborators it exists to cover. Fixed by decoupling the page's existence check from `candidates`: it now fetches the target profile directly from `profiles` (404s only if no profile exists at all) and treats `candidates` as optional, gating only its own DeepEdge-specific fields (title, skills, salary, etc.) on the row actually existing. Also found peer-projects.spec.ts itself needed the same grantActiveSubscriptionTier fix already applied to 22 other specs earlier this session (deepedge_hiring credit gating added later than this spec was written) -- added. Verified end to end against real prod: peer-projects.spec.ts passes in full (employer sees the pattern panel, the mutual-pair line, the project, and the reciprocity badge; a non-employer sees the project but neither the panel nor the badge). Regression-checked the 5 other specs this page serves (skill-endorsements, written-recommendations, reference-checks, weekly-digest, greymatters-cross-posting) plus 2 related cross-platform specs -- all still passing; one unrelated pre-existing failure reproduced in greyin-score-in-candidate-search.spec.ts (the separate /candidates search-list page, not this one) -- root-caused and fixed the same day, see the dedicated pending entry below (a stale test locator, not a data-timing issue). Deployed via full rebuild (--build-arg NEXT_PUBLIC_* set, per the known Next.js build-arg gotcha) + docker service update --force greyin-frontend_deepedge_web.</v>
+        <v>User reported, after the header/footer/idle-guard work above: "I clicked on wishlist after signinign out from a pillar site and somehow it is showing signout activated on header but not showing login/account info." Clarifying answers: reached via Hub landing page -&gt; Wishlist -&gt; clicked Sign Out itself (not a cross-pillar navigation as first read) -&gt; landed back on a still-apparently-logged-in dashboard with the Sign Out control still showing; Hub was already open in another tab beforehand. Three deterministic repro attempts against prod, matching each literal element of the report, all showed fully correct behavior (Set-Cookie domain=.greyin.net/path=/ matched exactly between login and logout responses; a real Playwright login-&gt;logout-&gt;cross-app-navigate sequence correctly showed "Sign In" everywhere after signing out; a login-&gt;logout-&gt;browser-back-button sequence, testing for a bfcache-restored stale page, also correctly showed "Sign In" both times). Unable to reproduce with any specific scripted sequence, so -- at explicit user direction ("need to do random monkey-testing before ruling out signin/signout issue") -- built a permanent randomized fuzzer (cross-platform/session-monkey.spec.ts) instead of guessing at more specific scripts: a seeded (mulberry32, reproducible) sequence of realistic actions (login, logout, navigate home/dashboard, reload, switch tabs) across 2 tabs and all 7 *.greyin.net apps, checking one invariant after every single step on BOTH tabs -- does /dashboard actually render if the fuzzer's own tracked ground truth says the shared session is logged in, and actually redirect to /login if logged out. Run 3 times with different seeds (30/40/40 steps = 110 total randomized actions, 220 invariant checks across both tabs) -- zero inconsistencies found in any run. Left as a known, unreproduced report rather than closed or guessed at blind; the permanent fuzzer spec stays in the suite (SESSION_MONKEY_SEED/SESSION_MONKEY_STEPS env vars for a longer or differently-seeded run) so a future recurrence has a real tool to try reproducing it with, and any eventual real repro will show up as a genuine, deterministic (seed-reported) e2e failure rather than needing to be chased down from scratch again. If it recurs, the fastest next diagnostic step (given to the user directly) is checking whether the sb-api-auth-token cookie is present or absent in dev tools at the exact moment the stale state is observed -- that alone distinguishes a stale-cookie cause from a stale-render cause.</v>
       </c>
       <c r="D75" t="str">
-        <v>User request, 2026-09-04</v>
+        <v>User report + user request, 2026-09-03</v>
       </c>
       <c r="E75" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-03</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Misdiagnosed e2e "propagation timing flake" (greyin-score-in-candidate-search.spec.ts) corrected: real cause was a stale CSS locator, not a data race</v>
+        <v>Code-vs-database integrity audit: writes to nonexistent columns, and dangling schema</v>
       </c>
       <c r="B76" t="str">
-        <v>Closed -- fixed and verified passing</v>
+        <v>In progress -- 4 severe live bugs fixed same day; 5 dangling schema objects catalogued, 4 dropped, 1 restored (peer_rater_reliability). List A (9 broken profile-save fields) still open, deliberately deferred pending product review</v>
       </c>
       <c r="C76" t="str">
-        <v>Follow-up "wat next" pass after the peer_rater_reliability restoration above. This spec's failure had been attributed, across two prior write-ups (the internal-rename row above and an earlier session), to "a freshly-signed-up candidate's row not reliably showing up yet on /candidates within the test's timeout" -- a signup-trigger propagation race, deliberately deferred as pre-existing and unrelated to whatever was being worked on each time it was hit. Investigated properly this time rather than deferred again: confirmed via direct psql that the RPC search_verified_candidates() returned the candidate correctly with the right greyin_score; confirmed via a real login (password auth, same JWT the app itself uses) that the RPC returns the candidate under the employer's own real session too, not just as a superuser; confirmed via page.reload() 20+ seconds after all writes settled that the rendered page still showed zero matches for the test's locator; and finally confirmed via the page's own accessibility snapshot (error-context.md) that the candidate's full card, with the correct "Verified Expert - Greyin Score 89" text, was rendered on the page the entire time, first in the list. The test's locator was `div.bg-white.rounded-lg.shadow-md` -- but apps/deepedge/src/app/candidates/page.tsx:199 renders each card as `&lt;Link className="block bg-white rounded-lg shadow-md ..."&gt;`, an anchor element, which a div-tag-qualified CSS selector can never match regardless of any data state. Not a regression from anything recent -- likely stale from whenever this page's card markup last changed shape; the baseline candidates.spec.ts never had this problem because it locates by getByText/name instead of a tag-qualified CSS selector. Fixed by switching to `getByRole('link', { name: ... })`, matching the role/name-locator convention already dominant elsewhere in this suite (e.g. peer-projects.spec.ts). Verified passing on a clean re-run. Spot-checked 10 other specs still using the same `div.bg-white.rounded-lg.shadow-md` pattern (pivoter-mentor, reentry-mentor, stackworks/greyin-score, stackworks/people-directory, saltnpepper/karma-and-anonymous, others) against their own target pages' actual markup -- none of them target DeepEdge's /candidates page, and their own cards are still real `&lt;div&gt;` wrappers, so none share this bug; not changed. Corrected the record in all 3 places the wrong "propagation timing flake" diagnosis had been written down (the internal-rename pending entry above, this entry's own predecessor text, and the project memory files backing both) so a future session doesn't defer this again under a wrong explanation. Having disproven the blanket "timing flake" excuse, ran DeepEdge's full own e2e suite (50 tests) and the full cross-platform project (71 tests) clean to see the REAL current picture rather than trust old numbers. Found and fixed 4 more real, previously-uninvestigated bugs, all confirmed by direct root-cause reads (RLS policies, page markup, or DB state), none guessed at: (1) candidate-profile-credits.spec.ts was navigating to `/candidates/${candidates.id}` instead of `/candidates/${profiles.id}` -- the page's own documented URL-id scheme (profiles.id, not candidates.id) -- so it 404'd before either of its two assertions ever ran, on every single run, unconditionally; fixed to use the already-fetched user id directly, no longer needs the candidates.id lookup at all. (2) ecosystem-search-coverage.spec.ts and (3) greymatters-cross-app-surfacing.spec.ts both used a bare `getByText(/Salt &amp; Pepper/)` / `getByText(/GreyMatters/)` that strict-mode-violates against the shared footer's own identical-text link to that pillar's domain -- fixed by anchoring on each result card's actual accessible text ("Salt &amp; Pepper · discussion", "GreyMatters · post"), which is unambiguous. (4) flexpro-trust-signal.spec.ts -- already a known, named, previously-flagged-but-never-fixed gap ("3 specs never call grantFreeagentSubscription before posting a gig") -- confirmed and fixed by adding the missing grant call; while doing so, found and fixed the SAME root cause independently biting 2 of the other 3 originally-named specs, mentor-sessions.spec.ts and mentor-monetization.spec.ts: `gigs`' own INSERT RLS policy ("An active subscriber can post a gig listing") requires an active flexpro_subscriptions row, which mentor-session creation also needs since it reuses the gigs table (056), but api/mentor-sessions/gigs/route.ts has no pre-check the way /gigs/new's regular flow does -- so a missing grant there fails silently as a generic "Could not create session type" error instead of a helpful /subscribe redirect; added the same grant to both specs, confirmed via psql's pg_policies that this was the exact real cause before touching either file. mentor-monetization.spec.ts now passes clean. DeepEdge's own suite: 50/50 (was reported as 36/44 in an earlier write-up, entirely due to the corrected misdiagnosis above plus these). Cross-platform: all originally-failing specs from this sweep now fixed and passing except one newly-surfaced, genuinely different, NOT-YET-FIXED bug -- mentor-sessions.spec.ts's paid-session path now gets past session-type creation (fixed above) but times out at the mocked-Razorpay checkout's own "Pay &amp; confirm" step (page.waitForURL to /orders/[id] never resolves); confirmed the mock IS in use (mockRazorpayCheckout, not a real-widget flake) so this is a real, separate, unexplored issue in the paid-checkout order-creation path specifically for a mentor-session order type, left open rather than guessed at further -- reported to the user as a new finding rather than chased down in the same pass. ROOT-CAUSED AND FIXED same week: apps/flexpro/src/app/api/orders/create/route.ts unconditionally validated `packageType` against a `{basic: 1, standard: 2, premium: 3}` multiplier map before ever checking whether this was a pre-claimed mentor-session order -- but mentor-sessions/checkout/[orderId]/page.tsx sends `packageType: 'mentor_session'`, not a real multiplier key, so every paid mentor-session checkout 400'd immediately on "Pay &amp; confirm" (the inline script's own `alert('Failed to start payment: ' + data.error)` path), never reaching `new Razorpay(...)`/`.open()` at all -- exactly matching the observed symptom of the button click never resolving to `/orders/[id]`. Confirmed via `book_mentor_slot()` (056_mentor_sessions.sql): the pre-claimed gig_orders row it creates already stores the exact correct `amount` (`COALESCE(gig.price_min, 0)`) at claim time, so no multiplier was ever needed for this path -- the same "trust the pre-claimed order's own amount" design the route's existing `clientJobEngagement` branch (for client-job-application payments) already used. Fixed by adding a third branch, `if (preClaimedOrderId &amp;&amp; !clientJobEngagement)`, mirroring that existing pattern: fetch the pre-claimed order, reject if a Razorpay order was already attached (409, same idempotency guard as clientJobEngagement), create the Razorpay order from the row's own stored amount, attach `razorpay_order_id`. Verified via grep that only the mentor-session checkout page sends `orderId` without `clientJobEngagement` -- the general gig checkout (`checkout/[id]/page.tsx`) never sends an `orderId` field at all (a genuinely new order every time) and the client-job payment page always sets `clientJobEngagement: true`, so neither of those two other flows touches the new branch. mentor-sessions.spec.ts now passes clean; regression-checked checkout-payment.spec.ts, client-jobs.spec.ts, and mentor-monetization.spec.ts (the other 3 specs exercising this same shared route) -- all still pass.</v>
+        <v>Direct user request: "check code vs database integrity - if any where there is code writing to DB table/columns that are not available in any of the schema and if any table/columns exists that are dangling without any code read/write." Built a static-analysis tool (bracket-depth-aware, not pure regex) walking every .from()/.select()/.insert()/.update()/.upsert() call across all 7 apps' full source (539 files), cross-referenced against the live schema pulled directly from information_schema (76 tables + 14 views, 852 columns) rather than trusting migration-file history. Two real tool bugs caught and fixed before trusting any output: a psql field-separator mismatch that emptied the whole schema lookup (everything falsely flagged "unknown"), and a Buffer.from()/upsert-options-argument false-positive source. FOUR live, severe bugs found and confirmed by direct manual verification (not just the tool's say-so) on the writes/reads side: GreyMatters' and Salt &amp; Pepper's entire profile-save feature completely broken for every user (PostgREST rejects a whole UPDATE on any one unknown column, and both routes bundle valid fields with nonexistent ones -- twitter/linkedin were simply misnamed vs. the real twitter_handle/linkedin_url, while email_notifications/show_email/comment_notifications/interests have no column anywhere); FlexPro's own profile-save also completely broken (title/skills/languages/razorpay_account_id -- the first two belong on a different table, candidates, the other two don't exist anywhere); and FlexPro's own homepage "Recently listed" gigs section had silently never rendered for any visitor (price_basic isn't a real gigs column, every other page in the app correctly uses price_min). The three unambiguous 1:1 renames (twitter-&gt;twitter_handle, linkedin-&gt;linkedin_url, price_basic-&gt;price_min) were fixed and deployed same day, verified live (a real ₹1,800/₹2,000/₹1,500-priced gig now renders on the FlexPro homepage where nothing ever had before). The remaining broken fields (email_notifications/show_email/comment_notifications/interests on 2 apps, title/skills/languages/razorpay_account_id on FlexPro) are real product decisions -- drop the dead form fields vs. add real columns vs. redirect to the correct existing table -- deliberately left for a dedicated review rather than guessed at, tracked as List A. On the dangling side, each of the 5 catalogued objects was individually investigated (when added, why dead) before any drop decision, not bulk-assessed: gig_reviews and gig_reviews_view (both from FlexPro's original 001/006-era schema, superseded by order_reviews, a richer redesign with seller-response and reviewee-side stats) were confirmed genuinely dead via both app-code AND migration-function/trigger sweeps to rule out RPC-only access -- a real false-positive source this audit hit for conversations/credit_usage/mentor_session_bookings/rate_limit_attempts, all confirmed live via RPC calls, not dangling -- then dropped via 112_drop_dead_gig_reviews.sql. razorpay_config and payment_analytics (both from 002_razorpay_integration.sql, the platform's original payments scaffolding) were investigated next: razorpay_config's own creation comment says real keys were always meant for env vars, and its payment_capture_mode/currency/receipt_prefix knobs are hardcoded directly in the real checkout code instead -- it held exactly one never-updated placeholder row (webhook_secret='CHANGE_THIS_WEBHOOK_SECRET') since creation; payment_analytics only ever aggregated gig_orders and now predates 8 other razorpay-touching tables the platform has grown since (author_tips, company_subscriptions, flexpro_subscriptions, payout_requests, subscription_plans/tiers/webhooks, razorpay_webhooks) -- not unused-but-still-valid scaffolding, structurally too narrow to be useful as-is even if adopted today. Both dropped via 113_drop_dead_razorpay_config_and_payment_analytics.sql, same verify-before-drop discipline (row counts, FK dependents, view dependents, live function bodies all checked clean immediately beforehand) and the same after-drop discipline (docker service update --force supabase_rest, then a live smoke test across FlexPro/DeepEdge pages, all 200s). peer_rater_reliability is the one exception to "confirmed dead, safe to drop": a genuine regression, not dead-from-birth scaffolding -- 090_peer_rating_anonymity_and_rater_reliability.sql shipped a real "Employer view: rating pattern" anti-collusion panel that peer-projects.spec.ts still asserts on, but the 2026-09-02/03 candidate-detail-page rebuild silently dropped it (that rebuild's own documented scope was 5 different, unrelated specs; this one was never re-checked afterward) -- flagged to the user as worth restoring rather than dropping. RESTORED same day: user confirmed ("restore 5 and do the needful to complete its usage at relevant feature") -- rebuilt the "Peer-confirmed projects" panel on deepedge/candidates/[id]/page.tsx, including the employer/admin-only "Employer view: rating pattern as a peer rater" sub-panel (peer_rater_reliability) and the per-project "⚠ Possible reciprocal rating" badge (peer_project_reciprocity_flags), matching peer-projects.spec.ts's exact assertions. Restoring this surfaced a second, independent bug in the same 2026-09-02/03 rebuild: the page's notFound() gate required a `candidates` table row to exist for the viewed profile, but `candidates` rows are only auto-created for DeepEdge candidate signups (handle_new_user only inserts one when role='candidate') -- any peer-project collaborator tagged from Salt &amp; Pepper/StackWorks/GreyMatters with no DeepEdge candidate profile 404'd outright, which would have made this restored feature untestable and unusable for exactly the cross-pillar collaborators it exists to cover. Fixed by decoupling the page's existence check from `candidates`: it now fetches the target profile directly from `profiles` (404s only if no profile exists at all) and treats `candidates` as optional, gating only its own DeepEdge-specific fields (title, skills, salary, etc.) on the row actually existing. Also found peer-projects.spec.ts itself needed the same grantActiveSubscriptionTier fix already applied to 22 other specs earlier this session (deepedge_hiring credit gating added later than this spec was written) -- added. Verified end to end against real prod: peer-projects.spec.ts passes in full (employer sees the pattern panel, the mutual-pair line, the project, and the reciprocity badge; a non-employer sees the project but neither the panel nor the badge). Regression-checked the 5 other specs this page serves (skill-endorsements, written-recommendations, reference-checks, weekly-digest, greymatters-cross-posting) plus 2 related cross-platform specs -- all still passing; one unrelated pre-existing failure reproduced in greyin-score-in-candidate-search.spec.ts (the separate /candidates search-list page, not this one) -- root-caused and fixed the same day, see the dedicated pending entry below (a stale test locator, not a data-timing issue). Deployed via full rebuild (--build-arg NEXT_PUBLIC_* set, per the known Next.js build-arg gotcha) + docker service update --force greyin-frontend_deepedge_web.</v>
       </c>
       <c r="D76" t="str">
-        <v>Follow-up during "wat next", 2026-09-04</v>
+        <v>User request, 2026-09-04</v>
       </c>
       <c r="E76" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-04</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Structural sync pass: dashboard header + ecosystem widget + homepage ecosystem-card section, across all 7 apps</v>
+        <v>Misdiagnosed e2e "propagation timing flake" (greyin-score-in-candidate-search.spec.ts) corrected: real cause was a stale CSS locator, not a data race</v>
       </c>
       <c r="B77" t="str">
-        <v>Done, live and e2e-verified</v>
+        <v>Closed -- fixed and verified passing</v>
       </c>
       <c r="C77" t="str">
-        <v>User shared two screenshots (a pillar homepage's "Part of the Greyin Ecosystem / One login, five more platforms" card section, and a colored-dot pillar list) and asked to check whether the card bar is consistently available on every pillar landing page, synchronize the *structure* -- not content -- of every landing page and dashboard page across the 7 apps, and add colored dots to the Greyin Hub's own pillar footer list matching the second screenshot. The Hub footer dots were quick and shipped immediately (`greyin-hub/src/components/SiteFooter.tsx`, matching the `w-2 h-2 rounded-full` dot pattern the 6 pillar apps' own footers already use). The larger synchronization task went through EnterPlanMode given its size (14 pages across 7 apps, several real design forks) -- two Explore passes surveyed every app's homepage/dashboard/SiteHeader/EcosystemWidget/NotificationBell, then 3 AskUserQuestion clarifications pinned down scope: (1) force all 7 dashboards onto one lean utility-bar shape rather than leaving greyin-hub/longlist on the heavier public SiteHeader; (2) do NOT invent new stats-bar/feature-grid homepage sections for the 5 apps lacking one -- that would mean fabricating per-app content, not just structure; (3) add the shared EcosystemWidget to all 7 dashboards (previously only on /profile pages + greyin-hub's own dashboard). Executed: dashboard header sync -- 4 apps (stackworks/flexpro/greymatters-blog/saltnpepper-community) already matched the target shape (logo, /feed, notifications, /profile, theme toggle, sign-out) and only needed their hand-rolled bell+own-unread-count-query swapped for the shared self-contained `&lt;NotificationBell /&gt;` component; deepedge was missing /profile + ThemeToggle entirely and had a name/email text block none of the other 4 show, fixed to match; longlist and greyin-hub previously rendered the full public SiteHeader (with Explore/More-Platforms dropdowns) on /dashboard, both switched to the same lean-bar shape -- longlist's omits /feed (no such route exists there), greyin-hub's reduces further to just logo+theme-toggle+sign-out (no /feed, no /profile route -- /dashboard already serves that role there -- and no NotificationBell/notifications-table usage anywhere in Hub's codebase, confirmed by direct grep before deciding not to invent a new notifications system for Hub as part of a "structural sync"). EcosystemWidget added to the 6 dashboards that lacked it, using each app's own `pillar_memberships` query for the `activePillars` prop (TypeScript caught this immediately -- the component requires it, not optional). Homepage ecosystem section: deepedge's one-line text mention (which had also silently gone stale -- it omitted Longlist entirely) was replaced with the same OTHER_PILLARS card-grid section 4 of the other 5 pillar apps already had; longlist had no ecosystem section at all, added net-new in the same position (immediately before the footer) the other apps already use. greyin-hub's homepage was deliberately left alone -- its own bigger pillar grid already IS the ecosystem overview, a difference in kind, not an inconsistency. Deployed all 7 apps (build-arg gotcha applied throughout) and verified live: curl confirmed the correct pillar count/colors render on deepedge and longlist's new sections (including Longlist itself, fixing that staleness), and the dashboard redirect-to-login behavior confirmed for all 3 rebuilt dashboards. A real regression surfaced during e2e verification: swapping the hand-rolled bell for `&lt;NotificationBell /&gt;` changed its accessible-name mechanism from a `title` HTML attribute to `aria-label` -- 8 existing specs across flexpro/deepedge/stackworks/saltnpepper/greymatters used `getByTitle('Notifications')` against exactly the dashboard pages this pass touched (careful not to touch deepedge's separate, untouched /employer/dashboard, which still correctly uses `getByTitle`) -- all 8 fixed to `getByLabel('Notifications')`. One spec (saltnpepper/notifications.spec.ts) showed a genuine, expected, minor behavioral difference: NotificationBell fetches its unread count client-side on mount (a brief empty state before the badge appears) versus the old bar's server-rendered count being present in the very first paint -- confirmed as a real but inherent property of the already-proven-elsewhere shared component (not a new bug) by retrying, which passed; not chased further since the same component has always behaved this way anywhere else it's used (every app's own SiteHeader). All 7 apps' typecheck+build clean throughout; final e2e regression sweep (23 tests across all touched specs) passed, 2 unrelated local-network flakes aside.</v>
+        <v>Follow-up "wat next" pass after the peer_rater_reliability restoration above. This spec's failure had been attributed, across two prior write-ups (the internal-rename row above and an earlier session), to "a freshly-signed-up candidate's row not reliably showing up yet on /candidates within the test's timeout" -- a signup-trigger propagation race, deliberately deferred as pre-existing and unrelated to whatever was being worked on each time it was hit. Investigated properly this time rather than deferred again: confirmed via direct psql that the RPC search_verified_candidates() returned the candidate correctly with the right greyin_score; confirmed via a real login (password auth, same JWT the app itself uses) that the RPC returns the candidate under the employer's own real session too, not just as a superuser; confirmed via page.reload() 20+ seconds after all writes settled that the rendered page still showed zero matches for the test's locator; and finally confirmed via the page's own accessibility snapshot (error-context.md) that the candidate's full card, with the correct "Verified Expert - Greyin Score 89" text, was rendered on the page the entire time, first in the list. The test's locator was `div.bg-white.rounded-lg.shadow-md` -- but apps/deepedge/src/app/candidates/page.tsx:199 renders each card as `&lt;Link className="block bg-white rounded-lg shadow-md ..."&gt;`, an anchor element, which a div-tag-qualified CSS selector can never match regardless of any data state. Not a regression from anything recent -- likely stale from whenever this page's card markup last changed shape; the baseline candidates.spec.ts never had this problem because it locates by getByText/name instead of a tag-qualified CSS selector. Fixed by switching to `getByRole('link', { name: ... })`, matching the role/name-locator convention already dominant elsewhere in this suite (e.g. peer-projects.spec.ts). Verified passing on a clean re-run. Spot-checked 10 other specs still using the same `div.bg-white.rounded-lg.shadow-md` pattern (pivoter-mentor, reentry-mentor, stackworks/greyin-score, stackworks/people-directory, saltnpepper/karma-and-anonymous, others) against their own target pages' actual markup -- none of them target DeepEdge's /candidates page, and their own cards are still real `&lt;div&gt;` wrappers, so none share this bug; not changed. Corrected the record in all 3 places the wrong "propagation timing flake" diagnosis had been written down (the internal-rename pending entry above, this entry's own predecessor text, and the project memory files backing both) so a future session doesn't defer this again under a wrong explanation. Having disproven the blanket "timing flake" excuse, ran DeepEdge's full own e2e suite (50 tests) and the full cross-platform project (71 tests) clean to see the REAL current picture rather than trust old numbers. Found and fixed 4 more real, previously-uninvestigated bugs, all confirmed by direct root-cause reads (RLS policies, page markup, or DB state), none guessed at: (1) candidate-profile-credits.spec.ts was navigating to `/candidates/${candidates.id}` instead of `/candidates/${profiles.id}` -- the page's own documented URL-id scheme (profiles.id, not candidates.id) -- so it 404'd before either of its two assertions ever ran, on every single run, unconditionally; fixed to use the already-fetched user id directly, no longer needs the candidates.id lookup at all. (2) ecosystem-search-coverage.spec.ts and (3) greymatters-cross-app-surfacing.spec.ts both used a bare `getByText(/Salt &amp; Pepper/)` / `getByText(/GreyMatters/)` that strict-mode-violates against the shared footer's own identical-text link to that pillar's domain -- fixed by anchoring on each result card's actual accessible text ("Salt &amp; Pepper · discussion", "GreyMatters · post"), which is unambiguous. (4) flexpro-trust-signal.spec.ts -- already a known, named, previously-flagged-but-never-fixed gap ("3 specs never call grantFreeagentSubscription before posting a gig") -- confirmed and fixed by adding the missing grant call; while doing so, found and fixed the SAME root cause independently biting 2 of the other 3 originally-named specs, mentor-sessions.spec.ts and mentor-monetization.spec.ts: `gigs`' own INSERT RLS policy ("An active subscriber can post a gig listing") requires an active flexpro_subscriptions row, which mentor-session creation also needs since it reuses the gigs table (056), but api/mentor-sessions/gigs/route.ts has no pre-check the way /gigs/new's regular flow does -- so a missing grant there fails silently as a generic "Could not create session type" error instead of a helpful /subscribe redirect; added the same grant to both specs, confirmed via psql's pg_policies that this was the exact real cause before touching either file. mentor-monetization.spec.ts now passes clean. DeepEdge's own suite: 50/50 (was reported as 36/44 in an earlier write-up, entirely due to the corrected misdiagnosis above plus these). Cross-platform: all originally-failing specs from this sweep now fixed and passing except one newly-surfaced, genuinely different, NOT-YET-FIXED bug -- mentor-sessions.spec.ts's paid-session path now gets past session-type creation (fixed above) but times out at the mocked-Razorpay checkout's own "Pay &amp; confirm" step (page.waitForURL to /orders/[id] never resolves); confirmed the mock IS in use (mockRazorpayCheckout, not a real-widget flake) so this is a real, separate, unexplored issue in the paid-checkout order-creation path specifically for a mentor-session order type, left open rather than guessed at further -- reported to the user as a new finding rather than chased down in the same pass. ROOT-CAUSED AND FIXED same week: apps/flexpro/src/app/api/orders/create/route.ts unconditionally validated `packageType` against a `{basic: 1, standard: 2, premium: 3}` multiplier map before ever checking whether this was a pre-claimed mentor-session order -- but mentor-sessions/checkout/[orderId]/page.tsx sends `packageType: 'mentor_session'`, not a real multiplier key, so every paid mentor-session checkout 400'd immediately on "Pay &amp; confirm" (the inline script's own `alert('Failed to start payment: ' + data.error)` path), never reaching `new Razorpay(...)`/`.open()` at all -- exactly matching the observed symptom of the button click never resolving to `/orders/[id]`. Confirmed via `book_mentor_slot()` (056_mentor_sessions.sql): the pre-claimed gig_orders row it creates already stores the exact correct `amount` (`COALESCE(gig.price_min, 0)`) at claim time, so no multiplier was ever needed for this path -- the same "trust the pre-claimed order's own amount" design the route's existing `clientJobEngagement` branch (for client-job-application payments) already used. Fixed by adding a third branch, `if (preClaimedOrderId &amp;&amp; !clientJobEngagement)`, mirroring that existing pattern: fetch the pre-claimed order, reject if a Razorpay order was already attached (409, same idempotency guard as clientJobEngagement), create the Razorpay order from the row's own stored amount, attach `razorpay_order_id`. Verified via grep that only the mentor-session checkout page sends `orderId` without `clientJobEngagement` -- the general gig checkout (`checkout/[id]/page.tsx`) never sends an `orderId` field at all (a genuinely new order every time) and the client-job payment page always sets `clientJobEngagement: true`, so neither of those two other flows touches the new branch. mentor-sessions.spec.ts now passes clean; regression-checked checkout-payment.spec.ts, client-jobs.spec.ts, and mentor-monetization.spec.ts (the other 3 specs exercising this same shared route) -- all still pass.</v>
       </c>
       <c r="D77" t="str">
-        <v>User request, 2026-09-05</v>
+        <v>Follow-up during "wat next", 2026-09-04</v>
       </c>
       <c r="E77" t="str">
         <v>2026-09-05</v>
@@ -7228,13 +7228,13 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Post-sync visual follow-up: Hub dashboard header reverted to SiteHeader, dashboard-header/preview-banner dark-mode merge fixed, ecosystem-section/footer dark-mode merge fixed (all 7 apps)</v>
+        <v>Structural sync pass: dashboard header + ecosystem widget + homepage ecosystem-card section, across all 7 apps</v>
       </c>
       <c r="B78" t="str">
         <v>Done, live and e2e-verified</v>
       </c>
       <c r="C78" t="str">
-        <v>Direct follow-up after the user reviewed the structural sync pass above against two more screenshots (a pillar homepage's ecosystem-card section, and the Hub's own homepage header) and flagged three concrete visual problems. (1) "greyin hub dashboard looks different than the pillar dashboard pages" -- on reflection the user preferred Hub's dashboard use the SAME header as the rest of the Hub (the pillar-icon-row `&lt;SiteHeader /&gt;`, with its own already-built ThemeToggle + Sign Out), reversing the earlier plan's own choice (approved at the time) to give Hub a shorter custom lean bar since it lacks /feed and /profile routes -- reverted `apps/greyin-hub/src/app/dashboard/page.tsx` from the custom bar back to `&lt;SiteHeader /&gt;`, dropping the now-unused Image/ThemeToggle/LogOut imports built for that bar. (2) "greymatters landing page, gap needed between 5 pillar bar and footer" -- checking another pillar app's dark-mode screenshot first confirmed this was universal, not greymatters-specific: the ecosystem-card section's `dark:bg-gray-900` happened to exactly equal the footer's own fixed (theme-invariant) `bg-gray-900`, so in dark mode the two sections shared one solid color with only a barely-visible 1px border between them -- looked like a single merged block despite real padding being present. Fixed across all 6 apps using this section (stackworks/flexpro/greymatters-blog/saltnpepper-community/deepedge/longlist) by changing the section's dark background to `dark:bg-gray-950`, matching the page's own base background instead of the footer's -- the footer now visibly pops against a slightly darker section above it, the same depth-based separation that already worked correctly in light mode (white section vs. dark footer). (3) "preview build notice merging with pillar dashboard header in dark theme" -- same root shape of bug: every dashboard's hand-rolled header bar used `dark:bg-gray-900`, identical to the preview banner's own fixed `bg-gray-900`, while `SiteHeader.tsx` (used everywhere else) already correctly uses `dark:bg-gray-950` -- confirmed this was exclusively a dashboard-header issue via grep before touching anything. Fixed the same 6 dashboard headers (deepedge's is a `&lt;nav&gt;`, the other 5 are `&lt;header&gt;`) to `dark:bg-gray-950` (+ an explicit `dark:border-gray-800`, matching SiteHeader's own border treatment, on the 5 that lacked one). All fixes verified with real dark-mode screenshots (localStorage `greyin:theme=dark` + reload) before and after, not just code inspection -- confirmed the exact merge reported in each screenshot, then confirmed each fix visually resolved it. All 7 apps typecheck+build clean; e2e regression sweep (dashboard-activity/gig-quality, header-auth-state, longlist-activity, greyin-hub homepage -- 15 tests) passed, 1 unrelated local-network flake aside.</v>
+        <v>User shared two screenshots (a pillar homepage's "Part of the Greyin Ecosystem / One login, five more platforms" card section, and a colored-dot pillar list) and asked to check whether the card bar is consistently available on every pillar landing page, synchronize the *structure* -- not content -- of every landing page and dashboard page across the 7 apps, and add colored dots to the Greyin Hub's own pillar footer list matching the second screenshot. The Hub footer dots were quick and shipped immediately (`greyin-hub/src/components/SiteFooter.tsx`, matching the `w-2 h-2 rounded-full` dot pattern the 6 pillar apps' own footers already use). The larger synchronization task went through EnterPlanMode given its size (14 pages across 7 apps, several real design forks) -- two Explore passes surveyed every app's homepage/dashboard/SiteHeader/EcosystemWidget/NotificationBell, then 3 AskUserQuestion clarifications pinned down scope: (1) force all 7 dashboards onto one lean utility-bar shape rather than leaving greyin-hub/longlist on the heavier public SiteHeader; (2) do NOT invent new stats-bar/feature-grid homepage sections for the 5 apps lacking one -- that would mean fabricating per-app content, not just structure; (3) add the shared EcosystemWidget to all 7 dashboards (previously only on /profile pages + greyin-hub's own dashboard). Executed: dashboard header sync -- 4 apps (stackworks/flexpro/greymatters-blog/saltnpepper-community) already matched the target shape (logo, /feed, notifications, /profile, theme toggle, sign-out) and only needed their hand-rolled bell+own-unread-count-query swapped for the shared self-contained `&lt;NotificationBell /&gt;` component; deepedge was missing /profile + ThemeToggle entirely and had a name/email text block none of the other 4 show, fixed to match; longlist and greyin-hub previously rendered the full public SiteHeader (with Explore/More-Platforms dropdowns) on /dashboard, both switched to the same lean-bar shape -- longlist's omits /feed (no such route exists there), greyin-hub's reduces further to just logo+theme-toggle+sign-out (no /feed, no /profile route -- /dashboard already serves that role there -- and no NotificationBell/notifications-table usage anywhere in Hub's codebase, confirmed by direct grep before deciding not to invent a new notifications system for Hub as part of a "structural sync"). EcosystemWidget added to the 6 dashboards that lacked it, using each app's own `pillar_memberships` query for the `activePillars` prop (TypeScript caught this immediately -- the component requires it, not optional). Homepage ecosystem section: deepedge's one-line text mention (which had also silently gone stale -- it omitted Longlist entirely) was replaced with the same OTHER_PILLARS card-grid section 4 of the other 5 pillar apps already had; longlist had no ecosystem section at all, added net-new in the same position (immediately before the footer) the other apps already use. greyin-hub's homepage was deliberately left alone -- its own bigger pillar grid already IS the ecosystem overview, a difference in kind, not an inconsistency. Deployed all 7 apps (build-arg gotcha applied throughout) and verified live: curl confirmed the correct pillar count/colors render on deepedge and longlist's new sections (including Longlist itself, fixing that staleness), and the dashboard redirect-to-login behavior confirmed for all 3 rebuilt dashboards. A real regression surfaced during e2e verification: swapping the hand-rolled bell for `&lt;NotificationBell /&gt;` changed its accessible-name mechanism from a `title` HTML attribute to `aria-label` -- 8 existing specs across flexpro/deepedge/stackworks/saltnpepper/greymatters used `getByTitle('Notifications')` against exactly the dashboard pages this pass touched (careful not to touch deepedge's separate, untouched /employer/dashboard, which still correctly uses `getByTitle`) -- all 8 fixed to `getByLabel('Notifications')`. One spec (saltnpepper/notifications.spec.ts) showed a genuine, expected, minor behavioral difference: NotificationBell fetches its unread count client-side on mount (a brief empty state before the badge appears) versus the old bar's server-rendered count being present in the very first paint -- confirmed as a real but inherent property of the already-proven-elsewhere shared component (not a new bug) by retrying, which passed; not chased further since the same component has always behaved this way anywhere else it's used (every app's own SiteHeader). All 7 apps' typecheck+build clean throughout; final e2e regression sweep (23 tests across all touched specs) passed, 2 unrelated local-network flakes aside.</v>
       </c>
       <c r="D78" t="str">
         <v>User request, 2026-09-05</v>
@@ -7245,13 +7245,13 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Second visual follow-up: redundant Dashboard link on Hub, EcosystemWidget single-row layout, pillar dashboard-bar icon/color/label consistency</v>
+        <v>Post-sync visual follow-up: Hub dashboard header reverted to SiteHeader, dashboard-header/preview-banner dark-mode merge fixed, ecosystem-section/footer dark-mode merge fixed (all 7 apps)</v>
       </c>
       <c r="B79" t="str">
         <v>Done, live and e2e-verified</v>
       </c>
       <c r="C79" t="str">
-        <v>Third round of the same visual-polish thread. (1) "dashboard link not needed again on greyin hub dashboard" -- since Hub's dashboard now uses `&lt;SiteHeader /&gt;` (reverted in the prior round), it showed a "Dashboard" nav link even while already on /dashboard; fixed by adding `usePathname()` to `greyin-hub/src/components/SiteHeader.tsx` and hiding that one link (desktop + mobile nav) when `pathname === '/dashboard'` -- every other page keeps the link. (2) "'Your Greyin Ecosystem' status can be 6 block in single row instead of 3x2" -- `EcosystemWidget.tsx`'s grid was `grid-cols-1 sm:grid-cols-2` (2-wide, horizontal icon-left cards with a full description line); changed to `grid-cols-2 sm:grid-cols-3 lg:grid-cols-6` with a shorter vertical card (dot on top, name, "Active"/"Visit to join") so 6 fit in one row at desktop width -- applied identically across all 7 apps' copies of this file (no shared package; hand-duplicated per this platform's established convention). (3) "each pillar landing page header must have same pillar icon used on greyin landing page... no need of dashboard next to pillar name and sync color" -- investigated concretely rather than guessed: greyin-hub's SiteHeader.tsx has a canonical PILLAR_ICONS map (deepedge=Building2, greymatters=BookOpen, saltnpepper=Users, flexpro=Briefcase, stackworks=FlaskConical, longlist=Telescope) and every pillar app's own SiteHeader.tsx already imports and uses this exact same icon for its own logo -- marketing/landing headers were already correct. The actual mismatch was in each app's separate, hand-rolled DASHBOARD bar (not SiteHeader): deepedge's had no icon at all (plus a stray "Dashboard" text label neither the user's screenshot nor any other app's bar has, and used text-blue-600 despite deepedge's real brand color being indigo everywhere else -- homepage, buttons, everything); flexpro's dashboard bar used a Package icon instead of Briefcase; greymatters-blog's used PenTool instead of BookOpen; and flexpro/greymatters-blog/saltnpepper-community's dashboard-bar app-name text all used a generic text-indigo-600 regardless of the app's own real accent (confirmed via each app's own homepage hero classes: flexpro=orange, greymatters=sky, saltnpepper=purple -- a genuine pre-existing copy-paste bug, not a deliberate choice). Fixed all of it: deepedge's bar gets a Building2 icon + indigo color + the "Dashboard" label removed; flexpro's gets Briefcase + orange; greymatters-blog's gets BookOpen + sky; saltnpepper-community's gets purple (icon was already correct, Users); stackworks (FlaskConical/teal) and longlist (Telescope/amber) needed no change, already correct. All 7 apps typecheck+build clean; e2e regression sweep (deepedge homepage/auth/notification-bell, greyin-hub homepage, dashboard-activity-and-gig-quality, header-auth-state -- 18 tests) passed clean, no flakes.</v>
+        <v>Direct follow-up after the user reviewed the structural sync pass above against two more screenshots (a pillar homepage's ecosystem-card section, and the Hub's own homepage header) and flagged three concrete visual problems. (1) "greyin hub dashboard looks different than the pillar dashboard pages" -- on reflection the user preferred Hub's dashboard use the SAME header as the rest of the Hub (the pillar-icon-row `&lt;SiteHeader /&gt;`, with its own already-built ThemeToggle + Sign Out), reversing the earlier plan's own choice (approved at the time) to give Hub a shorter custom lean bar since it lacks /feed and /profile routes -- reverted `apps/greyin-hub/src/app/dashboard/page.tsx` from the custom bar back to `&lt;SiteHeader /&gt;`, dropping the now-unused Image/ThemeToggle/LogOut imports built for that bar. (2) "greymatters landing page, gap needed between 5 pillar bar and footer" -- checking another pillar app's dark-mode screenshot first confirmed this was universal, not greymatters-specific: the ecosystem-card section's `dark:bg-gray-900` happened to exactly equal the footer's own fixed (theme-invariant) `bg-gray-900`, so in dark mode the two sections shared one solid color with only a barely-visible 1px border between them -- looked like a single merged block despite real padding being present. Fixed across all 6 apps using this section (stackworks/flexpro/greymatters-blog/saltnpepper-community/deepedge/longlist) by changing the section's dark background to `dark:bg-gray-950`, matching the page's own base background instead of the footer's -- the footer now visibly pops against a slightly darker section above it, the same depth-based separation that already worked correctly in light mode (white section vs. dark footer). (3) "preview build notice merging with pillar dashboard header in dark theme" -- same root shape of bug: every dashboard's hand-rolled header bar used `dark:bg-gray-900`, identical to the preview banner's own fixed `bg-gray-900`, while `SiteHeader.tsx` (used everywhere else) already correctly uses `dark:bg-gray-950` -- confirmed this was exclusively a dashboard-header issue via grep before touching anything. Fixed the same 6 dashboard headers (deepedge's is a `&lt;nav&gt;`, the other 5 are `&lt;header&gt;`) to `dark:bg-gray-950` (+ an explicit `dark:border-gray-800`, matching SiteHeader's own border treatment, on the 5 that lacked one). All fixes verified with real dark-mode screenshots (localStorage `greyin:theme=dark` + reload) before and after, not just code inspection -- confirmed the exact merge reported in each screenshot, then confirmed each fix visually resolved it. All 7 apps typecheck+build clean; e2e regression sweep (dashboard-activity/gig-quality, header-auth-state, longlist-activity, greyin-hub homepage -- 15 tests) passed, 1 unrelated local-network flake aside.</v>
       </c>
       <c r="D79" t="str">
         <v>User request, 2026-09-05</v>
@@ -7262,13 +7262,13 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Platform-wide pillar icon/color consistency sweep: 39 files across deepedge, flexpro, greymatters-blog</v>
+        <v>Second visual follow-up: redundant Dashboard link on Hub, EcosystemWidget single-row layout, pillar dashboard-bar icon/color/label consistency</v>
       </c>
       <c r="B80" t="str">
         <v>Done, live and e2e-verified</v>
       </c>
       <c r="C80" t="str">
-        <v>Direct follow-up to the second visual-polish round above -- user asked, via a "wat next" AskUserQuestion, to sweep for more of the same copy-paste icon/color bug found in dashboard bars. Delegated the search to an Explore agent (read-only, no edits) checking every hand-rolled header across all 7 apps -- employer-dashboard variants, admin pages, login/signup/verify/reset-password, and any other page rendering its own logo outside the shared SiteHeader/SiteFooter/dashboard-bar components already fixed. Confirmed each app's own SiteHeader.tsx was already correct everywhere (imports and uses the right icon from the canonical PILLAR_ICONS map) -- the drift was isolated to standalone pages that each hand-roll their own header instead of using SiteHeader. Found real, live bugs in 3 apps, spot-verified directly (not just trusting the agent) before any edit: deepedge -- 17 files used `Briefcase` instead of the canonical `Building2` icon (a stray leftover, likely from an early shared template), 4 more files (dashboard/applications, jobs/[id]/apply, feed, companies/[id]) additionally used `text-blue-600` instead of deepedge's real indigo, and 4 employer/* pages (settings, post-job, jobs/[id]/applications, jobs/[id]/edit) had no icon at all, just bare text. flexpro -- 11 files used `text-blue-600` or, in the mentor-sessions/* pages, `text-indigo-600`, instead of flexpro's real orange (confirmed via flexpro's own homepage hero classes before touching anything -- this is a genuine brand-color bug, not a deliberate choice, matching the exact same pattern already found and fixed in dashboard bars the round before). greymatters-blog -- 11 files used `text-blue-600` instead of its real sky-blue, same pattern. Every file with more than one matching color string was individually inspected before editing (not blindly sed'd) since several admin pages reuse the same blue on an unrelated ShieldCheck/Sparkles icon elsewhere on the page that was correctly left untouched -- only the logo instance, inside the `&lt;a href="https://greyin.net"&gt;` block, was changed in those files; files confirmed to have exactly one clean occurrence (import + single JSX use, no icon reused elsewhere, no pre-existing conflicting import) were fixed via scoped sed, the rest via individual Edit calls. stackworks, longlist, and saltnpepper-community were confirmed fully clean by the same sweep -- no changes needed there. All 3 touched apps typecheck+build clean, deployed live, and e2e-verified: 104/106 tests passed across deepedge+flexpro+greymatters' full own suites, the only 2 failures being `image-upload.spec.ts` in flexpro and greymatters -- at the time believed a pre-existing, previously-flagged-but-never-investigated flake unrelated to this change; **root-caused and fixed the same week, see the dedicated entry below** -- it was a stale test locator, not a real flake.</v>
+        <v>Third round of the same visual-polish thread. (1) "dashboard link not needed again on greyin hub dashboard" -- since Hub's dashboard now uses `&lt;SiteHeader /&gt;` (reverted in the prior round), it showed a "Dashboard" nav link even while already on /dashboard; fixed by adding `usePathname()` to `greyin-hub/src/components/SiteHeader.tsx` and hiding that one link (desktop + mobile nav) when `pathname === '/dashboard'` -- every other page keeps the link. (2) "'Your Greyin Ecosystem' status can be 6 block in single row instead of 3x2" -- `EcosystemWidget.tsx`'s grid was `grid-cols-1 sm:grid-cols-2` (2-wide, horizontal icon-left cards with a full description line); changed to `grid-cols-2 sm:grid-cols-3 lg:grid-cols-6` with a shorter vertical card (dot on top, name, "Active"/"Visit to join") so 6 fit in one row at desktop width -- applied identically across all 7 apps' copies of this file (no shared package; hand-duplicated per this platform's established convention). (3) "each pillar landing page header must have same pillar icon used on greyin landing page... no need of dashboard next to pillar name and sync color" -- investigated concretely rather than guessed: greyin-hub's SiteHeader.tsx has a canonical PILLAR_ICONS map (deepedge=Building2, greymatters=BookOpen, saltnpepper=Users, flexpro=Briefcase, stackworks=FlaskConical, longlist=Telescope) and every pillar app's own SiteHeader.tsx already imports and uses this exact same icon for its own logo -- marketing/landing headers were already correct. The actual mismatch was in each app's separate, hand-rolled DASHBOARD bar (not SiteHeader): deepedge's had no icon at all (plus a stray "Dashboard" text label neither the user's screenshot nor any other app's bar has, and used text-blue-600 despite deepedge's real brand color being indigo everywhere else -- homepage, buttons, everything); flexpro's dashboard bar used a Package icon instead of Briefcase; greymatters-blog's used PenTool instead of BookOpen; and flexpro/greymatters-blog/saltnpepper-community's dashboard-bar app-name text all used a generic text-indigo-600 regardless of the app's own real accent (confirmed via each app's own homepage hero classes: flexpro=orange, greymatters=sky, saltnpepper=purple -- a genuine pre-existing copy-paste bug, not a deliberate choice). Fixed all of it: deepedge's bar gets a Building2 icon + indigo color + the "Dashboard" label removed; flexpro's gets Briefcase + orange; greymatters-blog's gets BookOpen + sky; saltnpepper-community's gets purple (icon was already correct, Users); stackworks (FlaskConical/teal) and longlist (Telescope/amber) needed no change, already correct. All 7 apps typecheck+build clean; e2e regression sweep (deepedge homepage/auth/notification-bell, greyin-hub homepage, dashboard-activity-and-gig-quality, header-auth-state -- 18 tests) passed clean, no flakes.</v>
       </c>
       <c r="D80" t="str">
         <v>User request, 2026-09-05</v>
@@ -7279,13 +7279,13 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>List A resolved: 9 broken profile-save fields across GreyMatters/Salt &amp; Pepper/FlexPro, deferred from the DB-integrity audit</v>
+        <v>Platform-wide pillar icon/color consistency sweep: 39 files across deepedge, flexpro, greymatters-blog</v>
       </c>
       <c r="B81" t="str">
         <v>Done, live and e2e-verified</v>
       </c>
       <c r="C81" t="str">
-        <v>User asked to resume List A -- the product decisions deliberately deferred from the 2026-09-04 integrity audit (see that pending entry). Before proposing anything, checked whether any code anywhere actually consumes each broken field (email sends, public display, matching/search) and what real infrastructure already exists elsewhere on the platform, then presented per-field recommendations with reasoning; user approved proceeding with all of them. GreyMatters' email_notifications/show_email and Salt &amp; Pepper's email_notifications/comment_notifications: confirmed fully inert (no email-sending code anywhere, no display logic reads show_email) -- dropped the UI entirely (removed the checkboxes and their whole now-empty "Writing Preferences"/"Notification Preferences" sections) rather than add dead columns, since building real functionality would mean building an outbound email system this platform has already deliberately avoided (SMTP rate-limit issue; the weekly digest was built in-app for the same reason). Salt &amp; Pepper's "interests" (confirmed unread anywhere, but plausible community-directory value, cheap to add): added a real text[] column (migration 114). FlexPro's "title" (its own generic professional title, distinct from candidates.current_title which is DeepEdge's current-employer-title concept) and "languages": added real columns (114). FlexPro's "skills": redirected to the existing, already-platform-wide profile_skills table (confirmed live via skill_endorsements/skill_ratings, and already synced into from DeepEdge's candidates.skills via a trigger) instead of a new profiles column -- full-replace semantics on save (delete skills no longer listed, add new ones), confirmed safe since skill_endorsements.skill is a plain text match, not an FK, so removing a skill never cascades or destroys endorsement history. FlexPro's "razorpay_account_id": confirmed a separate, real payout_requests table (bank_account_name/number/ifsc + Razorpay-X fields) already handles payouts via a working /earnings page -- dropped the dead field entirely rather than wire up a second, redundant payout path. Two more real bugs found while building e2e coverage for this (no profile-save spec existed for any of these 3 apps before now, which is exactly how they stayed silently broken): GreyMatters and Salt &amp; Pepper's profile pages both read back the OLD, wrong field names for their own already-fixed columns from the 2026-09-04 audit (profile?.twitter instead of profile?.twitter_handle; profile?.linkedin instead of profile?.linkedin_url) -- the write side had been corrected that day but the read/display side never was, so a save silently succeeded while the form kept showing blank/stale values on every reload. Fixed both. Added a new profile-update.spec.ts per app (3 total, all previously absent) covering the exact fields that used to be silently dropped; FlexPro's additionally exercises the profile_skills full-replace round-trip (add two skills, save, reload; remove one, save, reload, confirm only the remaining one persists). All 3 apps typecheck+build clean, deployed live. Also fixed, found in the same e2e pass: a 4th spec (saltnpepper/mentor-session-link.spec.ts, cross-app) hit the exact same "gigs' INSERT RLS requires an active flexpro_subscriptions row, mentor-session creation has no pre-check" gap already fixed in 2 other specs earlier the same week -- same fix applied, confirmed via grep that no other spec creating a mentor-session gig was still missing it. Full regression sweep across all 3 apps' own suites (82 tests) passed clean except 2 -- at the time believed pre-existing, already-documented, unrelated flakes (image-upload.spec.ts in flexpro/greymatters, root-caused and fixed the same week, see the dedicated entry below) -- and 1 pre-existing flaky pass-on-retry (karma-and-anonymous.spec.ts), unrelated.</v>
+        <v>Direct follow-up to the second visual-polish round above -- user asked, via a "wat next" AskUserQuestion, to sweep for more of the same copy-paste icon/color bug found in dashboard bars. Delegated the search to an Explore agent (read-only, no edits) checking every hand-rolled header across all 7 apps -- employer-dashboard variants, admin pages, login/signup/verify/reset-password, and any other page rendering its own logo outside the shared SiteHeader/SiteFooter/dashboard-bar components already fixed. Confirmed each app's own SiteHeader.tsx was already correct everywhere (imports and uses the right icon from the canonical PILLAR_ICONS map) -- the drift was isolated to standalone pages that each hand-roll their own header instead of using SiteHeader. Found real, live bugs in 3 apps, spot-verified directly (not just trusting the agent) before any edit: deepedge -- 17 files used `Briefcase` instead of the canonical `Building2` icon (a stray leftover, likely from an early shared template), 4 more files (dashboard/applications, jobs/[id]/apply, feed, companies/[id]) additionally used `text-blue-600` instead of deepedge's real indigo, and 4 employer/* pages (settings, post-job, jobs/[id]/applications, jobs/[id]/edit) had no icon at all, just bare text. flexpro -- 11 files used `text-blue-600` or, in the mentor-sessions/* pages, `text-indigo-600`, instead of flexpro's real orange (confirmed via flexpro's own homepage hero classes before touching anything -- this is a genuine brand-color bug, not a deliberate choice, matching the exact same pattern already found and fixed in dashboard bars the round before). greymatters-blog -- 11 files used `text-blue-600` instead of its real sky-blue, same pattern. Every file with more than one matching color string was individually inspected before editing (not blindly sed'd) since several admin pages reuse the same blue on an unrelated ShieldCheck/Sparkles icon elsewhere on the page that was correctly left untouched -- only the logo instance, inside the `&lt;a href="https://greyin.net"&gt;` block, was changed in those files; files confirmed to have exactly one clean occurrence (import + single JSX use, no icon reused elsewhere, no pre-existing conflicting import) were fixed via scoped sed, the rest via individual Edit calls. stackworks, longlist, and saltnpepper-community were confirmed fully clean by the same sweep -- no changes needed there. All 3 touched apps typecheck+build clean, deployed live, and e2e-verified: 104/106 tests passed across deepedge+flexpro+greymatters' full own suites, the only 2 failures being `image-upload.spec.ts` in flexpro and greymatters -- at the time believed a pre-existing, previously-flagged-but-never-investigated flake unrelated to this change; **root-caused and fixed the same week, see the dedicated entry below** -- it was a stale test locator, not a real flake.</v>
       </c>
       <c r="D81" t="str">
         <v>User request, 2026-09-05</v>
@@ -7296,24 +7296,41 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>image-upload.spec.ts (flexpro + greymatters) root-caused: a stale test locator, not a real flake -- had been flagged as an unexplained pre-existing failure across at least 3 separate sessions/passes without ever being investigated</v>
+        <v>List A resolved: 9 broken profile-save fields across GreyMatters/Salt &amp; Pepper/FlexPro, deferred from the DB-integrity audit</v>
       </c>
       <c r="B82" t="str">
-        <v>Done, fixed, verified passing</v>
+        <v>Done, live and e2e-verified</v>
       </c>
       <c r="C82" t="str">
-        <v>Follow-up "wat next" pass -- swept memory for anything still flagged-but-never-actually-investigated (the same discipline that found SEC-040) and found this: `image-upload.spec.ts` had failed in every regression sweep this session touched flexpro or greymatters (at least 4 separate runs across different unrelated passes), each time waved off as "a known, previously-documented pre-existing flake" without anyone actually looking at why. Investigated properly instead of deferring again: added temporary diagnostic logging (the real hidden `image_url` value at submit time, the real `&lt;img&gt;` src rendered on the published page) rather than guessing, and found the upload pipeline was never broken at all -- the client-side upload succeeds, the DB write succeeds (confirmed via direct query), the display page renders the real image correctly. The ONLY problem was the test's own locator: `ImageUploader.tsx` (identical in both apps) nests every upload under the uploader's own `user.id` before the folder name (`${user.id}/${folder}/...`), so the real storage path is `public-images/&lt;userId&gt;/gig-images/&lt;file&gt;` (or `.../post-covers/&lt;file&gt;` for greymatters) -- not `public-images/gig-images/` or `public-images/post-covers/` adjacent, which both tests' locators incorrectly assumed and could never match regardless of whether the upload itself worked, ever, since the day these tests were written. Fixed both locators to match on the actual unique folder segment (`/gig-images/`, `/post-covers/`) instead of assuming adjacency to the bucket name. Verified via direct diagnostic capture of the real production URL before fixing (not just "it passes now") -- confirmed the real shape once, then fixed and re-verified passing, stable across repeated runs. Grepped for any other spec assuming the same wrong adjacency -- none found, these were the only two. Lesson for this codebase: a test failure chalked up to "known pre-existing flake" across multiple sessions without ever being opened once is exactly the kind of debt that compounds silently -- this one had zero connection to whatever each session was actually working on each time it was seen, which is precisely why it kept getting deferred instead of fixed.</v>
+        <v>User asked to resume List A -- the product decisions deliberately deferred from the 2026-09-04 integrity audit (see that pending entry). Before proposing anything, checked whether any code anywhere actually consumes each broken field (email sends, public display, matching/search) and what real infrastructure already exists elsewhere on the platform, then presented per-field recommendations with reasoning; user approved proceeding with all of them. GreyMatters' email_notifications/show_email and Salt &amp; Pepper's email_notifications/comment_notifications: confirmed fully inert (no email-sending code anywhere, no display logic reads show_email) -- dropped the UI entirely (removed the checkboxes and their whole now-empty "Writing Preferences"/"Notification Preferences" sections) rather than add dead columns, since building real functionality would mean building an outbound email system this platform has already deliberately avoided (SMTP rate-limit issue; the weekly digest was built in-app for the same reason). Salt &amp; Pepper's "interests" (confirmed unread anywhere, but plausible community-directory value, cheap to add): added a real text[] column (migration 114). FlexPro's "title" (its own generic professional title, distinct from candidates.current_title which is DeepEdge's current-employer-title concept) and "languages": added real columns (114). FlexPro's "skills": redirected to the existing, already-platform-wide profile_skills table (confirmed live via skill_endorsements/skill_ratings, and already synced into from DeepEdge's candidates.skills via a trigger) instead of a new profiles column -- full-replace semantics on save (delete skills no longer listed, add new ones), confirmed safe since skill_endorsements.skill is a plain text match, not an FK, so removing a skill never cascades or destroys endorsement history. FlexPro's "razorpay_account_id": confirmed a separate, real payout_requests table (bank_account_name/number/ifsc + Razorpay-X fields) already handles payouts via a working /earnings page -- dropped the dead field entirely rather than wire up a second, redundant payout path. Two more real bugs found while building e2e coverage for this (no profile-save spec existed for any of these 3 apps before now, which is exactly how they stayed silently broken): GreyMatters and Salt &amp; Pepper's profile pages both read back the OLD, wrong field names for their own already-fixed columns from the 2026-09-04 audit (profile?.twitter instead of profile?.twitter_handle; profile?.linkedin instead of profile?.linkedin_url) -- the write side had been corrected that day but the read/display side never was, so a save silently succeeded while the form kept showing blank/stale values on every reload. Fixed both. Added a new profile-update.spec.ts per app (3 total, all previously absent) covering the exact fields that used to be silently dropped; FlexPro's additionally exercises the profile_skills full-replace round-trip (add two skills, save, reload; remove one, save, reload, confirm only the remaining one persists). All 3 apps typecheck+build clean, deployed live. Also fixed, found in the same e2e pass: a 4th spec (saltnpepper/mentor-session-link.spec.ts, cross-app) hit the exact same "gigs' INSERT RLS requires an active flexpro_subscriptions row, mentor-session creation has no pre-check" gap already fixed in 2 other specs earlier the same week -- same fix applied, confirmed via grep that no other spec creating a mentor-session gig was still missing it. Full regression sweep across all 3 apps' own suites (82 tests) passed clean except 2 -- at the time believed pre-existing, already-documented, unrelated flakes (image-upload.spec.ts in flexpro/greymatters, root-caused and fixed the same week, see the dedicated entry below) -- and 1 pre-existing flaky pass-on-retry (karma-and-anonymous.spec.ts), unrelated.</v>
       </c>
       <c r="D82" t="str">
-        <v>Follow-up during "wat next", 2026-09-05</v>
+        <v>User request, 2026-09-05</v>
       </c>
       <c r="E82" t="str">
         <v>2026-09-05</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>image-upload.spec.ts (flexpro + greymatters) root-caused: a stale test locator, not a real flake -- had been flagged as an unexplained pre-existing failure across at least 3 separate sessions/passes without ever being investigated</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Done, fixed, verified passing</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Follow-up "wat next" pass -- swept memory for anything still flagged-but-never-actually-investigated (the same discipline that found SEC-040) and found this: `image-upload.spec.ts` had failed in every regression sweep this session touched flexpro or greymatters (at least 4 separate runs across different unrelated passes), each time waved off as "a known, previously-documented pre-existing flake" without anyone actually looking at why. Investigated properly instead of deferring again: added temporary diagnostic logging (the real hidden `image_url` value at submit time, the real `&lt;img&gt;` src rendered on the published page) rather than guessing, and found the upload pipeline was never broken at all -- the client-side upload succeeds, the DB write succeeds (confirmed via direct query), the display page renders the real image correctly. The ONLY problem was the test's own locator: `ImageUploader.tsx` (identical in both apps) nests every upload under the uploader's own `user.id` before the folder name (`${user.id}/${folder}/...`), so the real storage path is `public-images/&lt;userId&gt;/gig-images/&lt;file&gt;` (or `.../post-covers/&lt;file&gt;` for greymatters) -- not `public-images/gig-images/` or `public-images/post-covers/` adjacent, which both tests' locators incorrectly assumed and could never match regardless of whether the upload itself worked, ever, since the day these tests were written. Fixed both locators to match on the actual unique folder segment (`/gig-images/`, `/post-covers/`) instead of assuming adjacency to the bucket name. Verified via direct diagnostic capture of the real production URL before fixing (not just "it passes now") -- confirmed the real shape once, then fixed and re-verified passing, stable across repeated runs. Grepped for any other spec assuming the same wrong adjacency -- none found, these were the only two. Lesson for this codebase: a test failure chalked up to "known pre-existing flake" across multiple sessions without ever being opened once is exactly the kind of debt that compounds silently -- this one had zero connection to whatever each session was actually working on each time it was seen, which is precisely why it kept getting deferred instead of fixed.</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Follow-up during "wat next", 2026-09-05</v>
+      </c>
+      <c r="E83" t="str">
+        <v>2026-09-05</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E83"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Longlist rail gets an Admin link pointing to Greyin Hub's centralized moderation panel
Longlist's WorkspaceShell was built before this pillar had any admin
capability at all, and was never revisited after moderation was added
directly into Greyin Hub's /admin/longlist (migration 140) rather than
as a local panel here -- leaving zero visible indication to an admin
that any moderation existed for this pillar, unlike every other app's
self-evident local Admin rail link.

Threaded a `role` prop through WorkspaceShell and all 8 page callers,
and added an Admin item (same separated-section style as the other
apps) pointing to that external Hub URL directly, since this app has no
local /admin route of its own.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements-traceability/greyin-requirements-traceability.xlsx
+++ b/docs/requirements-traceability/greyin-requirements-traceability.xlsx
@@ -5908,7 +5908,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E90"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -7430,9 +7430,26 @@
         <v>2026-09-12</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Longlist rail given its own Admin link, pointing to Greyin Hub's centralized moderation panel</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Done, live and e2e-verified</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Follow-up: "check why still no admin role/page visible at longlist pillar page in addition to admin panel." Root cause: Longlist's WorkspaceShell was built 2026-09-05 with an explicit comment stating "No admin section at all in this app" -- true at the time, but Longlist gained real admin capability 3 days later (migration 140, 2026-09-08) built directly into Greyin Hub's /admin/longlist rather than as a local panel (no financial actions here to protect the way FlexPro/DeepEdge/StackWorks's local admin panels do -- see the prior "why does longlist not have admin role/panel" investigation this same session). Nobody revisited the rail after that shipped, so an admin looking at Longlist itself had zero indication any moderation capability existed for this pillar at all, unlike every other app's self-evident local "Admin" rail link. Fixed by threading a new `role` prop through WorkspaceShell (component + both RailContents render calls + all 8 page.tsx callers, 6 of which didn't select `role` in their own profile query yet) and adding an Admin item in the same separated-section-above-Across-Greyin style the other 5 apps use -- except this one is a plain external `&lt;a href="https://greyin.net/admin/longlist"&gt;`, not a Next `&lt;Link&gt;` to a local route this app doesn't have. New e2e coverage: an admin sees the link with the correct external href, in its own separated section; a non-admin sees none. Typechecked, built, deployed; full Longlist suite (10 specs) passes clean.</v>
+      </c>
+      <c r="D90" t="str">
+        <v>User request, 2026-09-12</v>
+      </c>
+      <c r="E90" t="str">
+        <v>2026-09-12</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E90"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add collapsible sidebar + dark-mode banner color, with tests and docs
WorkspaceShell.tsx across all 6 apps with a persistent rail (DeepEdge,
FlexPro, StackWorks, Salt & Pepper, GreyMatters, Longlist) can now
collapse to an icon-only strip via a toggle button, persisted in
localStorage. The preview-build banner gets a distinct dark:bg-black
across all 7 apps instead of blending into the rail/header below it.

Adds e2e coverage (collapse/expand, label-hiding via title tooltips,
localStorage persistence, StackWorks' split nav/profileItem paths) and
updates the requirements-traceability workbook + architecture doc.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements-traceability/greyin-requirements-traceability.xlsx
+++ b/docs/requirements-traceability/greyin-requirements-traceability.xlsx
@@ -5908,7 +5908,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E92"/>
   <cols>
     <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -7464,9 +7464,26 @@
         <v>2026-09-13</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Collapsible sidebar (icon-only rail) across all 6 apps with a persistent WorkspaceShell, plus a distinct dark-mode color for the preview-build banner</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Done, live and e2e-verified</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Follow-up to the sidebar-organization round: "check if sidebar at all applicable places can be collapsible with a thinner bar appearing with just icons" and "change the color of the preview build notice in dark theme to some other color other than the sidebar." Added a `collapsed` boolean to WorkspaceShell.tsx in all 6 apps with a persistent rail (DeepEdge, FlexPro, StackWorks, Salt &amp; Pepper, GreyMatters, Longlist), toggled via a chevron button on the rail's right edge and persisted to localStorage (`greyin:sidebar-collapsed`, read on mount to avoid an SSR/hydration flash) -- a pure per-browser display preference, not a profiles column, matching how the theme toggle already persists. Collapsed state shrinks the aside from w-64 to an icon-only w-16 (`transition-[width] duration-200`, content column's `lg:pl-64`/`lg:pl-16` mirrors it), hides every nav label/section-header/user-name text via `{!collapsed &amp;&amp; label}` while keeping every icon (`shrink-0` added so icons never squish) and adding a `title` tooltip carrying the hidden label. The mobile drawer's own separate `&lt;RailContents&gt;` call site deliberately never passes `collapsed` -- it is a temporary full-width overlay that should never render collapsed. Applied the same mechanical transformation to all 6 near-duplicate WorkspaceShell.tsx copies, adapting per-app quirks: StackWorks' RailContents splits its nav array around a builder-only "Post a Project" insert and a separately-rendered trailing `profileItem` (both needed their own collapsed treatment, confirmed via a dedicated regression test); Longlist's Admin link is a plain external `&lt;a&gt;` (no local /admin route) that got the same title/collapsed treatment; GreyMatters has no separate "Greyin Hub" row in its Across-Greyin block since it renders itself as the current pillar. Separately, the preview-build banner used the exact same `bg-gray-900` as the rail/header in dark mode with no visible seam between the two -- changed to `bg-gray-900 dark:bg-black`, a deliberately different shade (not just a slightly darker gray) chosen so the banner reads as its own strip in dark mode, applied identically to all 7 apps' layout.tsx (including greyin-hub, which has no persistent sidebar but still had the same blending issue against its own header). Caught one real test-writing bug while verifying live, not a product bug: a collapsed link's accessible NAME still resolves to its label via the `title` attribute (the browser's accessible-name algorithm falls back to `title` when there is no visible text) -- so `getByRole('link', {name: ...})` still matched a collapsed, visually-icon-only link; fixed by asserting hidden state via `toHaveText('')` instead, confirmed correct against a live screenshot showing the rail genuinely collapsed to icon-only. New/updated e2e coverage: workspace-shell.spec.ts (DeepEdge) gained a full toggle/hide-labels/localStorage-persistence/expand-again test; workspace-shell-admin.spec.ts (StackWorks) gained a dedicated regression test for the split nav/profileItem render paths. All 7 apps typechecked, built, deployed; new tests plus a 26-test regression sweep across deepedge/stackworks/flexpro/saltnpepper/greymatters/longlist workspace-shell specs passes clean.</v>
+      </c>
+      <c r="D92" t="str">
+        <v>User request, 2026-09-13</v>
+      </c>
+      <c r="E92" t="str">
+        <v>2026-09-13</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E92"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>